<commit_message>
The decision log holds each outside-review batch by name: batches 3, 4 and 5 recorded in his words (DEC-2746, DEC-2747, DEC-2748)
His question, 2026-10-07: was the decision log — the one master — being updated, not only the Changelog?
It held batches 1 and 2 (DEC-2440, DEC-2484) and the standing rule that audit changes are his (DEC-2634),
but not which changes batches 3 and 4 made, and nothing for batch 5. Each batch now has its own row, in
his words of approval, naming every function it changed and every point held. DEC-2748 states it keeps
his rule A46 (DEC-0279) rather than replacing it. Each has its Changelog row the same day; the gate that
stops a build for a decision with no Changelog row fired on all three before the rows were written.
Gates exit 0.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
+++ b/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
@@ -25408,7 +25408,7 @@
       </c>
       <c r="G409" s="2" t="inlineStr">
         <is>
-          <t>MK-PF-M-014 Wealth generated, MK-PF-M-017 Return, MK-PF-M-006 WHAT EACH CATEGORY EARNED — RETURN</t>
+          <t>MK-PF-M-014 Wealth generated, MK-PF-M-006 WHAT EACH CATEGORY EARNED — RETURN, MK-PF-M-017 Return</t>
         </is>
       </c>
       <c r="H409" s="2" t="inlineStr">
@@ -25494,7 +25494,7 @@
       </c>
       <c r="G411" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-020 THIS MONTH — free to use, MK-XS-M-006 Income · In (received) · In (take-home)</t>
+          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-CF-M-020 THIS MONTH — free to use</t>
         </is>
       </c>
       <c r="H411" s="2" t="inlineStr">
@@ -25580,7 +25580,7 @@
       </c>
       <c r="G413" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-007 Left / Over · left to spend this month</t>
         </is>
       </c>
       <c r="H413" s="2" t="inlineStr">
@@ -25623,7 +25623,7 @@
       </c>
       <c r="G414" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-007 Left / Over · left to spend this month</t>
         </is>
       </c>
       <c r="H414" s="2" t="inlineStr">
@@ -27472,7 +27472,7 @@
       </c>
       <c r="G457" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-007 Left / Over · left to spend this month</t>
         </is>
       </c>
       <c r="H457" s="2" t="inlineStr">
@@ -27644,7 +27644,7 @@
       </c>
       <c r="G461" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-014 Employer 401(k) match</t>
+          <t>MK-MN-M-012 Gross / year, MK-MN-M-014 Employer 401(k) match, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H461" s="2" t="inlineStr">
@@ -27816,7 +27816,7 @@
       </c>
       <c r="G465" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-007 Left / Over · left to spend this month</t>
         </is>
       </c>
       <c r="H465" s="2" t="inlineStr">
@@ -28633,7 +28633,7 @@
       </c>
       <c r="G484" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H484" s="2" t="inlineStr">
@@ -28676,7 +28676,7 @@
       </c>
       <c r="G485" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed</t>
         </is>
       </c>
       <c r="H485" s="2" t="inlineStr">
@@ -28719,7 +28719,7 @@
       </c>
       <c r="G486" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-005 + Draw from savings</t>
         </is>
       </c>
       <c r="H486" s="2" t="inlineStr">
@@ -28762,7 +28762,7 @@
       </c>
       <c r="G487" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-004 = Guaranteed</t>
         </is>
       </c>
       <c r="H487" s="2" t="inlineStr">
@@ -28805,7 +28805,7 @@
       </c>
       <c r="G488" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-005 + Draw from savings</t>
         </is>
       </c>
       <c r="H488" s="2" t="inlineStr">
@@ -29923,7 +29923,7 @@
       </c>
       <c r="G514" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H514" s="2" t="inlineStr">
@@ -29966,7 +29966,7 @@
       </c>
       <c r="G515" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H515" s="2" t="inlineStr">
@@ -30009,7 +30009,7 @@
       </c>
       <c r="G516" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H516" s="2" t="inlineStr">
@@ -30052,7 +30052,7 @@
       </c>
       <c r="G517" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N</t>
         </is>
       </c>
       <c r="H517" s="2" t="inlineStr">
@@ -30138,7 +30138,7 @@
       </c>
       <c r="G519" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-024 You could cover a $X hit, MK-MN-M-026 your $X/month of essentials, MK-MN-M-025 You'd have $X left — about N months of e</t>
+          <t>MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-024 You could cover a $X hit, MK-MN-M-026 your $X/month of essentials</t>
         </is>
       </c>
       <c r="H519" s="2" t="inlineStr">
@@ -30181,7 +30181,7 @@
       </c>
       <c r="G520" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-024 You could cover a $X hit, MK-MN-M-026 your $X/month of essentials, MK-MN-M-025 You'd have $X left — about N months of e</t>
+          <t>MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-024 You could cover a $X hit, MK-MN-M-026 your $X/month of essentials</t>
         </is>
       </c>
       <c r="H520" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Other investments: the rows add up to the total again — each account holding alternatives is a row at its alternatives part
Found re-checking all five batches against his two rules (2026-10-07). The second round made Total value
read alternatives held inside a brokerage, but the rows still listed whole alternatives accounts, so the
rows no longer added up to the total. Each account that holds alternatives is now a row at its part; a
brokerage row says which part it is and opens its account page. Test: recheck_2026-10-07.test.ts.
Formula in words, drawing Alternatives v02 updated. 4,080 tests green; gates exit 0.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
+++ b/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
@@ -9217,6 +9217,7 @@
 MK-NW-F-021 investmentsTotal
 MK-NW-F-022 investableAssets
 MK-NW-F-027 accountClassBreakdown
+MK-NW-F-028 classPortionLabel
 MK-NW-F-029 assetAllocation
 MK-NW-F-030 earmarkDefault
 MK-NW-F-031 primaryCarIdOf
@@ -9237,6 +9238,7 @@
 MK-NW-F-064 bondRateSensitivity
 MK-NW-F-065 buildNetWorth
 MK-NW-F-066 sumWhere
+MK-NW-F-067 plural
 MK-NW-F-069 priceAtYield
 MK-NW-F-070 accruedInterestCaveat
 MK-NW-F-072 rowOf
@@ -9309,6 +9311,7 @@
 MK-XS-F-064 currentIdToken
 MK-XS-F-083 fetchPriceSeries
 MK-XS-F-112 relayUrl
+MK-XS-F-120 nameOf
 MK-XS-F-121 isYm
 MK-XS-F-122 n
 MK-XS-F-147 call
@@ -25501,7 +25504,7 @@
       </c>
       <c r="G409" s="2" t="inlineStr">
         <is>
-          <t>MK-PF-M-014 Wealth generated, MK-PF-M-017 Return, MK-PF-M-006 WHAT EACH CATEGORY EARNED — RETURN</t>
+          <t>MK-PF-M-014 Wealth generated, MK-PF-M-006 WHAT EACH CATEGORY EARNED — RETURN, MK-PF-M-017 Return</t>
         </is>
       </c>
       <c r="H409" s="2" t="inlineStr">
@@ -25673,7 +25676,7 @@
       </c>
       <c r="G413" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H413" s="2" t="inlineStr">
@@ -25716,7 +25719,7 @@
       </c>
       <c r="G414" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H414" s="2" t="inlineStr">
@@ -25845,7 +25848,7 @@
       </c>
       <c r="G417" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-020 THIS MONTH — free to use</t>
         </is>
       </c>
       <c r="H417" s="2" t="inlineStr">
@@ -26920,7 +26923,7 @@
       </c>
       <c r="G442" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
+          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
         </is>
       </c>
       <c r="H442" s="2" t="inlineStr">
@@ -27006,7 +27009,7 @@
       </c>
       <c r="G444" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
+          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
         </is>
       </c>
       <c r="H444" s="2" t="inlineStr">
@@ -27049,7 +27052,7 @@
       </c>
       <c r="G445" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
+          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
         </is>
       </c>
       <c r="H445" s="2" t="inlineStr">
@@ -27264,7 +27267,7 @@
       </c>
       <c r="G450" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
+          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
         </is>
       </c>
       <c r="H450" s="2" t="inlineStr">
@@ -27565,7 +27568,7 @@
       </c>
       <c r="G457" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H457" s="2" t="inlineStr">
@@ -27737,7 +27740,7 @@
       </c>
       <c r="G461" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-013 Take-home / month, MK-MN-M-014 Employer 401(k) match, MK-MN-M-011 TAKE-HOME / YEAR</t>
+          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-014 Employer 401(k) match</t>
         </is>
       </c>
       <c r="H461" s="2" t="inlineStr">
@@ -27909,7 +27912,7 @@
       </c>
       <c r="G465" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H465" s="2" t="inlineStr">
@@ -28726,7 +28729,7 @@
       </c>
       <c r="G484" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H484" s="2" t="inlineStr">
@@ -28769,7 +28772,7 @@
       </c>
       <c r="G485" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H485" s="2" t="inlineStr">
@@ -28812,7 +28815,7 @@
       </c>
       <c r="G486" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-005 + Draw from savings</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H486" s="2" t="inlineStr">
@@ -28855,7 +28858,7 @@
       </c>
       <c r="G487" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H487" s="2" t="inlineStr">
@@ -28898,7 +28901,7 @@
       </c>
       <c r="G488" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H488" s="2" t="inlineStr">

</xml_diff>

<commit_message>
A hand-built account is split across classes at today's values, not at what was paid
Found re-checking all five batches (2026-10-07): the split shared out the invested part by what each
holding cost, because hand-built holdings carry no broker price — so a stock bought at $100 and worth
$300 showed a third of its value. Each holding now keeps the value its account balance was built from.
Test in recheck_2026-10-07.test.ts; formula in words and standard §4 updated. 4,081 tests; gates exit 0.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
+++ b/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
@@ -25590,7 +25590,7 @@
       </c>
       <c r="G411" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-020 THIS MONTH — free to use, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
+          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-CF-M-020 THIS MONTH — free to use</t>
         </is>
       </c>
       <c r="H411" s="2" t="inlineStr">
@@ -25676,7 +25676,7 @@
       </c>
       <c r="G413" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H413" s="2" t="inlineStr">
@@ -25719,7 +25719,7 @@
       </c>
       <c r="G414" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H414" s="2" t="inlineStr">
@@ -25848,7 +25848,7 @@
       </c>
       <c r="G417" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H417" s="2" t="inlineStr">
@@ -26923,7 +26923,7 @@
       </c>
       <c r="G442" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
+          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
         </is>
       </c>
       <c r="H442" s="2" t="inlineStr">
@@ -27009,7 +27009,7 @@
       </c>
       <c r="G444" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
+          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
         </is>
       </c>
       <c r="H444" s="2" t="inlineStr">
@@ -27052,7 +27052,7 @@
       </c>
       <c r="G445" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
+          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
         </is>
       </c>
       <c r="H445" s="2" t="inlineStr">
@@ -27267,7 +27267,7 @@
       </c>
       <c r="G450" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
+          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
         </is>
       </c>
       <c r="H450" s="2" t="inlineStr">
@@ -27482,7 +27482,7 @@
       </c>
       <c r="G455" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H455" s="2" t="inlineStr">
@@ -27525,7 +27525,7 @@
       </c>
       <c r="G456" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H456" s="2" t="inlineStr">
@@ -27568,7 +27568,7 @@
       </c>
       <c r="G457" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H457" s="2" t="inlineStr">
@@ -27611,7 +27611,7 @@
       </c>
       <c r="G458" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-012 Gross / year</t>
+          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month, MK-MN-M-012 Gross / year</t>
         </is>
       </c>
       <c r="H458" s="2" t="inlineStr">
@@ -27654,7 +27654,7 @@
       </c>
       <c r="G459" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-012 Gross / year</t>
+          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month, MK-MN-M-012 Gross / year</t>
         </is>
       </c>
       <c r="H459" s="2" t="inlineStr">
@@ -27697,7 +27697,7 @@
       </c>
       <c r="G460" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
+          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H460" s="2" t="inlineStr">
@@ -27740,7 +27740,7 @@
       </c>
       <c r="G461" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-014 Employer 401(k) match</t>
+          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month, MK-MN-M-014 Employer 401(k) match</t>
         </is>
       </c>
       <c r="H461" s="2" t="inlineStr">
@@ -27912,7 +27912,7 @@
       </c>
       <c r="G465" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H465" s="2" t="inlineStr">
@@ -28772,7 +28772,7 @@
       </c>
       <c r="G485" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-004 = Guaranteed</t>
         </is>
       </c>
       <c r="H485" s="2" t="inlineStr">
@@ -28815,7 +28815,7 @@
       </c>
       <c r="G486" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H486" s="2" t="inlineStr">
@@ -28858,7 +28858,7 @@
       </c>
       <c r="G487" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-004 = Guaranteed</t>
         </is>
       </c>
       <c r="H487" s="2" t="inlineStr">
@@ -28901,7 +28901,7 @@
       </c>
       <c r="G488" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H488" s="2" t="inlineStr">

</xml_diff>

<commit_message>
A CD and a money-market fund sit with Investments, not Cash — his rule DEC-0051 (batch 06 fix brief, own commit so it can be reverted alone)
isCashKind (MK-NW-F-006) listed kind cd — and money_market — as cash, while their class is Bonds & CDs and
Stocks / Funds: one CD sat under Cash on one total and Investments on another. The brief named the CD;
the money-market fund is the same defect (recorded as F6, as he reported it) and moved with it. The
add-account form now offers both with Investments. Probes that recorded the contradiction now assert it is
closed. 4,105 tests green; gates exit 0.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
+++ b/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
@@ -25510,7 +25510,7 @@
       </c>
       <c r="G409" s="2" t="inlineStr">
         <is>
-          <t>MK-PF-M-014 Wealth generated, MK-PF-M-017 Return, MK-PF-M-006 WHAT EACH CATEGORY EARNED — RETURN</t>
+          <t>MK-PF-M-014 Wealth generated, MK-PF-M-006 WHAT EACH CATEGORY EARNED — RETURN, MK-PF-M-017 Return</t>
         </is>
       </c>
       <c r="H409" s="2" t="inlineStr">
@@ -25596,7 +25596,7 @@
       </c>
       <c r="G411" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-020 THIS MONTH — free to use, MK-XS-M-006 Income · In (received) · In (take-home)</t>
+          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-CF-M-020 THIS MONTH — free to use</t>
         </is>
       </c>
       <c r="H411" s="2" t="inlineStr">
@@ -25778,7 +25778,7 @@
       </c>
       <c r="I415" s="2" t="n"/>
     </row>
-    <row r="416" ht="45" customHeight="1">
+    <row r="416" ht="60" customHeight="1">
       <c r="A416" s="2" t="inlineStr">
         <is>
           <t>money figure — more than one row could be it</t>
@@ -25811,7 +25811,7 @@
       </c>
       <c r="G416" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-CF-M-001 Expenses, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-CF-M-001 Expenses, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H416" s="2" t="inlineStr">
@@ -25854,7 +25854,7 @@
       </c>
       <c r="G417" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H417" s="2" t="inlineStr">
@@ -25897,7 +25897,7 @@
       </c>
       <c r="G418" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-020 THIS MONTH — free to use, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-CF-M-020 THIS MONTH — free to use</t>
         </is>
       </c>
       <c r="H418" s="2" t="inlineStr">
@@ -26929,7 +26929,7 @@
       </c>
       <c r="G442" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
+          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
         </is>
       </c>
       <c r="H442" s="2" t="inlineStr">
@@ -27015,7 +27015,7 @@
       </c>
       <c r="G444" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
+          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
         </is>
       </c>
       <c r="H444" s="2" t="inlineStr">
@@ -27058,7 +27058,7 @@
       </c>
       <c r="G445" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
+          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
         </is>
       </c>
       <c r="H445" s="2" t="inlineStr">
@@ -27273,7 +27273,7 @@
       </c>
       <c r="G450" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
+          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
         </is>
       </c>
       <c r="H450" s="2" t="inlineStr">
@@ -27617,7 +27617,7 @@
       </c>
       <c r="G458" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month, MK-MN-M-012 Gross / year</t>
+          <t>MK-MN-M-012 Gross / year, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H458" s="2" t="inlineStr">
@@ -27660,7 +27660,7 @@
       </c>
       <c r="G459" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month, MK-MN-M-012 Gross / year</t>
+          <t>MK-MN-M-012 Gross / year, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H459" s="2" t="inlineStr">
@@ -27746,7 +27746,7 @@
       </c>
       <c r="G461" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-014 Employer 401(k) match, MK-MN-M-013 Take-home / month</t>
+          <t>MK-MN-M-014 Employer 401(k) match, MK-MN-M-012 Gross / year, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H461" s="2" t="inlineStr">
@@ -28735,7 +28735,7 @@
       </c>
       <c r="G484" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H484" s="2" t="inlineStr">
@@ -28778,7 +28778,7 @@
       </c>
       <c r="G485" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-005 + Draw from savings</t>
+          <t>MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H485" s="2" t="inlineStr">
@@ -28821,7 +28821,7 @@
       </c>
       <c r="G486" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H486" s="2" t="inlineStr">
@@ -28864,7 +28864,7 @@
       </c>
       <c r="G487" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-004 = Guaranteed</t>
         </is>
       </c>
       <c r="H487" s="2" t="inlineStr">
@@ -28907,7 +28907,7 @@
       </c>
       <c r="G488" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-005 + Draw from savings</t>
+          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-004 = Guaranteed</t>
         </is>
       </c>
       <c r="H488" s="2" t="inlineStr">
@@ -30025,7 +30025,7 @@
       </c>
       <c r="G514" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H514" s="2" t="inlineStr">
@@ -30068,7 +30068,7 @@
       </c>
       <c r="G515" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H515" s="2" t="inlineStr">
@@ -30111,7 +30111,7 @@
       </c>
       <c r="G516" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H516" s="2" t="inlineStr">
@@ -30154,7 +30154,7 @@
       </c>
       <c r="G517" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N</t>
         </is>
       </c>
       <c r="H517" s="2" t="inlineStr">

</xml_diff>

<commit_message>
His approval of the eight tenets (DEC-3523, 'tenets approved'): file marked approved, Changelog row, the Net worth module brief for OpenAI rewritten with them
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
+++ b/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
@@ -25527,7 +25527,7 @@
       </c>
       <c r="G409" s="2" t="inlineStr">
         <is>
-          <t>MK-PF-M-014 Wealth generated, MK-PF-M-017 Return, MK-PF-M-006 WHAT EACH CATEGORY EARNED — RETURN</t>
+          <t>MK-PF-M-014 Wealth generated, MK-PF-M-006 WHAT EACH CATEGORY EARNED — RETURN, MK-PF-M-017 Return</t>
         </is>
       </c>
       <c r="H409" s="2" t="inlineStr">
@@ -25613,7 +25613,7 @@
       </c>
       <c r="G411" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-020 THIS MONTH — free to use, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
+          <t>MK-CF-M-034 Your 401(k)s, MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-020 THIS MONTH — free to use</t>
         </is>
       </c>
       <c r="H411" s="2" t="inlineStr">
@@ -25699,7 +25699,7 @@
       </c>
       <c r="G413" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-XS-M-007 Left / Over · left to spend this month</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H413" s="2" t="inlineStr">
@@ -25742,7 +25742,7 @@
       </c>
       <c r="G414" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-XS-M-007 Left / Over · left to spend this month</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H414" s="2" t="inlineStr">
@@ -25795,7 +25795,7 @@
       </c>
       <c r="I415" s="2" t="n"/>
     </row>
-    <row r="416" ht="45" customHeight="1">
+    <row r="416" ht="60" customHeight="1">
       <c r="A416" s="2" t="inlineStr">
         <is>
           <t>money figure — more than one row could be it</t>
@@ -25828,7 +25828,7 @@
       </c>
       <c r="G416" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-CF-M-001 Expenses, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-CF-M-001 Expenses, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H416" s="2" t="inlineStr">
@@ -25871,7 +25871,7 @@
       </c>
       <c r="G417" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H417" s="2" t="inlineStr">
@@ -27591,7 +27591,7 @@
       </c>
       <c r="G457" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-XS-M-007 Left / Over · left to spend this month</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H457" s="2" t="inlineStr">
@@ -27634,7 +27634,7 @@
       </c>
       <c r="G458" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
+          <t>MK-MN-M-012 Gross / year, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H458" s="2" t="inlineStr">
@@ -27677,7 +27677,7 @@
       </c>
       <c r="G459" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
+          <t>MK-MN-M-012 Gross / year, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H459" s="2" t="inlineStr">
@@ -27720,7 +27720,7 @@
       </c>
       <c r="G460" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
+          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H460" s="2" t="inlineStr">
@@ -27763,7 +27763,7 @@
       </c>
       <c r="G461" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-014 Employer 401(k) match, MK-MN-M-013 Take-home / month</t>
+          <t>MK-MN-M-012 Gross / year, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-014 Employer 401(k) match</t>
         </is>
       </c>
       <c r="H461" s="2" t="inlineStr">
@@ -27935,7 +27935,7 @@
       </c>
       <c r="G465" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-XS-M-007 Left / Over · left to spend this month</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H465" s="2" t="inlineStr">
@@ -28752,7 +28752,7 @@
       </c>
       <c r="G484" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed</t>
         </is>
       </c>
       <c r="H484" s="2" t="inlineStr">
@@ -28795,7 +28795,7 @@
       </c>
       <c r="G485" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H485" s="2" t="inlineStr">
@@ -28838,7 +28838,7 @@
       </c>
       <c r="G486" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-005 + Draw from savings</t>
         </is>
       </c>
       <c r="H486" s="2" t="inlineStr">
@@ -28881,7 +28881,7 @@
       </c>
       <c r="G487" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H487" s="2" t="inlineStr">
@@ -28924,7 +28924,7 @@
       </c>
       <c r="G488" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H488" s="2" t="inlineStr">
@@ -30257,7 +30257,7 @@
       </c>
       <c r="G519" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit</t>
+          <t>MK-MN-M-024 You could cover a $X hit, MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-026 your $X/month of essentials</t>
         </is>
       </c>
       <c r="H519" s="2" t="inlineStr">
@@ -30300,7 +30300,7 @@
       </c>
       <c r="G520" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit</t>
+          <t>MK-MN-M-024 You could cover a $X hit, MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-026 your $X/month of essentials</t>
         </is>
       </c>
       <c r="H520" s="2" t="inlineStr">

</xml_diff>

<commit_message>
A missing balance stays in view on Net worth: 'not entered' by category, by institution and on a debt row — never $0, −$0 or dropped (DEC-3279e, tenet 3)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
+++ b/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
@@ -559,7 +559,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>moneykeel_calc_master_calculation-master_v01.xlsx · census 2026-10-09</t>
+          <t>moneykeel_calc_master_calculation-master_v01.xlsx · census 2026-10-10</t>
         </is>
       </c>
       <c r="C9" s="2" t="n"/>
@@ -15932,22 +15932,22 @@
       </c>
       <c r="D158" s="2" t="inlineStr">
         <is>
-          <t>afternoon | ava | your &lt;name&gt;: $#</t>
+          <t>estimate | social security | $#</t>
         </is>
       </c>
       <c r="E158" s="2" t="inlineStr">
         <is>
-          <t>worker</t>
+          <t>retiree</t>
         </is>
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>spoken, visible</t>
+          <t>visible</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>$4,795 | this month</t>
         </is>
       </c>
       <c r="H158" s="2" t="inlineStr">
@@ -15975,22 +15975,22 @@
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>estimate | social security | $#</t>
+          <t>evening | ava | your &lt;name&gt;: $#</t>
         </is>
       </c>
       <c r="E159" s="2" t="inlineStr">
         <is>
-          <t>retiree</t>
+          <t>worker</t>
         </is>
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>visible</t>
+          <t>spoken, visible</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t>$4,795 | this month</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="H159" s="2" t="inlineStr">
@@ -25643,7 +25643,7 @@
       </c>
       <c r="G409" s="2" t="inlineStr">
         <is>
-          <t>MK-PF-M-014 Wealth generated, MK-PF-M-017 Return, MK-PF-M-006 WHAT EACH CATEGORY EARNED — RETURN</t>
+          <t>MK-PF-M-014 Wealth generated, MK-PF-M-006 WHAT EACH CATEGORY EARNED — RETURN, MK-PF-M-017 Return</t>
         </is>
       </c>
       <c r="H409" s="2" t="inlineStr">
@@ -25729,7 +25729,7 @@
       </c>
       <c r="G411" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-XS-M-006 Income · In (received) · In (take-home)</t>
+          <t>MK-CF-M-034 Your 401(k)s, MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H411" s="2" t="inlineStr">
@@ -25815,7 +25815,7 @@
       </c>
       <c r="G413" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H413" s="2" t="inlineStr">
@@ -25858,7 +25858,7 @@
       </c>
       <c r="G414" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H414" s="2" t="inlineStr">
@@ -25901,7 +25901,7 @@
       </c>
       <c r="G415" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-059 total interest, MK-CF-M-004 each row of the month — what it is and w</t>
+          <t>MK-CF-M-004 each row of the month — what it is and w, MK-CF-M-059 total interest</t>
         </is>
       </c>
       <c r="H415" s="2" t="inlineStr">
@@ -25911,7 +25911,7 @@
       </c>
       <c r="I415" s="2" t="n"/>
     </row>
-    <row r="416" ht="60" customHeight="1">
+    <row r="416" ht="45" customHeight="1">
       <c r="A416" s="2" t="inlineStr">
         <is>
           <t>money figure — more than one row could be it</t>
@@ -25944,7 +25944,7 @@
       </c>
       <c r="G416" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-CF-M-001 Expenses, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
+          <t>MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-CF-M-001 Expenses, MK-CF-M-020 THIS MONTH — free to use</t>
         </is>
       </c>
       <c r="H416" s="2" t="inlineStr">
@@ -25987,7 +25987,7 @@
       </c>
       <c r="G417" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
+          <t>MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-020 THIS MONTH — free to use</t>
         </is>
       </c>
       <c r="H417" s="2" t="inlineStr">
@@ -27621,7 +27621,7 @@
       </c>
       <c r="G455" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H455" s="2" t="inlineStr">
@@ -27664,7 +27664,7 @@
       </c>
       <c r="G456" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H456" s="2" t="inlineStr">
@@ -27707,7 +27707,7 @@
       </c>
       <c r="G457" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H457" s="2" t="inlineStr">
@@ -27879,7 +27879,7 @@
       </c>
       <c r="G461" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-014 Employer 401(k) match</t>
+          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-012 Gross / year</t>
         </is>
       </c>
       <c r="H461" s="2" t="inlineStr">
@@ -28051,7 +28051,7 @@
       </c>
       <c r="G465" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H465" s="2" t="inlineStr">
@@ -28911,7 +28911,7 @@
       </c>
       <c r="G485" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H485" s="2" t="inlineStr">
@@ -28954,7 +28954,7 @@
       </c>
       <c r="G486" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H486" s="2" t="inlineStr">
@@ -28997,7 +28997,7 @@
       </c>
       <c r="G487" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-004 = Guaranteed</t>
         </is>
       </c>
       <c r="H487" s="2" t="inlineStr">
@@ -29040,7 +29040,7 @@
       </c>
       <c r="G488" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-004 = Guaranteed</t>
         </is>
       </c>
       <c r="H488" s="2" t="inlineStr">
@@ -30158,7 +30158,7 @@
       </c>
       <c r="G514" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H514" s="2" t="inlineStr">
@@ -30201,7 +30201,7 @@
       </c>
       <c r="G515" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H515" s="2" t="inlineStr">
@@ -30244,7 +30244,7 @@
       </c>
       <c r="G516" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H516" s="2" t="inlineStr">
@@ -30287,7 +30287,7 @@
       </c>
       <c r="G517" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N</t>
+          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month</t>
         </is>
       </c>
       <c r="H517" s="2" t="inlineStr">
@@ -30373,7 +30373,7 @@
       </c>
       <c r="G519" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-024 You could cover a $X hit</t>
+          <t>MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-024 You could cover a $X hit, MK-MN-M-026 your $X/month of essentials</t>
         </is>
       </c>
       <c r="H519" s="2" t="inlineStr">
@@ -30416,7 +30416,7 @@
       </c>
       <c r="G520" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-024 You could cover a $X hit</t>
+          <t>MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-024 You could cover a $X hit, MK-MN-M-026 your $X/month of essentials</t>
         </is>
       </c>
       <c r="H520" s="2" t="inlineStr">

</xml_diff>

<commit_message>
His decisions DEC-3656 (MK-NW-F-091) and DEC-3657: a worked-back beginning uses a CD's rate and refuses, by name, a holding with no price history; a missing balance reads "Value not entered"
- No daily record: a CD at 5%, $10,500 today, one year back → beginning $10,000, wealth generated $500 (was $10,500 and $0).
- A bond typed by hand: no beginning, no wealth generated; "The beginning can't be worked back: Fidelity Brokerage has no price history."
- Day one opens every window today, so no window back-fills a beginning.
- Net worth: "Ally · Value not entered" (was "Ally · not entered").
- Decision log, Changelog (anchored), ruling notes on Performance v17 and Net worth v08, formulas in words for MK-NW-F-091, F-127..F-130, O-008. 4,691 tests green.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
+++ b/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
@@ -1299,6 +1299,7 @@
 MK-NW-F-048 uberGroupRows
 MK-NW-F-067 plural
 MK-NW-F-068 prettyDay
+MK-NW-F-071 isCertificateOfDeposit
 MK-NW-F-090 windowStartKey
 MK-NW-F-091 pricedGainOf
 MK-NW-F-092 investmentAccountIdsOf
@@ -1312,6 +1313,10 @@
 MK-NW-F-115 liveRent
 MK-NW-F-116 rentedIdsOf
 MK-NW-F-117 propertyUseMap
+MK-NW-F-127 gainOfRow
+MK-NW-F-128 heldValueOf
+MK-NW-F-129 gainRowName
+MK-NW-F-130 cannotWorkBackSentence
 MK-NW-O-004 theEmergencyFund
 MK-NW-O-005 theAlternativesOutlook
 MK-NW-O-008 thePerformance
@@ -1736,6 +1741,7 @@
 MK-NW-F-068 prettyDay
 MK-NW-F-069 priceAtYield
 MK-NW-F-070 accruedInterestCaveat
+MK-NW-F-071 isCertificateOfDeposit
 MK-NW-F-072 rowOf
 MK-NW-F-073 itemising
 MK-NW-F-077 ALL
@@ -1757,6 +1763,10 @@
 MK-NW-F-124 maturityParts
 MK-NW-F-125 isPastMaturity
 MK-NW-F-126 yearlyInterestNow
+MK-NW-F-127 gainOfRow
+MK-NW-F-128 heldValueOf
+MK-NW-F-129 gainRowName
+MK-NW-F-130 cannotWorkBackSentence
 MK-NW-O-001 theBonds
 MK-NW-O-008 thePerformance
 MK-PF-F-001 totalShares
@@ -2330,6 +2340,7 @@
 MK-NW-F-054 reclassifyAccounts
 MK-NW-F-067 plural
 MK-NW-F-068 prettyDay
+MK-NW-F-071 isCertificateOfDeposit
 MK-NW-F-077 ALL
 MK-NW-F-078 ONE
 MK-NW-F-084 categoryEarnings
@@ -2347,6 +2358,10 @@
 MK-NW-F-121 holdingTagClass
 MK-NW-F-122 holdingTagFor
 MK-NW-F-123 holdingNameEvidence
+MK-NW-F-127 gainOfRow
+MK-NW-F-128 heldValueOf
+MK-NW-F-129 gainRowName
+MK-NW-F-130 cannotWorkBackSentence
 MK-NW-O-002 theAccount
 MK-NW-O-008 thePerformance
 MK-PF-F-001 totalShares
@@ -3074,6 +3089,11 @@
 MK-CF-O-010 theMonth
 MK-NW-F-008 incomeBearingClassOf
 MK-NW-F-011 assetClassOf
+MK-NW-F-012 taxTreatmentOf
+MK-NW-F-023 wrapperWord
+MK-NW-F-024 accountLastFour
+MK-NW-F-025 accountDisplayName
+MK-NW-F-026 accountDisplayNames
 MK-NW-F-055 isBond
 MK-NW-F-056 bondInfo
 MK-NW-F-057 annualCoupon
@@ -3084,9 +3104,11 @@
 MK-NW-F-064 bondRateSensitivity
 MK-NW-F-069 priceAtYield
 MK-NW-F-070 accruedInterestCaveat
+MK-NW-F-071 isCertificateOfDeposit
 MK-NW-F-072 rowOf
 MK-NW-F-077 ALL
 MK-NW-F-078 ONE
+MK-NW-F-091 pricedGainOf
 MK-NW-F-104 closedWith
 MK-NW-F-105 whyNoReturn
 MK-NW-F-112 yearlyInterest
@@ -3095,8 +3117,26 @@
 MK-NW-F-124 maturityParts
 MK-NW-F-125 isPastMaturity
 MK-NW-F-126 yearlyInterestNow
+MK-NW-F-127 gainOfRow
+MK-NW-F-128 heldValueOf
+MK-NW-F-129 gainRowName
+MK-NW-F-130 cannotWorkBackSentence
 MK-NW-O-001 theBonds
 MK-NW-O-008 thePerformance
+MK-PF-F-001 totalShares
+MK-PF-F-002 costBasis
+MK-PF-F-004 marketValue
+MK-PF-F-005 unrealizedGain
+MK-PF-F-007 totalROI
+MK-PF-F-008 startDateFor
+MK-PF-F-009 latestClose
+MK-PF-F-010 periodReturn
+MK-PF-F-011 periodReturnSince
+MK-PF-F-012 earliestPurchaseDate
+MK-PF-F-013 benchmarkTicker
+MK-PF-F-014 buildPerformance
+MK-PF-F-029 closeAsOf
+MK-PF-F-031 contractMultiplier
 MK-PL-F-012 waterfall
 MK-ST-F-010 nameEvidence
 MK-ST-F-013 personalFlowTotals
@@ -3134,7 +3174,7 @@
         </is>
       </c>
       <c r="I7" s="2" t="n">
-        <v>126</v>
+        <v>151</v>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
@@ -3214,16 +3254,11 @@
 MK-NW-F-004 portfolioActualReturn
 MK-NW-F-005 accountAllowsTicker
 MK-NW-F-007 assetKind
-MK-NW-F-012 taxTreatmentOf
 MK-NW-F-014 isRealAsset
 MK-NW-F-015 totalAssets
 MK-NW-F-016 cashTotal
 MK-NW-F-021 investmentsTotal
 MK-NW-F-022 investableAssets
-MK-NW-F-023 wrapperWord
-MK-NW-F-024 accountLastFour
-MK-NW-F-025 accountDisplayName
-MK-NW-F-026 accountDisplayNames
 MK-NW-F-027 accountClassBreakdown
 MK-NW-F-029 assetAllocation
 MK-NW-F-030 earmarkDefault
@@ -3245,7 +3280,6 @@
 MK-NW-F-068 prettyDay
 MK-NW-F-084 categoryEarnings
 MK-NW-F-090 windowStartKey
-MK-NW-F-091 pricedGainOf
 MK-NW-F-092 investmentAccountIdsOf
 MK-NW-F-103 investmentRecordDates
 MK-NW-F-106 mortgagesByProperty
@@ -3259,21 +3293,7 @@
 MK-NW-F-122 holdingTagFor
 MK-NW-F-123 holdingNameEvidence
 MK-NW-O-003 theNetWorth
-MK-PF-F-001 totalShares
-MK-PF-F-002 costBasis
-MK-PF-F-004 marketValue
-MK-PF-F-005 unrealizedGain
-MK-PF-F-007 totalROI
-MK-PF-F-008 startDateFor
-MK-PF-F-009 latestClose
-MK-PF-F-010 periodReturn
-MK-PF-F-011 periodReturnSince
-MK-PF-F-012 earliestPurchaseDate
-MK-PF-F-013 benchmarkTicker
-MK-PF-F-014 buildPerformance
 MK-PF-F-020 portfolioBenchReturn
-MK-PF-F-029 closeAsOf
-MK-PF-F-031 contractMultiplier
 MK-PF-F-034 closeOnOrBefore
 MK-PL-F-001 taxBucketSplit
 MK-PL-F-011 buildGoalsState
@@ -3374,19 +3394,19 @@
         <is>
           <t>MK-XS-I-001 account balance — read by MK-NW-F-056, MK-NW-F-078, MK-NW-O-001, MK-NW-O-008, MK-ST-F-027, MK-ST-F-028
 MK-XS-I-001 account balance — read by MK-ST-F-027
-MK-XS-I-002 account type (taxable, pre-tax, Roth) — read by MK-NW-F-011, MK-NW-F-120, MK-NW-O-001
-MK-XS-I-003 institution name — read by MK-NW-F-056, MK-NW-F-072, MK-NW-O-001
-MK-XS-I-004 holding quantity (shares) — read by MK-CF-F-062, MK-ST-F-027, MK-ST-F-028, MK-ST-F-082
+MK-XS-I-002 account type (taxable, pre-tax, Roth) — read by MK-NW-F-011, MK-NW-F-012, MK-NW-F-025, MK-NW-F-120, MK-NW-O-001
+MK-XS-I-003 institution name — read by MK-NW-F-025, MK-NW-F-026, MK-NW-F-056, MK-NW-F-071, MK-NW-F-072, MK-NW-O-001
+MK-XS-I-004 holding quantity (shares) — read by MK-CF-F-062, MK-NW-F-091, MK-NW-F-128, MK-PF-F-001, MK-PF-F-002, MK-PF-F-004, MK
 MK-XS-I-004 holding quantity (shares) — read by MK-ST-F-027
+MK-XS-I-005 holding price — read by MK-NW-F-091, MK-NW-F-128, MK-PF-F-009, MK-PF-F-010, MK-PF-F-011, MK-PF-F-014, MK
 MK-XS-I-005 holding price — read by MK-ST-F-027
-MK-XS-I-005 holding price — read by MK-ST-F-027, MK-ST-F-028
+MK-XS-I-007 purchase price and date (per lot) — read by MK-PF-F-002, MK-PF-F-005, MK-PF-F-007, MK-PF-F-012, MK-PF-F-013, MK-PF-F-014, MK
 MK-XS-I-007 purchase price and date (per lot) — read by MK-ST-F-027
-MK-XS-I-007 purchase price and date (per lot) — read by MK-ST-F-027, MK-ST-F-028
 MK-XS-I-009 transaction date — read by MK-NW-O-008
 MK-XS-I-010 transaction words (the institution's own wording) — read by MK-ST-F-013
 MK-XS-I-011 bond face value — read by MK-NW-F-056, MK-NW-F-057, MK-NW-F-060, MK-NW-F-061, MK-NW-F-064, MK-NW-F-069, MK
-MK-XS-I-012 bond coupon rate — read by MK-NW-F-056, MK-NW-F-057, MK-NW-F-060, MK-NW-F-064, MK-NW-F-070, MK-NW-F-072, MK
-MK-XS-I-013 bond maturity date — read by MK-NW-F-056, MK-NW-F-058, MK-NW-F-060, MK-NW-F-061, MK-NW-F-069, MK-NW-F-072, MK
+MK-XS-I-012 bond coupon rate — read by MK-NW-F-056, MK-NW-F-057, MK-NW-F-060, MK-NW-F-064, MK-NW-F-070, MK-NW-F-071, MK
+MK-XS-I-013 bond maturity date — read by MK-NW-F-056, MK-NW-F-058, MK-NW-F-060, MK-NW-F-061, MK-NW-F-069, MK-NW-F-071, MK
 MK-XS-I-014 debt balance — read by MK-CF-F-157, MK-CF-O-010
 MK-XS-I-015 debt interest rate — read by MK-CF-F-157, MK-CF-O-010
 MK-XS-I-016 debt minimum payment — read by MK-CF-F-023, MK-CF-F-157, MK-CF-O-010
@@ -3415,9 +3435,10 @@
 MK-XS-I-048 the person’s own asset-class answer — read by MK-ST-F-027
 MK-XS-I-049 bond price — what the bond is worth today — read by MK-NW-F-056, MK-NW-F-057, MK-NW-F-059, MK-NW-F-060, MK-NW-F-061, MK-NW-F-064, MK
 MK-XS-I-052 the day of the month a debt payment is due — read by MK-CF-F-005
-MK-XS-I-055 the wrapper an account sits in — ISA, 401(k), IRA and the rest — read by MK-CF-F-005, MK-CF-F-075, MK-CF-F-156, MK-NW-F-011, MK-NW-F-056, MK-NW-F-120, MK
+MK-XS-I-055 the wrapper an account sits in — ISA, 401(k), IRA and the rest — read by MK-CF-F-005, MK-CF-F-075, MK-CF-F-156, MK-NW-F-011, MK-NW-F-012, MK-NW-F-023, MK
 MK-XS-I-059 the month a bonus lands — read by MK-CF-F-088, MK-CF-F-092
 MK-XS-I-060 how a person is paid — weekly, fortnightly, monthly — read by MK-CF-F-130
+MK-XS-I-063 option contract multiplier — 100 unless the broker or the person states otherwise — read by MK-PF-F-002, MK-PF-F-004, MK-PF-F-031
 MK-XS-I-064 the unit beside a quantity — shares, coins, contracts, ounces or units — read by MK-CF-F-003, MK-CF-F-008, MK-CF-F-204, MK-NW-F-078
 MK-XS-I-065 accrued interest on a bond — interest earned since the last coupon — read by MK-NW-F-056, MK-NW-F-060, MK-NW-F-070, MK-NW-F-072
 [the code's record, this build — evidence for the ruling, not the row's statement: it cannot see inputs handed in as arguments, and it counts every branch below the producer]</t>
@@ -3981,6 +4002,7 @@
 MK-NW-F-048 uberGroupRows
 MK-NW-F-067 plural
 MK-NW-F-068 prettyDay
+MK-NW-F-071 isCertificateOfDeposit
 MK-NW-F-090 windowStartKey
 MK-NW-F-091 pricedGainOf
 MK-NW-F-092 investmentAccountIdsOf
@@ -3988,6 +4010,10 @@
 MK-NW-F-104 closedWith
 MK-NW-F-105 whyNoReturn
 MK-NW-F-107 propertyUses
+MK-NW-F-127 gainOfRow
+MK-NW-F-128 heldValueOf
+MK-NW-F-129 gainRowName
+MK-NW-F-130 cannotWorkBackSentence
 MK-NW-O-004 theEmergencyFund
 MK-NW-O-008 thePerformance
 MK-PF-F-005 unrealizedGain
@@ -6512,12 +6538,16 @@
 MK-HM-F-004 milestoneCrossed
 MK-NW-F-004 portfolioActualReturn
 MK-NW-F-007 assetKind
+MK-NW-F-012 taxTreatmentOf
 MK-NW-F-014 isRealAsset
 MK-NW-F-015 totalAssets
 MK-NW-F-016 cashTotal
 MK-NW-F-021 investmentsTotal
 MK-NW-F-022 investableAssets
 MK-NW-F-023 wrapperWord
+MK-NW-F-024 accountLastFour
+MK-NW-F-025 accountDisplayName
+MK-NW-F-026 accountDisplayNames
 MK-NW-F-027 accountClassBreakdown
 MK-NW-F-029 assetAllocation
 MK-NW-F-030 earmarkDefault
@@ -6537,6 +6567,7 @@
 MK-NW-F-066 sumWhere
 MK-NW-F-067 plural
 MK-NW-F-068 prettyDay
+MK-NW-F-071 isCertificateOfDeposit
 MK-NW-F-090 windowStartKey
 MK-NW-F-091 pricedGainOf
 MK-NW-F-092 investmentAccountIdsOf
@@ -6553,6 +6584,10 @@
 MK-NW-F-121 holdingTagClass
 MK-NW-F-122 holdingTagFor
 MK-NW-F-123 holdingNameEvidence
+MK-NW-F-127 gainOfRow
+MK-NW-F-128 heldValueOf
+MK-NW-F-129 gainRowName
+MK-NW-F-130 cannotWorkBackSentence
 MK-NW-O-003 theNetWorth
 MK-NW-O-008 thePerformance
 MK-PF-F-001 totalShares
@@ -7114,12 +7149,16 @@
 MK-HM-F-006 money0
 MK-NW-F-004 portfolioActualReturn
 MK-NW-F-007 assetKind
+MK-NW-F-012 taxTreatmentOf
 MK-NW-F-014 isRealAsset
 MK-NW-F-015 totalAssets
 MK-NW-F-016 cashTotal
 MK-NW-F-021 investmentsTotal
 MK-NW-F-022 investableAssets
 MK-NW-F-023 wrapperWord
+MK-NW-F-024 accountLastFour
+MK-NW-F-025 accountDisplayName
+MK-NW-F-026 accountDisplayNames
 MK-NW-F-027 accountClassBreakdown
 MK-NW-F-029 assetAllocation
 MK-NW-F-030 earmarkDefault
@@ -7136,6 +7175,7 @@
 MK-NW-F-054 reclassifyAccounts
 MK-NW-F-065 buildNetWorth
 MK-NW-F-066 sumWhere
+MK-NW-F-071 isCertificateOfDeposit
 MK-NW-F-090 windowStartKey
 MK-NW-F-091 pricedGainOf
 MK-NW-F-092 investmentAccountIdsOf
@@ -7152,6 +7192,10 @@
 MK-NW-F-121 holdingTagClass
 MK-NW-F-122 holdingTagFor
 MK-NW-F-123 holdingNameEvidence
+MK-NW-F-127 gainOfRow
+MK-NW-F-128 heldValueOf
+MK-NW-F-129 gainRowName
+MK-NW-F-130 cannotWorkBackSentence
 MK-NW-O-003 theNetWorth
 MK-NW-O-008 thePerformance
 MK-PF-F-001 totalShares
@@ -8054,12 +8098,16 @@
 MK-NW-F-007 assetKind
 MK-NW-F-008 incomeBearingClassOf
 MK-NW-F-011 assetClassOf
+MK-NW-F-012 taxTreatmentOf
 MK-NW-F-014 isRealAsset
 MK-NW-F-015 totalAssets
 MK-NW-F-016 cashTotal
 MK-NW-F-021 investmentsTotal
 MK-NW-F-022 investableAssets
 MK-NW-F-023 wrapperWord
+MK-NW-F-024 accountLastFour
+MK-NW-F-025 accountDisplayName
+MK-NW-F-026 accountDisplayNames
 MK-NW-F-027 accountClassBreakdown
 MK-NW-F-029 assetAllocation
 MK-NW-F-030 earmarkDefault
@@ -8086,6 +8134,7 @@
 MK-NW-F-066 sumWhere
 MK-NW-F-069 priceAtYield
 MK-NW-F-070 accruedInterestCaveat
+MK-NW-F-071 isCertificateOfDeposit
 MK-NW-F-072 rowOf
 MK-NW-F-077 ALL
 MK-NW-F-078 ONE
@@ -8110,6 +8159,10 @@
 MK-NW-F-124 maturityParts
 MK-NW-F-125 isPastMaturity
 MK-NW-F-126 yearlyInterestNow
+MK-NW-F-127 gainOfRow
+MK-NW-F-128 heldValueOf
+MK-NW-F-129 gainRowName
+MK-NW-F-130 cannotWorkBackSentence
 MK-NW-O-001 theBonds
 MK-NW-O-003 theNetWorth
 MK-NW-O-008 thePerformance
@@ -8929,12 +8982,16 @@
 MK-NW-F-007 assetKind
 MK-NW-F-008 incomeBearingClassOf
 MK-NW-F-011 assetClassOf
+MK-NW-F-012 taxTreatmentOf
 MK-NW-F-014 isRealAsset
 MK-NW-F-015 totalAssets
 MK-NW-F-016 cashTotal
 MK-NW-F-021 investmentsTotal
 MK-NW-F-022 investableAssets
 MK-NW-F-023 wrapperWord
+MK-NW-F-024 accountLastFour
+MK-NW-F-025 accountDisplayName
+MK-NW-F-026 accountDisplayNames
 MK-NW-F-027 accountClassBreakdown
 MK-NW-F-029 assetAllocation
 MK-NW-F-030 earmarkDefault
@@ -8961,6 +9018,7 @@
 MK-NW-F-066 sumWhere
 MK-NW-F-069 priceAtYield
 MK-NW-F-070 accruedInterestCaveat
+MK-NW-F-071 isCertificateOfDeposit
 MK-NW-F-072 rowOf
 MK-NW-F-077 ALL
 MK-NW-F-078 ONE
@@ -8986,6 +9044,10 @@
 MK-NW-F-124 maturityParts
 MK-NW-F-125 isPastMaturity
 MK-NW-F-126 yearlyInterestNow
+MK-NW-F-127 gainOfRow
+MK-NW-F-128 heldValueOf
+MK-NW-F-129 gainRowName
+MK-NW-F-130 cannotWorkBackSentence
 MK-NW-O-001 theBonds
 MK-NW-O-003 theNetWorth
 MK-NW-O-004 theEmergencyFund
@@ -25643,7 +25705,7 @@
       </c>
       <c r="G409" s="2" t="inlineStr">
         <is>
-          <t>MK-PF-M-014 Wealth generated, MK-PF-M-006 WHAT EACH CATEGORY EARNED — RETURN, MK-PF-M-017 Return</t>
+          <t>MK-PF-M-014 Wealth generated, MK-PF-M-017 Return, MK-PF-M-006 WHAT EACH CATEGORY EARNED — RETURN</t>
         </is>
       </c>
       <c r="H409" s="2" t="inlineStr">
@@ -25729,7 +25791,7 @@
       </c>
       <c r="G411" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-034 Your 401(k)s, MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
+          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-020 THIS MONTH — free to use, MK-XS-M-006 Income · In (received) · In (take-home)</t>
         </is>
       </c>
       <c r="H411" s="2" t="inlineStr">
@@ -25987,7 +26049,7 @@
       </c>
       <c r="G417" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-020 THIS MONTH — free to use</t>
         </is>
       </c>
       <c r="H417" s="2" t="inlineStr">
@@ -26030,7 +26092,7 @@
       </c>
       <c r="G418" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-020 THIS MONTH — free to use, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H418" s="2" t="inlineStr">
@@ -27062,7 +27124,7 @@
       </c>
       <c r="G442" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
+          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
         </is>
       </c>
       <c r="H442" s="2" t="inlineStr">
@@ -27148,7 +27210,7 @@
       </c>
       <c r="G444" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
+          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
         </is>
       </c>
       <c r="H444" s="2" t="inlineStr">
@@ -27191,7 +27253,7 @@
       </c>
       <c r="G445" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
+          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
         </is>
       </c>
       <c r="H445" s="2" t="inlineStr">
@@ -27406,7 +27468,7 @@
       </c>
       <c r="G450" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
+          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
         </is>
       </c>
       <c r="H450" s="2" t="inlineStr">
@@ -27750,7 +27812,7 @@
       </c>
       <c r="G458" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-012 Gross / year</t>
+          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H458" s="2" t="inlineStr">
@@ -27793,7 +27855,7 @@
       </c>
       <c r="G459" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-012 Gross / year</t>
+          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H459" s="2" t="inlineStr">
@@ -27879,7 +27941,7 @@
       </c>
       <c r="G461" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-012 Gross / year</t>
+          <t>MK-MN-M-014 Employer 401(k) match, MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H461" s="2" t="inlineStr">
@@ -28868,7 +28930,7 @@
       </c>
       <c r="G484" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed</t>
         </is>
       </c>
       <c r="H484" s="2" t="inlineStr">
@@ -28911,7 +28973,7 @@
       </c>
       <c r="G485" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-004 = Guaranteed</t>
         </is>
       </c>
       <c r="H485" s="2" t="inlineStr">
@@ -28954,7 +29016,7 @@
       </c>
       <c r="G486" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H486" s="2" t="inlineStr">
@@ -28997,7 +29059,7 @@
       </c>
       <c r="G487" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H487" s="2" t="inlineStr">

</xml_diff>

<commit_message>
His decisions of 2026-10-10 on OpenAI's open points: month-end windows (DEC-3768b), rent with words refused (DEC-3768c), "rent not included" on the emergency fund (DEC-3769)
- 1M from Mar 31 starts Feb 28 (was Mar 3); a year before Feb 29 is Feb 28 — windowStartKey and startDateFor.
- "about 2k" is not read as $2: one strict rent reader for rentAmount and rentalList; the Income screen refuses a change carrying a letter.
- Net worth emergency fund: "5.0 months, rent not included. Enter rent to include." when a rent entry has no amount; a tap opens Income.
- Decision log (with split), Changelog rows anchored, Net worth v08 note, formulas in words. 4,706 tests green.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
+++ b/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
@@ -1212,6 +1212,7 @@
 MK-ST-F-082 movementsOf
 MK-ST-F-083 accountValuesOn
 MK-ST-F-084 fillBetweenObservations
+MK-ST-F-085 rentFigure
 MK-XS-F-005 trendPoints
 MK-XS-F-006 pruneDaily
 MK-XS-F-008 normalizeSnapshot
@@ -1232,7 +1233,7 @@
         </is>
       </c>
       <c r="I2" s="2" t="n">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
@@ -1808,6 +1809,7 @@
 MK-ST-F-081 timeWeightedReturn
 MK-ST-F-082 movementsOf
 MK-ST-F-083 accountValuesOn
+MK-ST-F-085 rentFigure
 MK-XS-F-011 buildChangeWalk
 MK-XS-F-024 resolveLens
 MK-XS-F-025 tabOrder
@@ -2084,6 +2086,7 @@
 MK-ST-F-065 isoLocalDate
 MK-ST-F-075 agoLabel
 MK-ST-F-077 isStale
+MK-ST-F-085 rentFigure
 MK-XS-F-024 resolveLens
 MK-XS-F-025 tabOrder
 MK-XS-F-027 takeHomeMonthly
@@ -2405,6 +2408,7 @@
 MK-ST-F-081 timeWeightedReturn
 MK-ST-F-082 movementsOf
 MK-ST-F-083 accountValuesOn
+MK-ST-F-085 rentFigure
 MK-XS-F-011 buildChangeWalk
 MK-XS-F-024 resolveLens
 MK-XS-F-025 tabOrder
@@ -2651,6 +2655,7 @@
 MK-ST-F-053 money
 MK-ST-F-056 has
 MK-ST-F-065 isoLocalDate
+MK-ST-F-085 rentFigure
 MK-XS-F-027 takeHomeMonthly
 MK-XS-F-064 currentIdToken
 MK-XS-F-112 relayUrl
@@ -2660,7 +2665,7 @@
         </is>
       </c>
       <c r="I6" s="2" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
@@ -3164,6 +3169,7 @@
 MK-ST-F-081 timeWeightedReturn
 MK-ST-F-082 movementsOf
 MK-ST-F-083 accountValuesOn
+MK-ST-F-085 rentFigure
 MK-XS-F-011 buildChangeWalk
 MK-XS-F-027 takeHomeMonthly
 MK-XS-F-064 currentIdToken
@@ -3174,7 +3180,7 @@
         </is>
       </c>
       <c r="I7" s="2" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
@@ -3919,6 +3925,7 @@
 MK-ST-F-082 movementsOf
 MK-ST-F-083 accountValuesOn
 MK-ST-F-084 fillBetweenObservations
+MK-ST-F-085 rentFigure
 MK-XS-F-005 trendPoints
 MK-XS-F-006 pruneDaily
 MK-XS-F-008 normalizeSnapshot
@@ -3939,7 +3946,7 @@
         </is>
       </c>
       <c r="I9" s="2" t="n">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
@@ -4506,6 +4513,7 @@
 MK-ST-F-053 money
 MK-ST-F-056 has
 MK-ST-F-065 isoLocalDate
+MK-ST-F-085 rentFigure
 MK-XS-F-004 buildDatedGrid
 MK-XS-F-027 takeHomeMonthly
 MK-XS-F-064 currentIdToken
@@ -4516,7 +4524,7 @@
         </is>
       </c>
       <c r="I10" s="2" t="n">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
@@ -5017,6 +5025,7 @@
 MK-ST-F-073 rebuildDays
 MK-ST-F-079 dailyWindowStart
 MK-ST-F-084 fillBetweenObservations
+MK-ST-F-085 rentFigure
 MK-XS-F-006 pruneDaily
 MK-XS-F-017 currentAge
 MK-XS-F-024 resolveLens
@@ -5186,6 +5195,7 @@
 MK-ST-F-052 toNum
 MK-ST-F-056 has
 MK-ST-F-065 isoLocalDate
+MK-ST-F-085 rentFigure
 MK-XS-F-064 currentIdToken
 MK-XS-F-084 requestNotificationPermission
 MK-XS-F-087 scheduleRmdReminder
@@ -5445,6 +5455,7 @@
 MK-ST-F-073 rebuildDays
 MK-ST-F-079 dailyWindowStart
 MK-ST-F-084 fillBetweenObservations
+MK-ST-F-085 rentFigure
 MK-XS-F-006 pruneDaily
 MK-XS-F-017 currentAge
 MK-XS-F-024 resolveLens
@@ -5704,6 +5715,7 @@
 MK-ST-F-053 money
 MK-ST-F-056 has
 MK-ST-F-065 isoLocalDate
+MK-ST-F-085 rentFigure
 MK-XS-F-017 currentAge
 MK-XS-F-027 takeHomeMonthly
 MK-XS-F-064 currentIdToken
@@ -5715,7 +5727,7 @@
         </is>
       </c>
       <c r="I14" s="2" t="n">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
@@ -6201,6 +6213,7 @@
 MK-ST-F-039 on
 MK-ST-F-052 toNum
 MK-ST-F-056 has
+MK-ST-F-085 rentFigure
 MK-XS-F-064 currentIdToken
 MK-XS-F-112 relayUrl
 MK-XS-F-122 n
@@ -6449,6 +6462,7 @@
 MK-ST-F-053 money
 MK-ST-F-056 has
 MK-ST-F-065 isoLocalDate
+MK-ST-F-085 rentFigure
 MK-XS-F-027 takeHomeMonthly
 MK-XS-F-064 currentIdToken
 MK-XS-F-112 relayUrl
@@ -6458,7 +6472,7 @@
         </is>
       </c>
       <c r="I17" s="2" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
@@ -7050,6 +7064,7 @@
 MK-ST-F-053 money
 MK-ST-F-056 has
 MK-ST-F-065 isoLocalDate
+MK-ST-F-085 rentFigure
 MK-XS-F-027 takeHomeMonthly
 MK-XS-F-064 currentIdToken
 MK-XS-F-112 relayUrl
@@ -7059,7 +7074,7 @@
         </is>
       </c>
       <c r="I18" s="2" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
@@ -7622,6 +7637,7 @@
 MK-ST-F-053 money
 MK-ST-F-056 has
 MK-ST-F-065 isoLocalDate
+MK-ST-F-085 rentFigure
 MK-XS-F-027 takeHomeMonthly
 MK-XS-F-064 currentIdToken
 MK-XS-F-112 relayUrl
@@ -7631,7 +7647,7 @@
         </is>
       </c>
       <c r="I19" s="2" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
@@ -8257,6 +8273,7 @@
 MK-ST-F-082 movementsOf
 MK-ST-F-083 accountValuesOn
 MK-ST-F-084 fillBetweenObservations
+MK-ST-F-085 rentFigure
 MK-XS-F-005 trendPoints
 MK-XS-F-006 pruneDaily
 MK-XS-F-007 makeMonthlySnapshot
@@ -8449,11 +8466,12 @@
 MK-ST-F-039 on
 MK-ST-F-052 toNum
 MK-ST-F-056 has
+MK-ST-F-085 rentFigure
 MK-XS-F-122 n</t>
         </is>
       </c>
       <c r="I21" s="2" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
@@ -8691,6 +8709,7 @@
 MK-ST-F-053 money
 MK-ST-F-056 has
 MK-ST-F-065 isoLocalDate
+MK-ST-F-085 rentFigure
 MK-XS-F-027 takeHomeMonthly
 MK-XS-F-064 currentIdToken
 MK-XS-F-112 relayUrl
@@ -8700,7 +8719,7 @@
         </is>
       </c>
       <c r="I22" s="2" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
@@ -9150,6 +9169,7 @@
 MK-ST-F-082 movementsOf
 MK-ST-F-083 accountValuesOn
 MK-ST-F-084 fillBetweenObservations
+MK-ST-F-085 rentFigure
 MK-XS-F-005 trendPoints
 MK-XS-F-006 pruneDaily
 MK-XS-F-007 makeMonthlySnapshot
@@ -9502,6 +9522,7 @@
 MK-ST-F-082 movementsOf
 MK-ST-F-083 accountValuesOn
 MK-ST-F-084 fillBetweenObservations
+MK-ST-F-085 rentFigure
 MK-XS-F-005 trendPoints
 MK-XS-F-006 pruneDaily
 MK-XS-F-008 normalizeSnapshot
@@ -16037,7 +16058,7 @@
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>evening | ava | your &lt;name&gt;: $#</t>
+          <t>morning | ava | your &lt;name&gt;: $#</t>
         </is>
       </c>
       <c r="E159" s="2" t="inlineStr">
@@ -25791,7 +25812,7 @@
       </c>
       <c r="G411" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-020 THIS MONTH — free to use, MK-XS-M-006 Income · In (received) · In (take-home)</t>
+          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-XS-M-006 Income · In (received) · In (take-home)</t>
         </is>
       </c>
       <c r="H411" s="2" t="inlineStr">
@@ -25877,7 +25898,7 @@
       </c>
       <c r="G413" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-007 Left / Over · left to spend this month</t>
         </is>
       </c>
       <c r="H413" s="2" t="inlineStr">
@@ -25920,7 +25941,7 @@
       </c>
       <c r="G414" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-007 Left / Over · left to spend this month</t>
         </is>
       </c>
       <c r="H414" s="2" t="inlineStr">
@@ -27769,7 +27790,7 @@
       </c>
       <c r="G457" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-007 Left / Over · left to spend this month</t>
         </is>
       </c>
       <c r="H457" s="2" t="inlineStr">
@@ -27941,7 +27962,7 @@
       </c>
       <c r="G461" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-014 Employer 401(k) match, MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month</t>
+          <t>MK-MN-M-012 Gross / year, MK-MN-M-014 Employer 401(k) match, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H461" s="2" t="inlineStr">
@@ -28113,7 +28134,7 @@
       </c>
       <c r="G465" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-007 Left / Over · left to spend this month</t>
         </is>
       </c>
       <c r="H465" s="2" t="inlineStr">
@@ -28930,7 +28951,7 @@
       </c>
       <c r="G484" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H484" s="2" t="inlineStr">
@@ -28973,7 +28994,7 @@
       </c>
       <c r="G485" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H485" s="2" t="inlineStr">
@@ -29016,7 +29037,7 @@
       </c>
       <c r="G486" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H486" s="2" t="inlineStr">
@@ -29059,7 +29080,7 @@
       </c>
       <c r="G487" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H487" s="2" t="inlineStr">
@@ -29102,7 +29123,7 @@
       </c>
       <c r="G488" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed, MK-PL-M-005 + Draw from savings</t>
         </is>
       </c>
       <c r="H488" s="2" t="inlineStr">
@@ -30220,7 +30241,7 @@
       </c>
       <c r="G514" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H514" s="2" t="inlineStr">
@@ -30263,7 +30284,7 @@
       </c>
       <c r="G515" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H515" s="2" t="inlineStr">
@@ -30306,7 +30327,7 @@
       </c>
       <c r="G516" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H516" s="2" t="inlineStr">
@@ -30349,7 +30370,7 @@
       </c>
       <c r="G517" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N</t>
         </is>
       </c>
       <c r="H517" s="2" t="inlineStr">

</xml_diff>

<commit_message>
His decisions DEC-3836 and DEC-3837: "rent not included" wherever the emergency-fund months show; a CD bought through a broker is priced like a bond
- DEC-3836: Stress test, Job safety, Insights and Home's card carry "… months, rent not included. Enter rent to include." (Net worth already did); no number changed.
- DEC-3837: a CD asks once "Bought from the bank, or through a broker?" (Add an account and the Bonds form). Bank CD: yield = its rate (4.20%), no rate-move estimate; a bank CD with no face now yields its rate. Broker CD: worked out like a bond — $10,000 face, 4.2%, worth $9,850, 2 years → about 5.01% — with the rate-move estimate and accrued-interest note. Existing CDs read as bank CDs.
- Decision log (not-a-repeat notes for DEC-3769, DEC-2748b/f), Changelog anchored, ruling notes on Bonds v02 and Add an account by hand v02, formulas in words. 4,732 tests green.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
+++ b/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
@@ -1166,6 +1166,7 @@
 MK-NW-F-124 maturityParts
 MK-NW-F-125 isPastMaturity
 MK-NW-F-126 yearlyInterestNow
+MK-NW-F-131 pricedLikeBond
 MK-NW-O-001 theBonds
 MK-NW-O-003 theNetWorth
 MK-PF-F-001 totalShares
@@ -1233,7 +1234,7 @@
         </is>
       </c>
       <c r="I2" s="2" t="n">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
@@ -1768,6 +1769,7 @@
 MK-NW-F-128 heldValueOf
 MK-NW-F-129 gainRowName
 MK-NW-F-130 cannotWorkBackSentence
+MK-NW-F-131 pricedLikeBond
 MK-NW-O-001 theBonds
 MK-NW-O-008 thePerformance
 MK-PF-F-001 totalShares
@@ -2051,6 +2053,7 @@
 MK-NW-F-124 maturityParts
 MK-NW-F-125 isPastMaturity
 MK-NW-F-126 yearlyInterestNow
+MK-NW-F-131 pricedLikeBond
 MK-NW-O-001 theBonds
 MK-PF-F-005 unrealizedGain
 MK-PF-F-007 totalROI
@@ -2241,6 +2244,7 @@
 MK-NW-F-124 maturityParts
 MK-NW-F-125 isPastMaturity
 MK-NW-F-126 yearlyInterestNow
+MK-NW-F-131 pricedLikeBond
 MK-NW-O-001 theBonds
 MK-ST-F-010 nameEvidence
 MK-ST-F-027 accountId
@@ -2253,7 +2257,7 @@
         </is>
       </c>
       <c r="I5" s="2" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
@@ -2446,7 +2450,7 @@
 MK-XS-I-028 assumed return — read by MK-NW-O-001
 MK-XS-I-048 the person’s own asset-class answer — read by MK-NW-F-011, MK-ST-F-027
 MK-XS-I-049 bond price — what the bond is worth today — read by MK-NW-F-056, MK-NW-F-057, MK-NW-F-059, MK-NW-F-060, MK-NW-F-061, MK-NW-F-064, MK
-MK-XS-I-049 bond price — what the bond is worth today — read by MK-NW-F-057, MK-NW-F-060, MK-NW-F-064, MK-NW-F-069, MK-NW-F-119
+MK-XS-I-049 bond price — what the bond is worth today — read by MK-NW-F-057, MK-NW-F-060, MK-NW-F-064, MK-NW-F-069, MK-NW-F-119, MK-NW-F-131
 MK-XS-I-055 the wrapper an account sits in — ISA, 401(k), IRA and the rest — read by MK-NW-F-011, MK-NW-F-056, MK-NW-F-120, MK-NW-O-001
 MK-XS-I-065 accrued interest on a bond — interest earned since the last coupon — read by MK-NW-F-056, MK-NW-F-060, MK-NW-F-070, MK-NW-F-072
 MK-XS-I-065 accrued interest on a bond — interest earned since the last coupon — read by MK-NW-F-060
@@ -2457,7 +2461,8 @@
         <is>
           <t>An approximation, and labelled an estimate on screen.
 An estimate, and it wears the estimate label.
-FOUNDER 2026-09-27: a CD gets no estimate. It is not traded, so its value does not move with rates; the screen says that instead. KEEP — the app does not ask whether a CD is a bank one or a brokered one.
+DEC-3837, 2026-10-10: a CD bought through a broker trades, so it gets the estimate like a bond. A CD whose answer was never given is read as bought from the bank.
+FOUNDER 2026-09-27: a CD bought from the bank gets no estimate. It is not traded, so its value does not move with rates; the screen says that instead.
 NONE RECORDED — the declaration names none.</t>
         </is>
       </c>
@@ -2642,6 +2647,7 @@
 MK-NW-F-124 maturityParts
 MK-NW-F-125 isPastMaturity
 MK-NW-F-126 yearlyInterestNow
+MK-NW-F-131 pricedLikeBond
 MK-NW-O-001 theBonds
 MK-PL-F-012 waterfall
 MK-ST-F-010 nameEvidence
@@ -2665,7 +2671,7 @@
         </is>
       </c>
       <c r="I6" s="2" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
@@ -3126,6 +3132,7 @@
 MK-NW-F-128 heldValueOf
 MK-NW-F-129 gainRowName
 MK-NW-F-130 cannotWorkBackSentence
+MK-NW-F-131 pricedLikeBond
 MK-NW-O-001 theBonds
 MK-NW-O-008 thePerformance
 MK-PF-F-001 totalShares
@@ -3180,7 +3187,7 @@
         </is>
       </c>
       <c r="I7" s="2" t="n">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
@@ -3860,6 +3867,7 @@
 MK-NW-F-124 maturityParts
 MK-NW-F-125 isPastMaturity
 MK-NW-F-126 yearlyInterestNow
+MK-NW-F-131 pricedLikeBond
 MK-NW-O-001 theBonds
 MK-NW-O-003 theNetWorth
 MK-PF-F-001 totalShares
@@ -3946,7 +3954,7 @@
         </is>
       </c>
       <c r="I9" s="2" t="n">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
@@ -4491,6 +4499,7 @@
 MK-NW-F-124 maturityParts
 MK-NW-F-125 isPastMaturity
 MK-NW-F-126 yearlyInterestNow
+MK-NW-F-131 pricedLikeBond
 MK-NW-O-001 theBonds
 MK-PL-F-012 waterfall
 MK-PL-F-050 simulate
@@ -4524,7 +4533,7 @@
         </is>
       </c>
       <c r="I10" s="2" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
@@ -5680,6 +5689,7 @@
 MK-NW-F-124 maturityParts
 MK-NW-F-125 isPastMaturity
 MK-NW-F-126 yearlyInterestNow
+MK-NW-F-131 pricedLikeBond
 MK-NW-O-001 theBonds
 MK-PL-F-001 taxBucketSplit
 MK-PL-F-012 waterfall
@@ -5727,7 +5737,7 @@
         </is>
       </c>
       <c r="I14" s="2" t="n">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
@@ -6447,6 +6457,7 @@
 MK-NW-F-124 maturityParts
 MK-NW-F-125 isPastMaturity
 MK-NW-F-126 yearlyInterestNow
+MK-NW-F-131 pricedLikeBond
 MK-NW-O-001 theBonds
 MK-PL-F-012 waterfall
 MK-ST-F-010 nameEvidence
@@ -6472,7 +6483,7 @@
         </is>
       </c>
       <c r="I17" s="2" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
@@ -7051,6 +7062,7 @@
 MK-NW-F-124 maturityParts
 MK-NW-F-125 isPastMaturity
 MK-NW-F-126 yearlyInterestNow
+MK-NW-F-131 pricedLikeBond
 MK-NW-O-001 theBonds
 MK-PL-F-012 waterfall
 MK-ST-F-010 nameEvidence
@@ -7074,7 +7086,7 @@
         </is>
       </c>
       <c r="I18" s="2" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
@@ -7624,6 +7636,7 @@
 MK-NW-F-124 maturityParts
 MK-NW-F-125 isPastMaturity
 MK-NW-F-126 yearlyInterestNow
+MK-NW-F-131 pricedLikeBond
 MK-NW-O-001 theBonds
 MK-PL-F-012 waterfall
 MK-ST-F-010 nameEvidence
@@ -7647,7 +7660,7 @@
         </is>
       </c>
       <c r="I19" s="2" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
@@ -8179,6 +8192,7 @@
 MK-NW-F-128 heldValueOf
 MK-NW-F-129 gainRowName
 MK-NW-F-130 cannotWorkBackSentence
+MK-NW-F-131 pricedLikeBond
 MK-NW-O-001 theBonds
 MK-NW-O-003 theNetWorth
 MK-NW-O-008 thePerformance
@@ -8696,6 +8710,7 @@
 MK-NW-F-124 maturityParts
 MK-NW-F-125 isPastMaturity
 MK-NW-F-126 yearlyInterestNow
+MK-NW-F-131 pricedLikeBond
 MK-NW-O-001 theBonds
 MK-PL-F-012 waterfall
 MK-ST-F-010 nameEvidence
@@ -8719,7 +8734,7 @@
         </is>
       </c>
       <c r="I22" s="2" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
@@ -9067,6 +9082,7 @@
 MK-NW-F-128 heldValueOf
 MK-NW-F-129 gainRowName
 MK-NW-F-130 cannotWorkBackSentence
+MK-NW-F-131 pricedLikeBond
 MK-NW-O-001 theBonds
 MK-NW-O-003 theNetWorth
 MK-NW-O-004 theEmergencyFund
@@ -9474,6 +9490,7 @@
 MK-NW-F-124 maturityParts
 MK-NW-F-125 isPastMaturity
 MK-NW-F-126 yearlyInterestNow
+MK-NW-F-131 pricedLikeBond
 MK-NW-O-001 theBonds
 MK-NW-O-003 theNetWorth
 MK-NW-O-005 theAlternativesOutlook
@@ -10209,7 +10226,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>8 rows on the master · 21 places in the code print a dollar figure · 6 of them have no row · 11 rows not found on screen</t>
+          <t>8 rows on the master · 21 places in the code print a dollar figure · 6 of them have no row · 12 rows not found on screen</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -10419,7 +10436,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>2 rows on the master · 8 places in the code print a dollar figure · 3 of them have no row · 5 rows not found on screen</t>
+          <t>2 rows on the master · 8 places in the code print a dollar figure · 3 of them have no row · 6 rows not found on screen</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -11014,7 +11031,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>3 rows on the master · 6 places in the code print a dollar figure · 1 of them have no row · 1 rows not found on screen</t>
+          <t>3 rows on the master · 6 places in the code print a dollar figure · 1 of them have no row · 2 rows not found on screen</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -16015,22 +16032,22 @@
       </c>
       <c r="D158" s="2" t="inlineStr">
         <is>
-          <t>estimate | social security | $#</t>
+          <t>afternoon | ava | your &lt;name&gt;: $#</t>
         </is>
       </c>
       <c r="E158" s="2" t="inlineStr">
         <is>
-          <t>retiree</t>
+          <t>worker</t>
         </is>
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>visible</t>
+          <t>spoken, visible</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
-          <t>$4,795 | this month</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="H158" s="2" t="inlineStr">
@@ -16058,22 +16075,22 @@
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>morning | ava | your &lt;name&gt;: $#</t>
+          <t>estimate | social security | $#</t>
         </is>
       </c>
       <c r="E159" s="2" t="inlineStr">
         <is>
-          <t>worker</t>
+          <t>retiree</t>
         </is>
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>spoken, visible</t>
+          <t>visible</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>$4,795 | this month</t>
         </is>
       </c>
       <c r="H159" s="2" t="inlineStr">
@@ -22497,7 +22514,7 @@
       </c>
       <c r="B312" s="2" t="inlineStr">
         <is>
-          <t>/analytics · /jobsafety</t>
+          <t>/analytics · /jobsafety · /stress-test · /insights · /home</t>
         </is>
       </c>
       <c r="C312" s="2" t="inlineStr"/>
@@ -25812,7 +25829,7 @@
       </c>
       <c r="G411" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-XS-M-006 Income · In (received) · In (take-home)</t>
+          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-CF-M-020 THIS MONTH — free to use</t>
         </is>
       </c>
       <c r="H411" s="2" t="inlineStr">
@@ -25898,7 +25915,7 @@
       </c>
       <c r="G413" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-007 Left / Over · left to spend this month</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H413" s="2" t="inlineStr">
@@ -25941,7 +25958,7 @@
       </c>
       <c r="G414" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-007 Left / Over · left to spend this month</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H414" s="2" t="inlineStr">
@@ -25994,7 +26011,7 @@
       </c>
       <c r="I415" s="2" t="n"/>
     </row>
-    <row r="416" ht="45" customHeight="1">
+    <row r="416" ht="60" customHeight="1">
       <c r="A416" s="2" t="inlineStr">
         <is>
           <t>money figure — more than one row could be it</t>
@@ -26027,7 +26044,7 @@
       </c>
       <c r="G416" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-CF-M-001 Expenses, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-CF-M-001 Expenses, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H416" s="2" t="inlineStr">
@@ -26070,7 +26087,7 @@
       </c>
       <c r="G417" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H417" s="2" t="inlineStr">
@@ -26113,7 +26130,7 @@
       </c>
       <c r="G418" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-020 THIS MONTH — free to use, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-CF-M-020 THIS MONTH — free to use</t>
         </is>
       </c>
       <c r="H418" s="2" t="inlineStr">
@@ -27145,7 +27162,7 @@
       </c>
       <c r="G442" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
+          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
         </is>
       </c>
       <c r="H442" s="2" t="inlineStr">
@@ -27231,7 +27248,7 @@
       </c>
       <c r="G444" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
+          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
         </is>
       </c>
       <c r="H444" s="2" t="inlineStr">
@@ -27274,7 +27291,7 @@
       </c>
       <c r="G445" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
+          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
         </is>
       </c>
       <c r="H445" s="2" t="inlineStr">
@@ -27489,7 +27506,7 @@
       </c>
       <c r="G450" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
+          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
         </is>
       </c>
       <c r="H450" s="2" t="inlineStr">
@@ -27684,7 +27701,7 @@
       </c>
       <c r="C455" s="2" t="inlineStr">
         <is>
-          <t>src/screens/HomeScreen.tsx:503</t>
+          <t>src/screens/HomeScreen.tsx:505</t>
         </is>
       </c>
       <c r="D455" s="2" t="inlineStr">
@@ -27704,7 +27721,7 @@
       </c>
       <c r="G455" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H455" s="2" t="inlineStr">
@@ -27727,7 +27744,7 @@
       </c>
       <c r="C456" s="2" t="inlineStr">
         <is>
-          <t>src/screens/HomeScreen.tsx:516 (+1 spoken/visible twin)</t>
+          <t>src/screens/HomeScreen.tsx:518 (+1 spoken/visible twin)</t>
         </is>
       </c>
       <c r="D456" s="2" t="inlineStr">
@@ -27747,7 +27764,7 @@
       </c>
       <c r="G456" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H456" s="2" t="inlineStr">
@@ -27770,7 +27787,7 @@
       </c>
       <c r="C457" s="2" t="inlineStr">
         <is>
-          <t>src/screens/HomeScreen.tsx:517</t>
+          <t>src/screens/HomeScreen.tsx:519</t>
         </is>
       </c>
       <c r="D457" s="2" t="inlineStr">
@@ -27790,7 +27807,7 @@
       </c>
       <c r="G457" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-007 Left / Over · left to spend this month</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H457" s="2" t="inlineStr">
@@ -27962,7 +27979,7 @@
       </c>
       <c r="G461" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-014 Employer 401(k) match, MK-MN-M-013 Take-home / month</t>
+          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H461" s="2" t="inlineStr">
@@ -28134,7 +28151,7 @@
       </c>
       <c r="G465" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-007 Left / Over · left to spend this month</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H465" s="2" t="inlineStr">
@@ -28501,7 +28518,7 @@
       </c>
       <c r="C474" s="2" t="inlineStr">
         <is>
-          <t>src/screens/JobSafetyScreen.tsx:115</t>
+          <t>src/screens/JobSafetyScreen.tsx:117</t>
         </is>
       </c>
       <c r="D474" s="2" t="inlineStr">
@@ -28544,7 +28561,7 @@
       </c>
       <c r="C475" s="2" t="inlineStr">
         <is>
-          <t>src/screens/JobSafetyScreen.tsx:117</t>
+          <t>src/screens/JobSafetyScreen.tsx:119</t>
         </is>
       </c>
       <c r="D475" s="2" t="inlineStr">
@@ -28587,7 +28604,7 @@
       </c>
       <c r="C476" s="2" t="inlineStr">
         <is>
-          <t>src/screens/JobSafetyScreen.tsx:120</t>
+          <t>src/screens/JobSafetyScreen.tsx:132</t>
         </is>
       </c>
       <c r="D476" s="2" t="inlineStr">
@@ -28630,7 +28647,7 @@
       </c>
       <c r="C477" s="2" t="inlineStr">
         <is>
-          <t>src/screens/JobSafetyScreen.tsx:163</t>
+          <t>src/screens/JobSafetyScreen.tsx:175</t>
         </is>
       </c>
       <c r="D477" s="2" t="inlineStr">
@@ -28994,7 +29011,7 @@
       </c>
       <c r="G485" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H485" s="2" t="inlineStr">
@@ -29037,7 +29054,7 @@
       </c>
       <c r="G486" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H486" s="2" t="inlineStr">
@@ -29080,7 +29097,7 @@
       </c>
       <c r="G487" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H487" s="2" t="inlineStr">
@@ -29123,7 +29140,7 @@
       </c>
       <c r="G488" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed, MK-PL-M-005 + Draw from savings</t>
+          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H488" s="2" t="inlineStr">
@@ -30241,7 +30258,7 @@
       </c>
       <c r="G514" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H514" s="2" t="inlineStr">
@@ -30284,7 +30301,7 @@
       </c>
       <c r="G515" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H515" s="2" t="inlineStr">
@@ -30327,7 +30344,7 @@
       </c>
       <c r="G516" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H516" s="2" t="inlineStr">
@@ -30370,7 +30387,7 @@
       </c>
       <c r="G517" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N</t>
+          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month</t>
         </is>
       </c>
       <c r="H517" s="2" t="inlineStr">
@@ -30393,7 +30410,7 @@
       </c>
       <c r="C518" s="2" t="inlineStr">
         <is>
-          <t>src/screens/StressTestScreen.tsx:72 (+1 spoken/visible twin)</t>
+          <t>src/screens/StressTestScreen.tsx:74 (+1 spoken/visible twin)</t>
         </is>
       </c>
       <c r="D518" s="2" t="inlineStr">
@@ -30436,7 +30453,7 @@
       </c>
       <c r="C519" s="2" t="inlineStr">
         <is>
-          <t>src/screens/StressTestScreen.tsx:76</t>
+          <t>src/screens/StressTestScreen.tsx:78</t>
         </is>
       </c>
       <c r="D519" s="2" t="inlineStr">
@@ -30456,7 +30473,7 @@
       </c>
       <c r="G519" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-024 You could cover a $X hit, MK-MN-M-026 your $X/month of essentials</t>
+          <t>MK-MN-M-024 You could cover a $X hit, MK-MN-M-026 your $X/month of essentials, MK-MN-M-025 You'd have $X left — about N months of e</t>
         </is>
       </c>
       <c r="H519" s="2" t="inlineStr">
@@ -30479,7 +30496,7 @@
       </c>
       <c r="C520" s="2" t="inlineStr">
         <is>
-          <t>src/screens/StressTestScreen.tsx:93</t>
+          <t>src/screens/StressTestScreen.tsx:104</t>
         </is>
       </c>
       <c r="D520" s="2" t="inlineStr">
@@ -30499,7 +30516,7 @@
       </c>
       <c r="G520" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-024 You could cover a $X hit, MK-MN-M-026 your $X/month of essentials</t>
+          <t>MK-MN-M-024 You could cover a $X hit, MK-MN-M-026 your $X/month of essentials, MK-MN-M-025 You'd have $X left — about N months of e</t>
         </is>
       </c>
       <c r="H520" s="2" t="inlineStr">
@@ -30522,7 +30539,7 @@
       </c>
       <c r="C521" s="2" t="inlineStr">
         <is>
-          <t>src/screens/StressTestScreen.tsx:97</t>
+          <t>src/screens/StressTestScreen.tsx:108</t>
         </is>
       </c>
       <c r="D521" s="2" t="inlineStr">
@@ -30565,7 +30582,7 @@
       </c>
       <c r="C522" s="2" t="inlineStr">
         <is>
-          <t>src/screens/StressTestScreen.tsx:107</t>
+          <t>src/screens/StressTestScreen.tsx:118</t>
         </is>
       </c>
       <c r="D522" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Standards brought level with the decisions of 2026-10-09/10: how an account is classed and counted (sweep order, Treasury words, matured bonds, bank vs broker CD, worked-back beginning, Value not entered, rent not included, rent with words refused, itemising refuses a missing value), the month-end window rule, canon term 20; tracker row closed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
+++ b/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
@@ -25829,7 +25829,7 @@
       </c>
       <c r="G411" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-XS-M-006 Income · In (received) · In (take-home)</t>
         </is>
       </c>
       <c r="H411" s="2" t="inlineStr">
@@ -25915,7 +25915,7 @@
       </c>
       <c r="G413" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H413" s="2" t="inlineStr">
@@ -25958,7 +25958,7 @@
       </c>
       <c r="G414" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H414" s="2" t="inlineStr">
@@ -26011,7 +26011,7 @@
       </c>
       <c r="I415" s="2" t="n"/>
     </row>
-    <row r="416" ht="60" customHeight="1">
+    <row r="416" ht="45" customHeight="1">
       <c r="A416" s="2" t="inlineStr">
         <is>
           <t>money figure — more than one row could be it</t>
@@ -26044,7 +26044,7 @@
       </c>
       <c r="G416" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-CF-M-001 Expenses, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
+          <t>MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-CF-M-001 Expenses, MK-CF-M-020 THIS MONTH — free to use</t>
         </is>
       </c>
       <c r="H416" s="2" t="inlineStr">
@@ -26087,7 +26087,7 @@
       </c>
       <c r="G417" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
+          <t>MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-020 THIS MONTH — free to use</t>
         </is>
       </c>
       <c r="H417" s="2" t="inlineStr">
@@ -26130,7 +26130,7 @@
       </c>
       <c r="G418" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-020 THIS MONTH — free to use, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H418" s="2" t="inlineStr">
@@ -27162,7 +27162,7 @@
       </c>
       <c r="G442" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
+          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
         </is>
       </c>
       <c r="H442" s="2" t="inlineStr">
@@ -27248,7 +27248,7 @@
       </c>
       <c r="G444" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
+          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
         </is>
       </c>
       <c r="H444" s="2" t="inlineStr">
@@ -27291,7 +27291,7 @@
       </c>
       <c r="G445" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
+          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
         </is>
       </c>
       <c r="H445" s="2" t="inlineStr">
@@ -27506,7 +27506,7 @@
       </c>
       <c r="G450" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
+          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
         </is>
       </c>
       <c r="H450" s="2" t="inlineStr">
@@ -27721,7 +27721,7 @@
       </c>
       <c r="G455" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H455" s="2" t="inlineStr">
@@ -27764,7 +27764,7 @@
       </c>
       <c r="G456" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H456" s="2" t="inlineStr">
@@ -27807,7 +27807,7 @@
       </c>
       <c r="G457" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H457" s="2" t="inlineStr">
@@ -27850,7 +27850,7 @@
       </c>
       <c r="G458" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
+          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H458" s="2" t="inlineStr">
@@ -27893,7 +27893,7 @@
       </c>
       <c r="G459" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
+          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H459" s="2" t="inlineStr">
@@ -27936,7 +27936,7 @@
       </c>
       <c r="G460" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
+          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H460" s="2" t="inlineStr">
@@ -27979,7 +27979,7 @@
       </c>
       <c r="G461" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
+          <t>MK-MN-M-014 Employer 401(k) match, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-012 Gross / year</t>
         </is>
       </c>
       <c r="H461" s="2" t="inlineStr">
@@ -28151,7 +28151,7 @@
       </c>
       <c r="G465" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H465" s="2" t="inlineStr">
@@ -28968,7 +28968,7 @@
       </c>
       <c r="G484" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed</t>
         </is>
       </c>
       <c r="H484" s="2" t="inlineStr">
@@ -29011,7 +29011,7 @@
       </c>
       <c r="G485" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed</t>
         </is>
       </c>
       <c r="H485" s="2" t="inlineStr">
@@ -29097,7 +29097,7 @@
       </c>
       <c r="G487" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H487" s="2" t="inlineStr">
@@ -29140,7 +29140,7 @@
       </c>
       <c r="G488" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-004 = Guaranteed</t>
         </is>
       </c>
       <c r="H488" s="2" t="inlineStr">
@@ -30473,7 +30473,7 @@
       </c>
       <c r="G519" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-024 You could cover a $X hit, MK-MN-M-026 your $X/month of essentials, MK-MN-M-025 You'd have $X left — about N months of e</t>
+          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit, MK-MN-M-025 You'd have $X left — about N months of e</t>
         </is>
       </c>
       <c r="H519" s="2" t="inlineStr">
@@ -30516,7 +30516,7 @@
       </c>
       <c r="G520" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-024 You could cover a $X hit, MK-MN-M-026 your $X/month of essentials, MK-MN-M-025 You'd have $X left — about N months of e</t>
+          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit, MK-MN-M-025 You'd have $X left — about N months of e</t>
         </is>
       </c>
       <c r="H520" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Performance outside briefs rebuilt from today's code (v02, four batches, 45 functions): six removed money-weighted functions dropped, today's formulas, the time-weighted-return engine carded (MK-ST-F-080..082, allow-listed), instructions corrected to time-weighted; DEC-3768b governs id fixed (MK-PF-F-008)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
+++ b/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
@@ -559,7 +559,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>moneykeel_calc_master_calculation-master_v01.xlsx · census 2026-10-10</t>
+          <t>moneykeel_calc_master_calculation-master_v01.xlsx · census 2026-10-11</t>
         </is>
       </c>
       <c r="C9" s="2" t="n"/>
@@ -16032,22 +16032,22 @@
       </c>
       <c r="D158" s="2" t="inlineStr">
         <is>
-          <t>afternoon | ava | your &lt;name&gt;: $#</t>
+          <t>estimate | social security | $#</t>
         </is>
       </c>
       <c r="E158" s="2" t="inlineStr">
         <is>
-          <t>worker</t>
+          <t>retiree</t>
         </is>
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>spoken, visible</t>
+          <t>visible</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>$4,795 | this month</t>
         </is>
       </c>
       <c r="H158" s="2" t="inlineStr">
@@ -16075,22 +16075,22 @@
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>estimate | social security | $#</t>
+          <t>evening | ava | your &lt;name&gt;: $#</t>
         </is>
       </c>
       <c r="E159" s="2" t="inlineStr">
         <is>
-          <t>retiree</t>
+          <t>worker</t>
         </is>
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>visible</t>
+          <t>spoken, visible</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t>$4,795 | this month</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="H159" s="2" t="inlineStr">
@@ -25743,7 +25743,7 @@
       </c>
       <c r="G409" s="2" t="inlineStr">
         <is>
-          <t>MK-PF-M-014 Wealth generated, MK-PF-M-017 Return, MK-PF-M-006 WHAT EACH CATEGORY EARNED — RETURN</t>
+          <t>MK-PF-M-014 Wealth generated, MK-PF-M-006 WHAT EACH CATEGORY EARNED — RETURN, MK-PF-M-017 Return</t>
         </is>
       </c>
       <c r="H409" s="2" t="inlineStr">
@@ -25829,7 +25829,7 @@
       </c>
       <c r="G411" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-XS-M-006 Income · In (received) · In (take-home)</t>
+          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-020 THIS MONTH — free to use, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H411" s="2" t="inlineStr">
@@ -25915,7 +25915,7 @@
       </c>
       <c r="G413" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H413" s="2" t="inlineStr">
@@ -25958,7 +25958,7 @@
       </c>
       <c r="G414" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H414" s="2" t="inlineStr">
@@ -26087,7 +26087,7 @@
       </c>
       <c r="G417" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H417" s="2" t="inlineStr">
@@ -27162,7 +27162,7 @@
       </c>
       <c r="G442" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
+          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
         </is>
       </c>
       <c r="H442" s="2" t="inlineStr">
@@ -27248,7 +27248,7 @@
       </c>
       <c r="G444" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
+          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
         </is>
       </c>
       <c r="H444" s="2" t="inlineStr">
@@ -27291,7 +27291,7 @@
       </c>
       <c r="G445" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
+          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
         </is>
       </c>
       <c r="H445" s="2" t="inlineStr">
@@ -27506,7 +27506,7 @@
       </c>
       <c r="G450" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
+          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
         </is>
       </c>
       <c r="H450" s="2" t="inlineStr">
@@ -27807,7 +27807,7 @@
       </c>
       <c r="G457" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H457" s="2" t="inlineStr">
@@ -27850,7 +27850,7 @@
       </c>
       <c r="G458" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month</t>
+          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-012 Gross / year</t>
         </is>
       </c>
       <c r="H458" s="2" t="inlineStr">
@@ -27893,7 +27893,7 @@
       </c>
       <c r="G459" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month</t>
+          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-012 Gross / year</t>
         </is>
       </c>
       <c r="H459" s="2" t="inlineStr">
@@ -27936,7 +27936,7 @@
       </c>
       <c r="G460" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
+          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H460" s="2" t="inlineStr">
@@ -27979,7 +27979,7 @@
       </c>
       <c r="G461" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-014 Employer 401(k) match, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-012 Gross / year</t>
+          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-014 Employer 401(k) match</t>
         </is>
       </c>
       <c r="H461" s="2" t="inlineStr">
@@ -28151,7 +28151,7 @@
       </c>
       <c r="G465" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H465" s="2" t="inlineStr">
@@ -29011,7 +29011,7 @@
       </c>
       <c r="G485" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H485" s="2" t="inlineStr">
@@ -29054,7 +29054,7 @@
       </c>
       <c r="G486" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-005 + Draw from savings</t>
         </is>
       </c>
       <c r="H486" s="2" t="inlineStr">
@@ -29140,7 +29140,7 @@
       </c>
       <c r="G488" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-005 + Draw from savings</t>
         </is>
       </c>
       <c r="H488" s="2" t="inlineStr">
@@ -30258,7 +30258,7 @@
       </c>
       <c r="G514" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H514" s="2" t="inlineStr">
@@ -30301,7 +30301,7 @@
       </c>
       <c r="G515" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H515" s="2" t="inlineStr">
@@ -30344,7 +30344,7 @@
       </c>
       <c r="G516" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H516" s="2" t="inlineStr">
@@ -30387,7 +30387,7 @@
       </c>
       <c r="G517" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N</t>
         </is>
       </c>
       <c r="H517" s="2" t="inlineStr">
@@ -30473,7 +30473,7 @@
       </c>
       <c r="G519" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit, MK-MN-M-025 You'd have $X left — about N months of e</t>
+          <t>MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit</t>
         </is>
       </c>
       <c r="H519" s="2" t="inlineStr">
@@ -30516,7 +30516,7 @@
       </c>
       <c r="G520" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit, MK-MN-M-025 You'd have $X left — about N months of e</t>
+          <t>MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit</t>
         </is>
       </c>
       <c r="H520" s="2" t="inlineStr">

</xml_diff>

<commit_message>
OpenAI re-run brief for the whole Net worth module (v02: 119 functions, 90 decisions, the 61 changed since v01 named; builder --rerun-since) and the read-only audit of every function's inputs and use (workbook + summary + its scripts)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
+++ b/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
@@ -26219,7 +26219,7 @@
       </c>
       <c r="G414" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-020 THIS MONTH — free to use, MK-XS-M-006 Income · In (received) · In (take-home)</t>
+          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-XS-M-006 Income · In (received) · In (take-home)</t>
         </is>
       </c>
       <c r="H414" s="2" t="inlineStr">
@@ -26305,7 +26305,7 @@
       </c>
       <c r="G416" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H416" s="2" t="inlineStr">
@@ -26348,7 +26348,7 @@
       </c>
       <c r="G417" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H417" s="2" t="inlineStr">
@@ -26477,7 +26477,7 @@
       </c>
       <c r="G420" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H420" s="2" t="inlineStr">
@@ -27552,7 +27552,7 @@
       </c>
       <c r="G445" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
+          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
         </is>
       </c>
       <c r="H445" s="2" t="inlineStr">
@@ -27638,7 +27638,7 @@
       </c>
       <c r="G447" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
+          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
         </is>
       </c>
       <c r="H447" s="2" t="inlineStr">
@@ -27681,7 +27681,7 @@
       </c>
       <c r="G448" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
+          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
         </is>
       </c>
       <c r="H448" s="2" t="inlineStr">
@@ -27896,7 +27896,7 @@
       </c>
       <c r="G453" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
+          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
         </is>
       </c>
       <c r="H453" s="2" t="inlineStr">
@@ -28111,7 +28111,7 @@
       </c>
       <c r="G458" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H458" s="2" t="inlineStr">
@@ -28154,7 +28154,7 @@
       </c>
       <c r="G459" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H459" s="2" t="inlineStr">
@@ -28197,7 +28197,7 @@
       </c>
       <c r="G460" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H460" s="2" t="inlineStr">
@@ -28240,7 +28240,7 @@
       </c>
       <c r="G461" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month, MK-MN-M-012 Gross / year</t>
+          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H461" s="2" t="inlineStr">
@@ -28283,7 +28283,7 @@
       </c>
       <c r="G462" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month, MK-MN-M-012 Gross / year</t>
+          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H462" s="2" t="inlineStr">
@@ -28326,7 +28326,7 @@
       </c>
       <c r="G463" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
+          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H463" s="2" t="inlineStr">
@@ -28369,7 +28369,7 @@
       </c>
       <c r="G464" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-014 Employer 401(k) match, MK-MN-M-013 Take-home / month</t>
+          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H464" s="2" t="inlineStr">
@@ -28541,7 +28541,7 @@
       </c>
       <c r="G468" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H468" s="2" t="inlineStr">
@@ -29401,7 +29401,7 @@
       </c>
       <c r="G488" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H488" s="2" t="inlineStr">
@@ -29444,7 +29444,7 @@
       </c>
       <c r="G489" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-005 + Draw from savings</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H489" s="2" t="inlineStr">
@@ -29487,7 +29487,7 @@
       </c>
       <c r="G490" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H490" s="2" t="inlineStr">
@@ -29530,7 +29530,7 @@
       </c>
       <c r="G491" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-005 + Draw from savings</t>
+          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H491" s="2" t="inlineStr">

</xml_diff>

<commit_message>
His decision DEC-4439: in the time-weighted return, money that moves on a day counts for that whole day
Vanguard $50,000 + $10,000 that morning → $60,300: +0.50% (was +0.60%). A first deposit is measured on itself: $10,000 → $10,050 is +0.50%, → $9,800 is −2.00% (both were refused). The 'value below money added' refusal is gone; 'nothing to grow from' replaces the impossible cases. Moved tests marked with their arithmetic; Performance v17 note, standard, Changelog row, formulas in words. 5,077 tests green.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
+++ b/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
@@ -26133,7 +26133,7 @@
       </c>
       <c r="G412" s="2" t="inlineStr">
         <is>
-          <t>MK-PF-M-014 Wealth generated, MK-PF-M-006 WHAT EACH CATEGORY EARNED — RETURN, MK-PF-M-017 Return</t>
+          <t>MK-PF-M-014 Wealth generated, MK-PF-M-017 Return, MK-PF-M-006 WHAT EACH CATEGORY EARNED — RETURN</t>
         </is>
       </c>
       <c r="H412" s="2" t="inlineStr">
@@ -26219,7 +26219,7 @@
       </c>
       <c r="G414" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-XS-M-006 Income · In (received) · In (take-home)</t>
+          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-020 THIS MONTH — free to use, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H414" s="2" t="inlineStr">
@@ -26391,7 +26391,7 @@
       </c>
       <c r="G418" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-004 each row of the month — what it is and w, MK-CF-M-059 total interest</t>
+          <t>MK-CF-M-059 total interest, MK-CF-M-004 each row of the month — what it is and w</t>
         </is>
       </c>
       <c r="H418" s="2" t="inlineStr">
@@ -26477,7 +26477,7 @@
       </c>
       <c r="G420" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
+          <t>MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-020 THIS MONTH — free to use</t>
         </is>
       </c>
       <c r="H420" s="2" t="inlineStr">
@@ -28240,7 +28240,7 @@
       </c>
       <c r="G461" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
+          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month, MK-MN-M-012 Gross / year</t>
         </is>
       </c>
       <c r="H461" s="2" t="inlineStr">
@@ -28283,7 +28283,7 @@
       </c>
       <c r="G462" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
+          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month, MK-MN-M-012 Gross / year</t>
         </is>
       </c>
       <c r="H462" s="2" t="inlineStr">
@@ -28326,7 +28326,7 @@
       </c>
       <c r="G463" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
+          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H463" s="2" t="inlineStr">
@@ -28369,7 +28369,7 @@
       </c>
       <c r="G464" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
+          <t>MK-MN-M-014 Employer 401(k) match, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H464" s="2" t="inlineStr">
@@ -29358,7 +29358,7 @@
       </c>
       <c r="G487" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed</t>
         </is>
       </c>
       <c r="H487" s="2" t="inlineStr">
@@ -29401,7 +29401,7 @@
       </c>
       <c r="G488" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H488" s="2" t="inlineStr">
@@ -29444,7 +29444,7 @@
       </c>
       <c r="G489" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H489" s="2" t="inlineStr">
@@ -29487,7 +29487,7 @@
       </c>
       <c r="G490" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H490" s="2" t="inlineStr">
@@ -29530,7 +29530,7 @@
       </c>
       <c r="G491" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H491" s="2" t="inlineStr">
@@ -30648,7 +30648,7 @@
       </c>
       <c r="G517" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H517" s="2" t="inlineStr">
@@ -30691,7 +30691,7 @@
       </c>
       <c r="G518" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H518" s="2" t="inlineStr">
@@ -30734,7 +30734,7 @@
       </c>
       <c r="G519" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H519" s="2" t="inlineStr">
@@ -30777,7 +30777,7 @@
       </c>
       <c r="G520" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N</t>
+          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month</t>
         </is>
       </c>
       <c r="H520" s="2" t="inlineStr">
@@ -30863,7 +30863,7 @@
       </c>
       <c r="G522" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-024 You could cover a $X hit, MK-MN-M-026 your $X/month of essentials, MK-MN-M-025 You'd have $X left — about N months of e</t>
+          <t>MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit</t>
         </is>
       </c>
       <c r="H522" s="2" t="inlineStr">
@@ -30906,7 +30906,7 @@
       </c>
       <c r="G523" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-024 You could cover a $X hit, MK-MN-M-026 your $X/month of essentials, MK-MN-M-025 You'd have $X left — about N months of e</t>
+          <t>MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit</t>
         </is>
       </c>
       <c r="H523" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Net worth drawing check v02 (against c40588f3): five more fixes — an unpriced holding stays out of the change line (+0.53%), DEBTS shows $0 once an account exists, the minus sign everywhere, holding with no price paid, the market over the same days as a short price history; READ THIS FIRST rows for DEC-4439, DEC-4036c, DEC-4350. All 1,204 Net worth cases re-run.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
+++ b/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
@@ -559,7 +559,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>moneykeel_calc_master_calculation-master_v01.xlsx · census 2026-10-11</t>
+          <t>moneykeel_calc_master_calculation-master_v01.xlsx · census 2026-10-12</t>
         </is>
       </c>
       <c r="C9" s="2" t="n"/>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>9205</v>
+        <v>9207</v>
       </c>
       <c r="C16" s="2" t="n"/>
     </row>
@@ -14749,7 +14749,7 @@
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>−$# | -$#</t>
+          <t>−$# | −$#</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
@@ -16336,7 +16336,7 @@
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>morning | ava | your &lt;name&gt;: $#</t>
+          <t>evening | ava | your &lt;name&gt;: $#</t>
         </is>
       </c>
       <c r="E159" s="2" t="inlineStr">
@@ -26123,7 +26123,7 @@
       </c>
       <c r="E412" s="2" t="inlineStr">
         <is>
-          <t>$420, $600, $151,000, $165,000 … (1257 renders)</t>
+          <t>$420, $600, $151,000, $165,000 … (1260 renders)</t>
         </is>
       </c>
       <c r="F412" s="2" t="inlineStr">
@@ -26133,7 +26133,7 @@
       </c>
       <c r="G412" s="2" t="inlineStr">
         <is>
-          <t>MK-PF-M-014 Wealth generated, MK-PF-M-017 Return, MK-PF-M-006 WHAT EACH CATEGORY EARNED — RETURN</t>
+          <t>MK-PF-M-014 Wealth generated, MK-PF-M-006 WHAT EACH CATEGORY EARNED — RETURN, MK-PF-M-017 Return</t>
         </is>
       </c>
       <c r="H412" s="2" t="inlineStr">
@@ -26219,7 +26219,7 @@
       </c>
       <c r="G414" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-020 THIS MONTH — free to use, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
+          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-XS-M-006 Income · In (received) · In (take-home)</t>
         </is>
       </c>
       <c r="H414" s="2" t="inlineStr">
@@ -26305,7 +26305,7 @@
       </c>
       <c r="G416" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H416" s="2" t="inlineStr">
@@ -26348,7 +26348,7 @@
       </c>
       <c r="G417" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H417" s="2" t="inlineStr">
@@ -26391,7 +26391,7 @@
       </c>
       <c r="G418" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-059 total interest, MK-CF-M-004 each row of the month — what it is and w</t>
+          <t>MK-CF-M-004 each row of the month — what it is and w, MK-CF-M-059 total interest</t>
         </is>
       </c>
       <c r="H418" s="2" t="inlineStr">
@@ -26520,7 +26520,7 @@
       </c>
       <c r="G421" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-020 THIS MONTH — free to use, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-CF-M-020 THIS MONTH — free to use</t>
         </is>
       </c>
       <c r="H421" s="2" t="inlineStr">
@@ -28197,7 +28197,7 @@
       </c>
       <c r="G460" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H460" s="2" t="inlineStr">
@@ -28240,7 +28240,7 @@
       </c>
       <c r="G461" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month, MK-MN-M-012 Gross / year</t>
+          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H461" s="2" t="inlineStr">
@@ -28283,7 +28283,7 @@
       </c>
       <c r="G462" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month, MK-MN-M-012 Gross / year</t>
+          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H462" s="2" t="inlineStr">
@@ -28326,7 +28326,7 @@
       </c>
       <c r="G463" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
+          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H463" s="2" t="inlineStr">
@@ -28369,7 +28369,7 @@
       </c>
       <c r="G464" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-014 Employer 401(k) match, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
+          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-014 Employer 401(k) match</t>
         </is>
       </c>
       <c r="H464" s="2" t="inlineStr">
@@ -28541,7 +28541,7 @@
       </c>
       <c r="G468" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H468" s="2" t="inlineStr">
@@ -29358,7 +29358,7 @@
       </c>
       <c r="G487" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H487" s="2" t="inlineStr">
@@ -29401,7 +29401,7 @@
       </c>
       <c r="G488" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H488" s="2" t="inlineStr">
@@ -29444,7 +29444,7 @@
       </c>
       <c r="G489" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H489" s="2" t="inlineStr">
@@ -29487,7 +29487,7 @@
       </c>
       <c r="G490" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H490" s="2" t="inlineStr">
@@ -29530,7 +29530,7 @@
       </c>
       <c r="G491" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed, MK-PL-M-005 + Draw from savings</t>
         </is>
       </c>
       <c r="H491" s="2" t="inlineStr">
@@ -30863,7 +30863,7 @@
       </c>
       <c r="G522" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit</t>
+          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit, MK-MN-M-025 You'd have $X left — about N months of e</t>
         </is>
       </c>
       <c r="H522" s="2" t="inlineStr">
@@ -30906,7 +30906,7 @@
       </c>
       <c r="G523" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit</t>
+          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit, MK-MN-M-025 You'd have $X left — about N months of e</t>
         </is>
       </c>
       <c r="H523" s="2" t="inlineStr">

</xml_diff>

<commit_message>
His decisions DEC-4528 ('Add your debts ›' on every empty Debts door) and DEC-4529 (drawing errors corrected by a dated line on the drawing, with the arithmetic; a home's edit sheet no longer asks what it is invested in); the OpenAI re-run brief for Net worth rebuilt from this final code (v02: 119 functions, 93 decisions, 61 changed named)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
+++ b/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
@@ -16336,7 +16336,7 @@
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>evening | ava | your &lt;name&gt;: $#</t>
+          <t>morning | ava | your &lt;name&gt;: $#</t>
         </is>
       </c>
       <c r="E159" s="2" t="inlineStr">
@@ -26113,7 +26113,7 @@
       </c>
       <c r="C412" s="2" t="inlineStr">
         <is>
-          <t>MoneyKeel/functions/_figure-spec.ts:72</t>
+          <t>MoneyKeel/functions/_figure-spec.ts:74</t>
         </is>
       </c>
       <c r="D412" s="2" t="inlineStr">
@@ -26156,7 +26156,7 @@
       </c>
       <c r="C413" s="2" t="inlineStr">
         <is>
-          <t>MoneyKeel/functions/_figure-spec.ts:74</t>
+          <t>MoneyKeel/functions/_figure-spec.ts:76</t>
         </is>
       </c>
       <c r="D413" s="2" t="inlineStr">
@@ -26219,7 +26219,7 @@
       </c>
       <c r="G414" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-XS-M-006 Income · In (received) · In (take-home)</t>
+          <t>MK-CF-M-034 Your 401(k)s, MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H414" s="2" t="inlineStr">
@@ -26305,7 +26305,7 @@
       </c>
       <c r="G416" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H416" s="2" t="inlineStr">
@@ -26348,7 +26348,7 @@
       </c>
       <c r="G417" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H417" s="2" t="inlineStr">
@@ -26391,7 +26391,7 @@
       </c>
       <c r="G418" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-004 each row of the month — what it is and w, MK-CF-M-059 total interest</t>
+          <t>MK-CF-M-059 total interest, MK-CF-M-004 each row of the month — what it is and w</t>
         </is>
       </c>
       <c r="H418" s="2" t="inlineStr">
@@ -26401,7 +26401,7 @@
       </c>
       <c r="I418" s="2" t="n"/>
     </row>
-    <row r="419" ht="45" customHeight="1">
+    <row r="419" ht="60" customHeight="1">
       <c r="A419" s="2" t="inlineStr">
         <is>
           <t>money figure — more than one row could be it</t>
@@ -26434,7 +26434,7 @@
       </c>
       <c r="G419" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-CF-M-001 Expenses, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-CF-M-001 Expenses, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H419" s="2" t="inlineStr">
@@ -26477,7 +26477,7 @@
       </c>
       <c r="G420" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H420" s="2" t="inlineStr">
@@ -28111,7 +28111,7 @@
       </c>
       <c r="G458" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H458" s="2" t="inlineStr">
@@ -28154,7 +28154,7 @@
       </c>
       <c r="G459" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H459" s="2" t="inlineStr">
@@ -28197,7 +28197,7 @@
       </c>
       <c r="G460" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H460" s="2" t="inlineStr">
@@ -28240,7 +28240,7 @@
       </c>
       <c r="G461" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
+          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H461" s="2" t="inlineStr">
@@ -28283,7 +28283,7 @@
       </c>
       <c r="G462" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
+          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H462" s="2" t="inlineStr">
@@ -28326,7 +28326,7 @@
       </c>
       <c r="G463" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
+          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H463" s="2" t="inlineStr">
@@ -28369,7 +28369,7 @@
       </c>
       <c r="G464" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-014 Employer 401(k) match</t>
+          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H464" s="2" t="inlineStr">
@@ -28541,7 +28541,7 @@
       </c>
       <c r="G468" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H468" s="2" t="inlineStr">
@@ -29358,7 +29358,7 @@
       </c>
       <c r="G487" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed</t>
         </is>
       </c>
       <c r="H487" s="2" t="inlineStr">
@@ -29401,7 +29401,7 @@
       </c>
       <c r="G488" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed, MK-PL-M-005 + Draw from savings</t>
         </is>
       </c>
       <c r="H488" s="2" t="inlineStr">
@@ -29444,7 +29444,7 @@
       </c>
       <c r="G489" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-005 + Draw from savings</t>
         </is>
       </c>
       <c r="H489" s="2" t="inlineStr">
@@ -29487,7 +29487,7 @@
       </c>
       <c r="G490" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed</t>
         </is>
       </c>
       <c r="H490" s="2" t="inlineStr">
@@ -30648,7 +30648,7 @@
       </c>
       <c r="G517" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H517" s="2" t="inlineStr">
@@ -30691,7 +30691,7 @@
       </c>
       <c r="G518" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H518" s="2" t="inlineStr">
@@ -30734,7 +30734,7 @@
       </c>
       <c r="G519" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H519" s="2" t="inlineStr">
@@ -30777,7 +30777,7 @@
       </c>
       <c r="G520" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N</t>
         </is>
       </c>
       <c r="H520" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Performance: an entered 0% rate counts as 0%, an empty box stays unknown (DEC-2748b) — 6 of 6 places
MK-NW-F-127 gainOfRow, MK-NW-O-008 thePerformance, MK-NW-F-084 categoryEarnings,
account page rate, Add account form, Bonds edit/sell form.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
+++ b/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
@@ -26219,7 +26219,7 @@
       </c>
       <c r="G414" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-020 THIS MONTH — free to use, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
+          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-XS-M-006 Income · In (received) · In (take-home)</t>
         </is>
       </c>
       <c r="H414" s="2" t="inlineStr">
@@ -26305,7 +26305,7 @@
       </c>
       <c r="G416" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-XS-M-007 Left / Over · left to spend this month</t>
         </is>
       </c>
       <c r="H416" s="2" t="inlineStr">
@@ -26348,7 +26348,7 @@
       </c>
       <c r="G417" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-XS-M-007 Left / Over · left to spend this month</t>
         </is>
       </c>
       <c r="H417" s="2" t="inlineStr">
@@ -26401,7 +26401,7 @@
       </c>
       <c r="I418" s="2" t="n"/>
     </row>
-    <row r="419" ht="45" customHeight="1">
+    <row r="419" ht="60" customHeight="1">
       <c r="A419" s="2" t="inlineStr">
         <is>
           <t>money figure — more than one row could be it</t>
@@ -26434,7 +26434,7 @@
       </c>
       <c r="G419" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-CF-M-001 Expenses, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-CF-M-001 Expenses, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H419" s="2" t="inlineStr">
@@ -26477,7 +26477,7 @@
       </c>
       <c r="G420" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H420" s="2" t="inlineStr">
@@ -26520,7 +26520,7 @@
       </c>
       <c r="G421" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-020 THIS MONTH — free to use, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-CF-M-020 THIS MONTH — free to use</t>
         </is>
       </c>
       <c r="H421" s="2" t="inlineStr">
@@ -28197,7 +28197,7 @@
       </c>
       <c r="G460" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-XS-M-007 Left / Over · left to spend this month</t>
         </is>
       </c>
       <c r="H460" s="2" t="inlineStr">
@@ -28240,7 +28240,7 @@
       </c>
       <c r="G461" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
+          <t>MK-MN-M-013 Take-home / month, MK-MN-M-012 Gross / year, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H461" s="2" t="inlineStr">
@@ -28283,7 +28283,7 @@
       </c>
       <c r="G462" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
+          <t>MK-MN-M-013 Take-home / month, MK-MN-M-012 Gross / year, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H462" s="2" t="inlineStr">
@@ -28326,7 +28326,7 @@
       </c>
       <c r="G463" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
+          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H463" s="2" t="inlineStr">
@@ -28369,7 +28369,7 @@
       </c>
       <c r="G464" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
+          <t>MK-MN-M-013 Take-home / month, MK-MN-M-012 Gross / year, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H464" s="2" t="inlineStr">
@@ -28541,7 +28541,7 @@
       </c>
       <c r="G468" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-XS-M-007 Left / Over · left to spend this month</t>
         </is>
       </c>
       <c r="H468" s="2" t="inlineStr">
@@ -29358,7 +29358,7 @@
       </c>
       <c r="G487" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H487" s="2" t="inlineStr">
@@ -29401,7 +29401,7 @@
       </c>
       <c r="G488" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-005 + Draw from savings</t>
         </is>
       </c>
       <c r="H488" s="2" t="inlineStr">
@@ -29444,7 +29444,7 @@
       </c>
       <c r="G489" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-005 + Draw from savings</t>
         </is>
       </c>
       <c r="H489" s="2" t="inlineStr">
@@ -29487,7 +29487,7 @@
       </c>
       <c r="G490" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H490" s="2" t="inlineStr">
@@ -29530,7 +29530,7 @@
       </c>
       <c r="G491" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H491" s="2" t="inlineStr">
@@ -30648,7 +30648,7 @@
       </c>
       <c r="G517" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H517" s="2" t="inlineStr">
@@ -30691,7 +30691,7 @@
       </c>
       <c r="G518" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H518" s="2" t="inlineStr">
@@ -30734,7 +30734,7 @@
       </c>
       <c r="G519" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H519" s="2" t="inlineStr">
@@ -30777,7 +30777,7 @@
       </c>
       <c r="G520" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N</t>
+          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month</t>
         </is>
       </c>
       <c r="H520" s="2" t="inlineStr">
@@ -30863,7 +30863,7 @@
       </c>
       <c r="G522" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-024 You could cover a $X hit</t>
+          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit, MK-MN-M-025 You'd have $X left — about N months of e</t>
         </is>
       </c>
       <c r="H522" s="2" t="inlineStr">
@@ -30906,7 +30906,7 @@
       </c>
       <c r="G523" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-024 You could cover a $X hit</t>
+          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit, MK-MN-M-025 You'd have $X left — about N months of e</t>
         </is>
       </c>
       <c r="H523" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Performance: re-run all 203 outside cases — settle the last open ones
- a written (short) option keeps its sign and unit: '-1 contract' (DEC-0277), was refused
- latest close and close-on-or-before read the latest DATE in any order; every price list is put oldest first where it enters (fetchPriceSeries)
- the worked-back beginning case relabelled SETTLED by DEC-4644; stale open-point note on totalROI removed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
+++ b/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>9207</v>
+        <v>9219</v>
       </c>
       <c r="C16" s="2" t="n"/>
     </row>
@@ -17891,7 +17891,7 @@
       </c>
       <c r="D195" s="2" t="inlineStr">
         <is>
-          <t>🔗 | linked · # days old</t>
+          <t>› | 🔗 | linked · # days old</t>
         </is>
       </c>
       <c r="E195" s="2" t="inlineStr">
@@ -17906,7 +17906,7 @@
       </c>
       <c r="G195" s="2" t="inlineStr">
         <is>
-          <t>Vanguard Brokerage | $300,000</t>
+          <t>$300,000 | Open Vanguard Brokerage — this account's own page</t>
         </is>
       </c>
       <c r="H195" s="2" t="inlineStr">
@@ -26142,7 +26142,7 @@
       </c>
       <c r="G412" s="2" t="inlineStr">
         <is>
-          <t>MK-PF-M-014 Wealth generated, MK-PF-M-006 WHAT EACH CATEGORY EARNED — RETURN, MK-PF-M-017 Return</t>
+          <t>MK-PF-M-014 Wealth generated, MK-PF-M-017 Return, MK-PF-M-006 WHAT EACH CATEGORY EARNED — RETURN</t>
         </is>
       </c>
       <c r="H412" s="2" t="inlineStr">
@@ -26228,7 +26228,7 @@
       </c>
       <c r="G414" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-XS-M-006 Income · In (received) · In (take-home)</t>
+          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-CF-M-020 THIS MONTH — free to use</t>
         </is>
       </c>
       <c r="H414" s="2" t="inlineStr">
@@ -26400,7 +26400,7 @@
       </c>
       <c r="G418" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-004 each row of the month — what it is and w, MK-CF-M-059 total interest</t>
+          <t>MK-CF-M-059 total interest, MK-CF-M-004 each row of the month — what it is and w</t>
         </is>
       </c>
       <c r="H418" s="2" t="inlineStr">
@@ -26486,7 +26486,7 @@
       </c>
       <c r="G420" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
+          <t>MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H420" s="2" t="inlineStr">
@@ -27561,7 +27561,7 @@
       </c>
       <c r="G445" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
+          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
         </is>
       </c>
       <c r="H445" s="2" t="inlineStr">
@@ -27647,7 +27647,7 @@
       </c>
       <c r="G447" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
+          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
         </is>
       </c>
       <c r="H447" s="2" t="inlineStr">
@@ -27690,7 +27690,7 @@
       </c>
       <c r="G448" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
+          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
         </is>
       </c>
       <c r="H448" s="2" t="inlineStr">
@@ -27905,7 +27905,7 @@
       </c>
       <c r="G453" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
+          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
         </is>
       </c>
       <c r="H453" s="2" t="inlineStr">
@@ -28249,7 +28249,7 @@
       </c>
       <c r="G461" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month, MK-MN-M-012 Gross / year</t>
+          <t>MK-MN-M-012 Gross / year, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H461" s="2" t="inlineStr">
@@ -28292,7 +28292,7 @@
       </c>
       <c r="G462" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month, MK-MN-M-012 Gross / year</t>
+          <t>MK-MN-M-012 Gross / year, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H462" s="2" t="inlineStr">
@@ -28378,7 +28378,7 @@
       </c>
       <c r="G464" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month, MK-MN-M-014 Employer 401(k) match</t>
+          <t>MK-MN-M-014 Employer 401(k) match, MK-MN-M-012 Gross / year, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H464" s="2" t="inlineStr">
@@ -29367,7 +29367,7 @@
       </c>
       <c r="G487" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H487" s="2" t="inlineStr">
@@ -29410,7 +29410,7 @@
       </c>
       <c r="G488" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H488" s="2" t="inlineStr">
@@ -29453,7 +29453,7 @@
       </c>
       <c r="G489" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-005 + Draw from savings</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H489" s="2" t="inlineStr">
@@ -29496,7 +29496,7 @@
       </c>
       <c r="G490" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H490" s="2" t="inlineStr">
@@ -29539,7 +29539,7 @@
       </c>
       <c r="G491" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed</t>
         </is>
       </c>
       <c r="H491" s="2" t="inlineStr">
@@ -30657,7 +30657,7 @@
       </c>
       <c r="G517" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H517" s="2" t="inlineStr">
@@ -30700,7 +30700,7 @@
       </c>
       <c r="G518" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H518" s="2" t="inlineStr">
@@ -30743,7 +30743,7 @@
       </c>
       <c r="G519" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H519" s="2" t="inlineStr">
@@ -30786,7 +30786,7 @@
       </c>
       <c r="G520" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N</t>
         </is>
       </c>
       <c r="H520" s="2" t="inlineStr">
@@ -30872,7 +30872,7 @@
       </c>
       <c r="G522" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-024 You could cover a $X hit</t>
+          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit, MK-MN-M-025 You'd have $X left — about N months of e</t>
         </is>
       </c>
       <c r="H522" s="2" t="inlineStr">
@@ -30915,7 +30915,7 @@
       </c>
       <c r="G523" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-024 You could cover a $X hit</t>
+          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit, MK-MN-M-025 You'd have $X left — about N months of e</t>
         </is>
       </c>
       <c r="H523" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Net worth re-run: fixes DEC-4913 property use (A second home, both count toward retirement), Treasury Wine Estates / Apple Corp 4.5% Bond / UST classing, blank benchmark period, wording of MK-NW-F-015/039/045; Gemini 01-02 and OpenAI 01-03 re-run cases recorded
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
+++ b/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
@@ -1131,7 +1131,6 @@
 MK-NW-F-009 maturityClass
 MK-NW-F-011 assetClassOf
 MK-NW-F-014 isRealAsset
-MK-NW-F-015 totalAssets
 MK-NW-F-016 cashTotal
 MK-NW-F-021 investmentsTotal
 MK-NW-F-022 investableAssets
@@ -1239,7 +1238,7 @@
         </is>
       </c>
       <c r="I2" s="2" t="n">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
@@ -1445,7 +1444,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-I-001 account balance — read by MK-CF-F-111, MK-CF-F-133, MK-CF-F-134, MK-CF-F-136, MK-NW-F-015, MK-NW-F-016, MK
+          <t>MK-XS-I-001 account balance — read by MK-CF-F-111, MK-CF-F-133, MK-CF-F-134, MK-CF-F-136, MK-NW-F-016, MK-NW-F-027, MK
 MK-XS-I-001 account balance — read by MK-NW-F-056, MK-NW-F-078, MK-NW-O-001, MK-ST-F-027
 MK-XS-I-002 account type (taxable, pre-tax, Roth) — read by MK-CF-F-134, MK-CF-F-136, MK-NW-F-011, MK-NW-F-027, MK-NW-F-040, MK-NW-F-054, MK
 MK-XS-I-002 account type (taxable, pre-tax, Roth) — read by MK-NW-F-011, MK-NW-F-120, MK-NW-O-001
@@ -2804,7 +2803,6 @@
 MK-NW-F-010 wrapperAccount
 MK-NW-F-012 taxTreatmentOf
 MK-NW-F-014 isRealAsset
-MK-NW-F-015 totalAssets
 MK-NW-F-021 investmentsTotal
 MK-NW-F-022 investableAssets
 MK-NW-F-023 wrapperWord
@@ -3351,7 +3349,6 @@
 MK-NW-F-004 portfolioActualReturn
 MK-NW-F-005 accountAllowsTicker
 MK-NW-F-014 isRealAsset
-MK-NW-F-015 totalAssets
 MK-NW-F-016 cashTotal
 MK-NW-F-021 investmentsTotal
 MK-NW-F-022 investableAssets
@@ -3910,7 +3907,6 @@
 MK-NW-F-011 assetClassOf
 MK-NW-F-012 taxTreatmentOf
 MK-NW-F-014 isRealAsset
-MK-NW-F-015 totalAssets
 MK-NW-F-016 cashTotal
 MK-NW-F-021 investmentsTotal
 MK-NW-F-022 investableAssets
@@ -4057,7 +4053,7 @@
         </is>
       </c>
       <c r="I9" s="2" t="n">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
@@ -4248,7 +4244,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MK-XS-I-001 account balance — read by MK-CF-F-111, MK-CF-F-133, MK-CF-F-134, MK-CF-F-136, MK-NW-F-015, MK-NW-F-016, MK
+          <t xml:space="preserve">MK-XS-I-001 account balance — read by MK-CF-F-111, MK-CF-F-133, MK-CF-F-134, MK-CF-F-136, MK-NW-F-016, MK-NW-F-027, MK
 MK-XS-I-001 account balance — read by MK-NW-F-031, MK-NW-F-032, MK-NW-F-133, MK-PL-F-026, MK-ST-F-027
 MK-XS-I-001 account balance — read by MK-NW-F-031, MK-NW-F-032, MK-NW-F-133, MK-ST-F-027
 MK-XS-I-002 account type (taxable, pre-tax, Roth) — read by MK-CF-F-134, MK-CF-F-136, MK-NW-F-011, MK-NW-F-027, MK-NW-F-040, MK-NW-F-054, MK
@@ -6376,20 +6372,11 @@
 MK-NW-F-009 maturityClass
 MK-NW-F-011 assetClassOf
 MK-NW-F-014 isRealAsset
-MK-NW-F-015 totalAssets
 MK-NW-F-022 investableAssets
 MK-NW-F-023 wrapperWord
-MK-NW-F-027 accountClassBreakdown
-MK-NW-F-053 correctClassOf
-MK-NW-F-054 reclassifyAccounts
 MK-NW-F-066 sumWhere
-MK-NW-F-067 plural
 MK-NW-F-068 prettyDay
-MK-NW-F-109 holdingClassOf
 MK-NW-F-120 classEvidenceOf
-MK-NW-F-121 holdingTagClass
-MK-NW-F-122 holdingTagFor
-MK-NW-F-123 holdingNameEvidence
 MK-PL-F-034 lifeInsuranceNeed
 MK-ST-F-010 nameEvidence
 MK-ST-F-027 accountId
@@ -6743,7 +6730,6 @@
 MK-NW-F-007 assetKind
 MK-NW-F-012 taxTreatmentOf
 MK-NW-F-014 isRealAsset
-MK-NW-F-015 totalAssets
 MK-NW-F-016 cashTotal
 MK-NW-F-021 investmentsTotal
 MK-NW-F-022 investableAssets
@@ -7372,7 +7358,6 @@
 MK-NW-F-007 assetKind
 MK-NW-F-012 taxTreatmentOf
 MK-NW-F-014 isRealAsset
-MK-NW-F-015 totalAssets
 MK-NW-F-016 cashTotal
 MK-NW-F-021 investmentsTotal
 MK-NW-F-022 investableAssets
@@ -8352,7 +8337,6 @@
 MK-NW-F-011 assetClassOf
 MK-NW-F-012 taxTreatmentOf
 MK-NW-F-014 isRealAsset
-MK-NW-F-015 totalAssets
 MK-NW-F-016 cashTotal
 MK-NW-F-021 investmentsTotal
 MK-NW-F-022 investableAssets
@@ -9264,7 +9248,6 @@
 MK-NW-F-011 assetClassOf
 MK-NW-F-012 taxTreatmentOf
 MK-NW-F-014 isRealAsset
-MK-NW-F-015 totalAssets
 MK-NW-F-016 cashTotal
 MK-NW-F-021 investmentsTotal
 MK-NW-F-022 investableAssets
@@ -9704,7 +9687,6 @@
 MK-NW-F-009 maturityClass
 MK-NW-F-011 assetClassOf
 MK-NW-F-014 isRealAsset
-MK-NW-F-015 totalAssets
 MK-NW-F-016 cashTotal
 MK-NW-F-021 investmentsTotal
 MK-NW-F-022 investableAssets
@@ -16345,7 +16327,7 @@
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>evening | ava | your &lt;name&gt;: $#</t>
+          <t>morning | ava | your &lt;name&gt;: $#</t>
         </is>
       </c>
       <c r="E159" s="2" t="inlineStr">
@@ -26142,7 +26124,7 @@
       </c>
       <c r="G412" s="2" t="inlineStr">
         <is>
-          <t>MK-PF-M-014 Wealth generated, MK-PF-M-017 Return, MK-PF-M-006 WHAT EACH CATEGORY EARNED — RETURN</t>
+          <t>MK-PF-M-014 Wealth generated, MK-PF-M-006 WHAT EACH CATEGORY EARNED — RETURN, MK-PF-M-017 Return</t>
         </is>
       </c>
       <c r="H412" s="2" t="inlineStr">
@@ -26314,7 +26296,7 @@
       </c>
       <c r="G416" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-007 Left / Over · left to spend this month</t>
         </is>
       </c>
       <c r="H416" s="2" t="inlineStr">
@@ -26357,7 +26339,7 @@
       </c>
       <c r="G417" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-007 Left / Over · left to spend this month</t>
         </is>
       </c>
       <c r="H417" s="2" t="inlineStr">
@@ -26400,7 +26382,7 @@
       </c>
       <c r="G418" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-059 total interest, MK-CF-M-004 each row of the month — what it is and w</t>
+          <t>MK-CF-M-004 each row of the month — what it is and w, MK-CF-M-059 total interest</t>
         </is>
       </c>
       <c r="H418" s="2" t="inlineStr">
@@ -26410,7 +26392,7 @@
       </c>
       <c r="I418" s="2" t="n"/>
     </row>
-    <row r="419" ht="60" customHeight="1">
+    <row r="419" ht="45" customHeight="1">
       <c r="A419" s="2" t="inlineStr">
         <is>
           <t>money figure — more than one row could be it</t>
@@ -26443,7 +26425,7 @@
       </c>
       <c r="G419" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-CF-M-001 Expenses, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
+          <t>MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-CF-M-001 Expenses, MK-CF-M-020 THIS MONTH — free to use</t>
         </is>
       </c>
       <c r="H419" s="2" t="inlineStr">
@@ -26486,7 +26468,7 @@
       </c>
       <c r="G420" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
+          <t>MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-020 THIS MONTH — free to use</t>
         </is>
       </c>
       <c r="H420" s="2" t="inlineStr">
@@ -26529,7 +26511,7 @@
       </c>
       <c r="G421" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-020 THIS MONTH — free to use, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H421" s="2" t="inlineStr">
@@ -28206,7 +28188,7 @@
       </c>
       <c r="G460" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-007 Left / Over · left to spend this month</t>
         </is>
       </c>
       <c r="H460" s="2" t="inlineStr">
@@ -28249,7 +28231,7 @@
       </c>
       <c r="G461" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
+          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H461" s="2" t="inlineStr">
@@ -28292,7 +28274,7 @@
       </c>
       <c r="G462" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
+          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H462" s="2" t="inlineStr">
@@ -28335,7 +28317,7 @@
       </c>
       <c r="G463" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
+          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H463" s="2" t="inlineStr">
@@ -28378,7 +28360,7 @@
       </c>
       <c r="G464" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-014 Employer 401(k) match, MK-MN-M-012 Gross / year, MK-MN-M-011 TAKE-HOME / YEAR</t>
+          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-014 Employer 401(k) match</t>
         </is>
       </c>
       <c r="H464" s="2" t="inlineStr">
@@ -28550,7 +28532,7 @@
       </c>
       <c r="G468" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-007 Left / Over · left to spend this month</t>
         </is>
       </c>
       <c r="H468" s="2" t="inlineStr">
@@ -29410,7 +29392,7 @@
       </c>
       <c r="G488" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H488" s="2" t="inlineStr">
@@ -29453,7 +29435,7 @@
       </c>
       <c r="G489" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H489" s="2" t="inlineStr">
@@ -29496,7 +29478,7 @@
       </c>
       <c r="G490" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-004 = Guaranteed</t>
         </is>
       </c>
       <c r="H490" s="2" t="inlineStr">
@@ -29539,7 +29521,7 @@
       </c>
       <c r="G491" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-004 = Guaranteed</t>
         </is>
       </c>
       <c r="H491" s="2" t="inlineStr">
@@ -30083,7 +30065,7 @@
       </c>
       <c r="D504" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">: &lt;Text style={styles.instSrc} numberOfLines={2}&gt;{assetKind(a.kind)?.label} · {moneyCompact(earmarkedAmount(a, carId, homeId), 'M')}{simple ? '' : ` · ${info.source} · ${info.period}${info.estimate ? </t>
+          <t>: &lt;Text style={styles.instSrc} numberOfLines={2}&gt;{assetKind(a.kind)?.label} · {moneyCompact(earmarkedAmount(a, carId, homeId), 'M')}{simple ? '' : ` · ${info.source}${info.period ? ` · ${info.period}`</t>
         </is>
       </c>
       <c r="E504" s="2" t="inlineStr">
@@ -30657,7 +30639,7 @@
       </c>
       <c r="G517" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H517" s="2" t="inlineStr">
@@ -30700,7 +30682,7 @@
       </c>
       <c r="G518" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H518" s="2" t="inlineStr">
@@ -30743,7 +30725,7 @@
       </c>
       <c r="G519" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H519" s="2" t="inlineStr">
@@ -30786,7 +30768,7 @@
       </c>
       <c r="G520" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N</t>
+          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month</t>
         </is>
       </c>
       <c r="H520" s="2" t="inlineStr">
@@ -30872,7 +30854,7 @@
       </c>
       <c r="G522" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit, MK-MN-M-025 You'd have $X left — about N months of e</t>
+          <t>MK-MN-M-024 You could cover a $X hit, MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-026 your $X/month of essentials</t>
         </is>
       </c>
       <c r="H522" s="2" t="inlineStr">
@@ -30915,7 +30897,7 @@
       </c>
       <c r="G523" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit, MK-MN-M-025 You'd have $X left — about N months of e</t>
+          <t>MK-MN-M-024 You could cover a $X hit, MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-026 your $X/month of essentials</t>
         </is>
       </c>
       <c r="H523" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Net worth re-run part 3 fixes + DEC-4913 on Plan: Plan retirement money reads rent entries ($700,000 on every screen, agreement test), categoryEarnings shows stated bond rate when a bond row is worth $0, ledgerGroups keeps a missing balance as not known, card wording for windowStartKey / propertyUses
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
+++ b/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
@@ -16284,22 +16284,22 @@
       </c>
       <c r="D158" s="2" t="inlineStr">
         <is>
-          <t>estimate | social security | $#</t>
+          <t>afternoon | ava | your &lt;name&gt;: $#</t>
         </is>
       </c>
       <c r="E158" s="2" t="inlineStr">
         <is>
-          <t>retiree</t>
+          <t>worker</t>
         </is>
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>visible</t>
+          <t>spoken, visible</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
-          <t>$4,795 | this month</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="H158" s="2" t="inlineStr">
@@ -16327,22 +16327,22 @@
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>morning | ava | your &lt;name&gt;: $#</t>
+          <t>estimate | social security | $#</t>
         </is>
       </c>
       <c r="E159" s="2" t="inlineStr">
         <is>
-          <t>worker</t>
+          <t>retiree</t>
         </is>
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>spoken, visible</t>
+          <t>visible</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>$4,795 | this month</t>
         </is>
       </c>
       <c r="H159" s="2" t="inlineStr">
@@ -26210,7 +26210,7 @@
       </c>
       <c r="G414" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-CF-M-034 Your 401(k)s, MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H414" s="2" t="inlineStr">
@@ -26296,7 +26296,7 @@
       </c>
       <c r="G416" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-007 Left / Over · left to spend this month</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H416" s="2" t="inlineStr">
@@ -26339,7 +26339,7 @@
       </c>
       <c r="G417" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-007 Left / Over · left to spend this month</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H417" s="2" t="inlineStr">
@@ -26382,7 +26382,7 @@
       </c>
       <c r="G418" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-004 each row of the month — what it is and w, MK-CF-M-059 total interest</t>
+          <t>MK-CF-M-059 total interest, MK-CF-M-004 each row of the month — what it is and w</t>
         </is>
       </c>
       <c r="H418" s="2" t="inlineStr">
@@ -26392,7 +26392,7 @@
       </c>
       <c r="I418" s="2" t="n"/>
     </row>
-    <row r="419" ht="45" customHeight="1">
+    <row r="419" ht="60" customHeight="1">
       <c r="A419" s="2" t="inlineStr">
         <is>
           <t>money figure — more than one row could be it</t>
@@ -26425,7 +26425,7 @@
       </c>
       <c r="G419" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-CF-M-001 Expenses, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-CF-M-001 Expenses, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H419" s="2" t="inlineStr">
@@ -26468,7 +26468,7 @@
       </c>
       <c r="G420" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H420" s="2" t="inlineStr">
@@ -26620,7 +26620,7 @@
       </c>
       <c r="C424" s="2" t="inlineStr">
         <is>
-          <t>src/components/PlanInputs.tsx:122</t>
+          <t>src/components/PlanInputs.tsx:124</t>
         </is>
       </c>
       <c r="D424" s="2" t="inlineStr">
@@ -26663,7 +26663,7 @@
       </c>
       <c r="C425" s="2" t="inlineStr">
         <is>
-          <t>src/components/PlanInputs.tsx:144</t>
+          <t>src/components/PlanInputs.tsx:146</t>
         </is>
       </c>
       <c r="D425" s="2" t="inlineStr">
@@ -26706,7 +26706,7 @@
       </c>
       <c r="C426" s="2" t="inlineStr">
         <is>
-          <t>src/components/PlanInputs.tsx:151</t>
+          <t>src/components/PlanInputs.tsx:153</t>
         </is>
       </c>
       <c r="D426" s="2" t="inlineStr">
@@ -26749,7 +26749,7 @@
       </c>
       <c r="C427" s="2" t="inlineStr">
         <is>
-          <t>src/components/PlanInputs.tsx:163 (+1 spoken/visible twin)</t>
+          <t>src/components/PlanInputs.tsx:165 (+1 spoken/visible twin)</t>
         </is>
       </c>
       <c r="D427" s="2" t="inlineStr">
@@ -26792,7 +26792,7 @@
       </c>
       <c r="C428" s="2" t="inlineStr">
         <is>
-          <t>src/components/PlanInputs.tsx:181 (+2 spoken/visible twin)</t>
+          <t>src/components/PlanInputs.tsx:183 (+2 spoken/visible twin)</t>
         </is>
       </c>
       <c r="D428" s="2" t="inlineStr">
@@ -26835,7 +26835,7 @@
       </c>
       <c r="C429" s="2" t="inlineStr">
         <is>
-          <t>src/components/PlanInputs.tsx:251</t>
+          <t>src/components/PlanInputs.tsx:253</t>
         </is>
       </c>
       <c r="D429" s="2" t="inlineStr">
@@ -27050,7 +27050,7 @@
       </c>
       <c r="C434" s="2" t="inlineStr">
         <is>
-          <t>src/domain/planning/hub.ts:354</t>
+          <t>src/domain/planning/hub.ts:355</t>
         </is>
       </c>
       <c r="D434" s="2" t="inlineStr">
@@ -27543,7 +27543,7 @@
       </c>
       <c r="G445" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
+          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
         </is>
       </c>
       <c r="H445" s="2" t="inlineStr">
@@ -27629,7 +27629,7 @@
       </c>
       <c r="G447" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
+          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
         </is>
       </c>
       <c r="H447" s="2" t="inlineStr">
@@ -27672,7 +27672,7 @@
       </c>
       <c r="G448" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
+          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
         </is>
       </c>
       <c r="H448" s="2" t="inlineStr">
@@ -27887,7 +27887,7 @@
       </c>
       <c r="G453" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
+          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
         </is>
       </c>
       <c r="H453" s="2" t="inlineStr">
@@ -28188,7 +28188,7 @@
       </c>
       <c r="G460" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-007 Left / Over · left to spend this month</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H460" s="2" t="inlineStr">
@@ -28231,7 +28231,7 @@
       </c>
       <c r="G461" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
+          <t>MK-MN-M-012 Gross / year, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H461" s="2" t="inlineStr">
@@ -28274,7 +28274,7 @@
       </c>
       <c r="G462" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
+          <t>MK-MN-M-012 Gross / year, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H462" s="2" t="inlineStr">
@@ -28317,7 +28317,7 @@
       </c>
       <c r="G463" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
+          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H463" s="2" t="inlineStr">
@@ -28360,7 +28360,7 @@
       </c>
       <c r="G464" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-014 Employer 401(k) match</t>
+          <t>MK-MN-M-014 Employer 401(k) match, MK-MN-M-012 Gross / year, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H464" s="2" t="inlineStr">
@@ -28532,7 +28532,7 @@
       </c>
       <c r="G468" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-007 Left / Over · left to spend this month</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H468" s="2" t="inlineStr">
@@ -29349,7 +29349,7 @@
       </c>
       <c r="G487" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed</t>
         </is>
       </c>
       <c r="H487" s="2" t="inlineStr">
@@ -29392,7 +29392,7 @@
       </c>
       <c r="G488" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H488" s="2" t="inlineStr">
@@ -29435,7 +29435,7 @@
       </c>
       <c r="G489" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H489" s="2" t="inlineStr">
@@ -29478,7 +29478,7 @@
       </c>
       <c r="G490" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed</t>
         </is>
       </c>
       <c r="H490" s="2" t="inlineStr">
@@ -29521,7 +29521,7 @@
       </c>
       <c r="G491" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H491" s="2" t="inlineStr">
@@ -29759,7 +29759,7 @@
       </c>
       <c r="C497" s="2" t="inlineStr">
         <is>
-          <t>src/screens/RetirementCockpit.tsx:501</t>
+          <t>src/screens/RetirementCockpit.tsx:503</t>
         </is>
       </c>
       <c r="D497" s="2" t="inlineStr">
@@ -29802,7 +29802,7 @@
       </c>
       <c r="C498" s="2" t="inlineStr">
         <is>
-          <t>src/screens/RetirementCockpit.tsx:531</t>
+          <t>src/screens/RetirementCockpit.tsx:533</t>
         </is>
       </c>
       <c r="D498" s="2" t="inlineStr">
@@ -29845,7 +29845,7 @@
       </c>
       <c r="C499" s="2" t="inlineStr">
         <is>
-          <t>src/screens/RetirementCockpit.tsx:566</t>
+          <t>src/screens/RetirementCockpit.tsx:568</t>
         </is>
       </c>
       <c r="D499" s="2" t="inlineStr">
@@ -29888,7 +29888,7 @@
       </c>
       <c r="C500" s="2" t="inlineStr">
         <is>
-          <t>src/screens/RetirementCockpit.tsx:643</t>
+          <t>src/screens/RetirementCockpit.tsx:645</t>
         </is>
       </c>
       <c r="D500" s="2" t="inlineStr">
@@ -29931,7 +29931,7 @@
       </c>
       <c r="C501" s="2" t="inlineStr">
         <is>
-          <t>src/screens/RetirementCockpit.tsx:652</t>
+          <t>src/screens/RetirementCockpit.tsx:654</t>
         </is>
       </c>
       <c r="D501" s="2" t="inlineStr">
@@ -29974,7 +29974,7 @@
       </c>
       <c r="C502" s="2" t="inlineStr">
         <is>
-          <t>src/screens/RetirementCockpit.tsx:662</t>
+          <t>src/screens/RetirementCockpit.tsx:664</t>
         </is>
       </c>
       <c r="D502" s="2" t="inlineStr">
@@ -30017,7 +30017,7 @@
       </c>
       <c r="C503" s="2" t="inlineStr">
         <is>
-          <t>src/screens/RetirementCockpit.tsx:686</t>
+          <t>src/screens/RetirementCockpit.tsx:688</t>
         </is>
       </c>
       <c r="D503" s="2" t="inlineStr">
@@ -30060,7 +30060,7 @@
       </c>
       <c r="C504" s="2" t="inlineStr">
         <is>
-          <t>src/screens/RetirementCockpit.tsx:687</t>
+          <t>src/screens/RetirementCockpit.tsx:689</t>
         </is>
       </c>
       <c r="D504" s="2" t="inlineStr">
@@ -30103,7 +30103,7 @@
       </c>
       <c r="C505" s="2" t="inlineStr">
         <is>
-          <t>src/screens/RetirementCockpit.tsx:748</t>
+          <t>src/screens/RetirementCockpit.tsx:750</t>
         </is>
       </c>
       <c r="D505" s="2" t="inlineStr">
@@ -30146,7 +30146,7 @@
       </c>
       <c r="C506" s="2" t="inlineStr">
         <is>
-          <t>src/screens/RetirementCockpit.tsx:765</t>
+          <t>src/screens/RetirementCockpit.tsx:767</t>
         </is>
       </c>
       <c r="D506" s="2" t="inlineStr">
@@ -30189,7 +30189,7 @@
       </c>
       <c r="C507" s="2" t="inlineStr">
         <is>
-          <t>src/screens/RetirementCockpit.tsx:787</t>
+          <t>src/screens/RetirementCockpit.tsx:789</t>
         </is>
       </c>
       <c r="D507" s="2" t="inlineStr">
@@ -30232,7 +30232,7 @@
       </c>
       <c r="C508" s="2" t="inlineStr">
         <is>
-          <t>src/screens/RetirementCockpit.tsx:789</t>
+          <t>src/screens/RetirementCockpit.tsx:791</t>
         </is>
       </c>
       <c r="D508" s="2" t="inlineStr">
@@ -30275,7 +30275,7 @@
       </c>
       <c r="C509" s="2" t="inlineStr">
         <is>
-          <t>src/screens/RetirementCockpit.tsx:804</t>
+          <t>src/screens/RetirementCockpit.tsx:806</t>
         </is>
       </c>
       <c r="D509" s="2" t="inlineStr">
@@ -30318,7 +30318,7 @@
       </c>
       <c r="C510" s="2" t="inlineStr">
         <is>
-          <t>src/screens/RetirementCockpit.tsx:975</t>
+          <t>src/screens/RetirementCockpit.tsx:979</t>
         </is>
       </c>
       <c r="D510" s="2" t="inlineStr">
@@ -30361,7 +30361,7 @@
       </c>
       <c r="C511" s="2" t="inlineStr">
         <is>
-          <t>src/screens/RetirementCockpit.tsx:980</t>
+          <t>src/screens/RetirementCockpit.tsx:984</t>
         </is>
       </c>
       <c r="D511" s="2" t="inlineStr">
@@ -30639,7 +30639,7 @@
       </c>
       <c r="G517" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H517" s="2" t="inlineStr">
@@ -30682,7 +30682,7 @@
       </c>
       <c r="G518" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H518" s="2" t="inlineStr">
@@ -30725,7 +30725,7 @@
       </c>
       <c r="G519" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H519" s="2" t="inlineStr">
@@ -30768,7 +30768,7 @@
       </c>
       <c r="G520" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N</t>
         </is>
       </c>
       <c r="H520" s="2" t="inlineStr">
@@ -30854,7 +30854,7 @@
       </c>
       <c r="G522" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-024 You could cover a $X hit, MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-026 your $X/month of essentials</t>
+          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-024 You could cover a $X hit</t>
         </is>
       </c>
       <c r="H522" s="2" t="inlineStr">
@@ -30897,7 +30897,7 @@
       </c>
       <c r="G523" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-024 You could cover a $X hit, MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-026 your $X/month of essentials</t>
+          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-024 You could cover a $X hit</t>
         </is>
       </c>
       <c r="H523" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Net worth re-run part 4: one reading of a maturity date across all 13 readers (MK-NW-F-124 and others), cannotWorkBackSentence drops blank/duplicate names with has/have from the plural list; OpenAI part 4 cases recorded (133 of 145 agree)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
+++ b/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
@@ -1152,7 +1152,6 @@
 MK-NW-F-065 buildNetWorth
 MK-NW-F-066 sumWhere
 MK-NW-F-067 plural
-MK-NW-F-068 prettyDay
 MK-NW-F-069 priceAtYield
 MK-NW-F-070 accruedInterestCaveat
 MK-NW-F-072 rowOf
@@ -1238,7 +1237,7 @@
         </is>
       </c>
       <c r="I2" s="2" t="n">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
@@ -1302,6 +1301,7 @@
 MK-NW-F-046 historyCoverage
 MK-NW-F-047 uberGroupOf
 MK-NW-F-048 uberGroupRows
+MK-NW-F-068 prettyDay
 MK-NW-F-071 isCertificateOfDeposit
 MK-NW-F-090 windowStartKey
 MK-NW-F-091 pricedGainOf
@@ -1641,12 +1641,12 @@
 MK-NW-F-053 correctClassOf
 MK-NW-F-054 reclassifyAccounts
 MK-NW-F-067 plural
-MK-NW-F-068 prettyDay
 MK-NW-F-109 holdingClassOf
 MK-NW-F-120 classEvidenceOf
 MK-NW-F-121 holdingTagClass
 MK-NW-F-122 holdingTagFor
 MK-NW-F-123 holdingNameEvidence
+MK-NW-F-124 maturityParts
 MK-NW-O-002 theAccount
 MK-ST-F-010 nameEvidence
 MK-ST-F-013 personalFlowTotals
@@ -1758,6 +1758,7 @@
 MK-NW-F-060 approxYTM
 MK-NW-F-061 bondSummary
 MK-NW-F-064 bondRateSensitivity
+MK-NW-F-068 prettyDay
 MK-NW-F-069 priceAtYield
 MK-NW-F-070 accruedInterestCaveat
 MK-NW-F-071 isCertificateOfDeposit
@@ -1779,7 +1780,6 @@
 MK-NW-F-117 propertyUseMap
 MK-NW-F-118 itemizeMissingCount
 MK-NW-F-119 estimatedAccrued
-MK-NW-F-124 maturityParts
 MK-NW-F-125 isPastMaturity
 MK-NW-F-126 yearlyInterestNow
 MK-NW-F-127 gainOfRow
@@ -1875,7 +1875,7 @@
 MK-XS-I-008 transaction amount — read by MK-CF-F-118, MK-NW-O-002
 MK-XS-I-009 transaction date — read by MK-NW-O-002
 MK-XS-I-010 transaction words (the institution's own wording) — read by MK-NW-F-123, MK-ST-F-013
-MK-XS-I-013 bond maturity date — read by MK-NW-F-120, MK-ST-F-010
+MK-XS-I-013 bond maturity date — read by MK-NW-F-120, MK-NW-F-124, MK-ST-F-010
 MK-XS-I-024 logged expenses — read by MK-NW-O-002
 MK-XS-I-031 daily and monthly snapshots — read by MK-ST-F-030
 MK-XS-I-034 option positions — contracts, strike, expiry, put or call — read by MK-NW-F-027
@@ -2077,7 +2077,6 @@
 MK-NW-F-061 bondSummary
 MK-NW-F-064 bondRateSensitivity
 MK-NW-F-067 plural
-MK-NW-F-068 prettyDay
 MK-NW-F-069 priceAtYield
 MK-NW-F-070 accruedInterestCaveat
 MK-NW-F-072 rowOf
@@ -2281,7 +2280,6 @@
 MK-NW-F-061 bondSummary
 MK-NW-F-064 bondRateSensitivity
 MK-NW-F-067 plural
-MK-NW-F-068 prettyDay
 MK-NW-F-069 priceAtYield
 MK-NW-F-070 accruedInterestCaveat
 MK-NW-F-072 rowOf
@@ -2304,7 +2302,7 @@
         </is>
       </c>
       <c r="I5" s="2" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
@@ -2393,6 +2391,7 @@
 MK-NW-F-046 historyCoverage
 MK-NW-F-053 correctClassOf
 MK-NW-F-054 reclassifyAccounts
+MK-NW-F-068 prettyDay
 MK-NW-F-071 isCertificateOfDeposit
 MK-NW-F-077 ALL
 MK-NW-F-078 ONE
@@ -2498,6 +2497,8 @@
       <c r="L5" s="2" t="inlineStr">
         <is>
           <t>MK-XS-I-001 account balance — read by MK-NW-F-056, MK-NW-O-001, MK-ST-F-027
+MK-XS-I-001 account balance — read by MK-ST-F-027
+MK-XS-I-002 account type (taxable, pre-tax, Roth) — read by MK-NW-F-011, MK-NW-F-120
 MK-XS-I-002 account type (taxable, pre-tax, Roth) — read by MK-NW-F-011, MK-NW-F-120, MK-NW-O-001
 MK-XS-I-003 institution name — read by MK-NW-F-072, MK-NW-O-001
 MK-XS-I-004 holding quantity (shares) — read by MK-ST-F-027
@@ -2508,12 +2509,13 @@
 MK-XS-I-012 bond coupon rate — read by MK-NW-F-056, MK-NW-F-057, MK-NW-F-060, MK-NW-F-064, MK-NW-F-070, MK-NW-F-072, MK
 MK-XS-I-012 bond coupon rate — read by MK-NW-F-057, MK-NW-F-060, MK-NW-F-064, MK-NW-F-119
 MK-XS-I-013 bond maturity date — read by MK-NW-F-056, MK-NW-F-058, MK-NW-F-060, MK-NW-F-061, MK-NW-F-069, MK-NW-F-072, MK
-MK-XS-I-013 bond maturity date — read by MK-NW-F-058, MK-NW-F-060, MK-NW-F-069, MK-NW-F-119, MK-NW-F-124
+MK-XS-I-013 bond maturity date — read by MK-NW-F-058, MK-NW-F-060, MK-NW-F-069, MK-NW-F-119, MK-NW-F-120, MK-NW-F-124, MK
 MK-XS-I-028 assumed return — read by MK-NW-O-001
 MK-XS-I-048 the person’s own asset-class answer — read by MK-NW-F-011, MK-ST-F-027
 MK-XS-I-049 bond price — what the bond is worth today — read by MK-NW-F-056, MK-NW-F-057, MK-NW-F-059, MK-NW-F-060, MK-NW-F-061, MK-NW-F-064, MK
 MK-XS-I-049 bond price — what the bond is worth today — read by MK-NW-F-057, MK-NW-F-060, MK-NW-F-064, MK-NW-F-069, MK-NW-F-119, MK-NW-F-131
 MK-XS-I-055 the wrapper an account sits in — ISA, 401(k), IRA and the rest — read by MK-NW-F-011, MK-NW-F-056, MK-NW-F-120, MK-NW-O-001
+MK-XS-I-055 the wrapper an account sits in — ISA, 401(k), IRA and the rest — read by MK-NW-F-011, MK-NW-F-120
 MK-XS-I-065 accrued interest on a bond — interest earned since the last coupon — read by MK-NW-F-056, MK-NW-F-060, MK-NW-F-070, MK-NW-F-072
 MK-XS-I-065 accrued interest on a bond — interest earned since the last coupon — read by MK-NW-F-060
 [the code's record, this build — evidence for the ruling, not the row's statement: it cannot see inputs handed in as arguments, and it counts every branch below the producer]</t>
@@ -2696,7 +2698,6 @@
 MK-NW-F-061 bondSummary
 MK-NW-F-064 bondRateSensitivity
 MK-NW-F-067 plural
-MK-NW-F-068 prettyDay
 MK-NW-F-069 priceAtYield
 MK-NW-F-070 accruedInterestCaveat
 MK-NW-F-072 rowOf
@@ -2736,7 +2737,7 @@
         </is>
       </c>
       <c r="I6" s="2" t="n">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
@@ -2826,6 +2827,7 @@
 MK-NW-F-048 uberGroupRows
 MK-NW-F-065 buildNetWorth
 MK-NW-F-066 sumWhere
+MK-NW-F-068 prettyDay
 MK-NW-F-094 ledgerGroups
 MK-NW-F-106 mortgagesByProperty
 MK-NW-F-107 propertyUses
@@ -2960,7 +2962,7 @@
 MK-XS-I-011 bond face value — read by MK-NW-F-056, MK-NW-F-057, MK-NW-F-060, MK-NW-F-061, MK-NW-F-064, MK-NW-F-069, MK
 MK-XS-I-012 bond coupon rate — read by MK-NW-F-056, MK-NW-F-057, MK-NW-F-060, MK-NW-F-064, MK-NW-F-070, MK-NW-F-072, MK
 MK-XS-I-013 bond maturity date — read by MK-NW-F-056, MK-NW-F-058, MK-NW-F-060, MK-NW-F-061, MK-NW-F-069, MK-NW-F-072, MK
-MK-XS-I-013 bond maturity date — read by MK-NW-F-120, MK-ST-F-010
+MK-XS-I-013 bond maturity date — read by MK-NW-F-120, MK-NW-F-124, MK-ST-F-010
 MK-XS-I-014 debt balance — read by MK-CF-F-157, MK-CF-O-010
 MK-XS-I-015 debt interest rate — read by MK-CF-F-157, MK-CF-O-010
 MK-XS-I-016 debt minimum payment — read by MK-CF-F-023
@@ -3183,7 +3185,6 @@
 MK-NW-F-061 bondSummary
 MK-NW-F-064 bondRateSensitivity
 MK-NW-F-067 plural
-MK-NW-F-068 prettyDay
 MK-NW-F-069 priceAtYield
 MK-NW-F-070 accruedInterestCaveat
 MK-NW-F-071 isCertificateOfDeposit
@@ -3268,7 +3269,7 @@
         </is>
       </c>
       <c r="I7" s="2" t="n">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
@@ -3369,6 +3370,7 @@
 MK-NW-F-054 reclassifyAccounts
 MK-NW-F-065 buildNetWorth
 MK-NW-F-066 sumWhere
+MK-NW-F-068 prettyDay
 MK-NW-F-084 categoryEarnings
 MK-NW-F-092 investmentAccountIdsOf
 MK-NW-F-103 investmentRecordDates
@@ -3939,7 +3941,6 @@
 MK-NW-F-065 buildNetWorth
 MK-NW-F-066 sumWhere
 MK-NW-F-067 plural
-MK-NW-F-068 prettyDay
 MK-NW-F-069 priceAtYield
 MK-NW-F-070 accruedInterestCaveat
 MK-NW-F-072 rowOf
@@ -4053,7 +4054,7 @@
         </is>
       </c>
       <c r="I9" s="2" t="n">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
@@ -4109,6 +4110,7 @@
 MK-NW-F-046 historyCoverage
 MK-NW-F-047 uberGroupOf
 MK-NW-F-048 uberGroupRows
+MK-NW-F-068 prettyDay
 MK-NW-F-071 isCertificateOfDeposit
 MK-NW-F-090 windowStartKey
 MK-NW-F-091 pricedGainOf
@@ -4244,7 +4246,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MK-XS-I-001 account balance — read by MK-CF-F-111, MK-CF-F-133, MK-CF-F-134, MK-CF-F-136, MK-NW-F-016, MK-NW-F-027, MK
+          <t>MK-XS-I-001 account balance — read by MK-CF-F-111, MK-CF-F-133, MK-CF-F-134, MK-CF-F-136, MK-NW-F-016, MK-NW-F-027, MK
 MK-XS-I-001 account balance — read by MK-NW-F-031, MK-NW-F-032, MK-NW-F-133, MK-PL-F-026, MK-ST-F-027
 MK-XS-I-001 account balance — read by MK-NW-F-031, MK-NW-F-032, MK-NW-F-133, MK-ST-F-027
 MK-XS-I-002 account type (taxable, pre-tax, Roth) — read by MK-CF-F-134, MK-CF-F-136, MK-NW-F-011, MK-NW-F-027, MK-NW-F-040, MK-NW-F-054, MK
@@ -4268,7 +4270,7 @@
 MK-XS-I-011 bond face value — read by MK-NW-F-056, MK-NW-F-057, MK-NW-F-060, MK-NW-F-061, MK-NW-F-064, MK-NW-F-069, MK
 MK-XS-I-012 bond coupon rate — read by MK-NW-F-056, MK-NW-F-057, MK-NW-F-060, MK-NW-F-064, MK-NW-F-070, MK-NW-F-072, MK
 MK-XS-I-013 bond maturity date — read by MK-NW-F-056, MK-NW-F-058, MK-NW-F-060, MK-NW-F-061, MK-NW-F-069, MK-NW-F-072, MK
-MK-XS-I-013 bond maturity date — read by MK-NW-F-120, MK-ST-F-010
+MK-XS-I-013 bond maturity date — read by MK-NW-F-120, MK-NW-F-124, MK-ST-F-010
 MK-XS-I-014 debt balance — read by MK-CF-F-027, MK-CF-F-036, MK-CF-F-038, MK-CF-F-157, MK-CF-O-010, MK-NW-O-003
 MK-XS-I-015 debt interest rate — read by MK-CF-F-036, MK-CF-F-038, MK-CF-F-157, MK-CF-O-010
 MK-XS-I-016 debt minimum payment — read by MK-CF-F-023
@@ -4310,8 +4312,7 @@
 MK-XS-I-030 tax filing status and age — read by MK-CF-F-085, MK-CF-F-089, MK-CF-F-099, MK-CF-F-100, MK-CF-F-101, MK-CF-F-102, MK
 MK-XS-I-031 daily and monthly snapshots — read by MK-ST-F-028, MK-ST-F-030, MK-ST-F-035, MK-ST-F-036, MK-ST-F-072, MK-ST-F-073, MK
 MK-XS-I-031 daily and monthly snapshots — read by MK-ST-F-036
-MK-XS-I-032 expenses categories the person set up — read by MK-CF-F-004, MK-CF-F-008
-MK-XS-I-034 </t>
+MK-XS-I-032 expenses categories the person set up — read by MK-CF-F-004, MK-CF-F-008</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
@@ -4589,7 +4590,6 @@
 MK-NW-F-061 bondSummary
 MK-NW-F-064 bondRateSensitivity
 MK-NW-F-067 plural
-MK-NW-F-068 prettyDay
 MK-NW-F-069 priceAtYield
 MK-NW-F-070 accruedInterestCaveat
 MK-NW-F-072 rowOf
@@ -4642,7 +4642,7 @@
         </is>
       </c>
       <c r="I10" s="2" t="n">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
@@ -5089,7 +5089,6 @@
 MK-NW-F-053 correctClassOf
 MK-NW-F-054 reclassifyAccounts
 MK-NW-F-067 plural
-MK-NW-F-068 prettyDay
 MK-NW-F-110 primaryHomeIdOf
 MK-NW-F-114 rentAmount
 MK-NW-F-115 liveRent
@@ -5099,6 +5098,7 @@
 MK-NW-F-121 holdingTagClass
 MK-NW-F-122 holdingTagFor
 MK-NW-F-123 holdingNameEvidence
+MK-NW-F-124 maturityParts
 MK-NW-F-133 valueEntered
 MK-NW-F-134 carValueNotEnteredNotes
 MK-PF-F-001 totalShares
@@ -5315,13 +5315,13 @@
 MK-NW-F-032 earmarkedAmount
 MK-NW-F-033 retirementEarmarkedValue
 MK-NW-F-035 blendedVolatility
-MK-NW-F-068 prettyDay
 MK-NW-F-110 primaryHomeIdOf
 MK-NW-F-114 rentAmount
 MK-NW-F-115 liveRent
 MK-NW-F-116 rentedIdsOf
 MK-NW-F-117 propertyUseMap
 MK-NW-F-120 classEvidenceOf
+MK-NW-F-124 maturityParts
 MK-NW-F-133 valueEntered
 MK-NW-F-134 carValueNotEnteredNotes
 MK-PL-F-001 taxBucketSplit
@@ -5542,7 +5542,6 @@
 MK-NW-F-041 monthlyContributionsFromOnboarding
 MK-NW-F-053 correctClassOf
 MK-NW-F-054 reclassifyAccounts
-MK-NW-F-068 prettyDay
 MK-NW-F-110 primaryHomeIdOf
 MK-NW-F-114 rentAmount
 MK-NW-F-115 liveRent
@@ -5552,6 +5551,7 @@
 MK-NW-F-121 holdingTagClass
 MK-NW-F-122 holdingTagFor
 MK-NW-F-123 holdingNameEvidence
+MK-NW-F-124 maturityParts
 MK-NW-F-133 valueEntered
 MK-NW-F-134 carValueNotEnteredNotes
 MK-PF-F-001 totalShares
@@ -5834,7 +5834,6 @@
 MK-NW-F-061 bondSummary
 MK-NW-F-064 bondRateSensitivity
 MK-NW-F-067 plural
-MK-NW-F-068 prettyDay
 MK-NW-F-069 priceAtYield
 MK-NW-F-070 accruedInterestCaveat
 MK-NW-F-072 rowOf
@@ -5903,7 +5902,7 @@
         </is>
       </c>
       <c r="I14" s="2" t="n">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
@@ -6073,7 +6072,7 @@
 MK-XS-I-011 bond face value — read by MK-NW-F-056, MK-NW-F-057, MK-NW-F-060, MK-NW-F-061, MK-NW-F-064, MK-NW-F-069, MK
 MK-XS-I-012 bond coupon rate — read by MK-NW-F-056, MK-NW-F-057, MK-NW-F-060, MK-NW-F-064, MK-NW-F-070, MK-NW-F-072, MK
 MK-XS-I-013 bond maturity date — read by MK-NW-F-056, MK-NW-F-058, MK-NW-F-060, MK-NW-F-061, MK-NW-F-069, MK-NW-F-072, MK
-MK-XS-I-013 bond maturity date — read by MK-NW-F-120, MK-ST-F-010
+MK-XS-I-013 bond maturity date — read by MK-NW-F-120, MK-NW-F-124, MK-ST-F-010
 MK-XS-I-014 debt balance — read by MK-CF-F-034
 MK-XS-I-014 debt balance — read by MK-CF-F-157, MK-CF-O-010
 MK-XS-I-015 debt interest rate — read by MK-CF-F-034
@@ -6127,8 +6126,7 @@
 MK-XS-I-047 money to leave behind — read by MK-PL-F-067
 MK-XS-I-048 the person’s own asset-class answer — read by MK-NW-F-011, MK-ST-F-027
 MK-XS-I-049 bond price — what the bond is worth today — read by MK-NW-F-056, MK-NW-F-057, MK-NW-F-059, MK-NW-F-060, MK-NW-F-061, MK-NW-F-064, MK
-MK-XS-I-050 the share of an account earmarked for retirement — read by MK-NW-F-032
-MK-</t>
+MK-XS-I-050 the share of an account earmarked for retirement — read by MK</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
@@ -6375,8 +6373,8 @@
 MK-NW-F-022 investableAssets
 MK-NW-F-023 wrapperWord
 MK-NW-F-066 sumWhere
-MK-NW-F-068 prettyDay
 MK-NW-F-120 classEvidenceOf
+MK-NW-F-124 maturityParts
 MK-PL-F-034 lifeInsuranceNeed
 MK-ST-F-010 nameEvidence
 MK-ST-F-027 accountId
@@ -6609,7 +6607,6 @@
 MK-NW-F-061 bondSummary
 MK-NW-F-064 bondRateSensitivity
 MK-NW-F-067 plural
-MK-NW-F-068 prettyDay
 MK-NW-F-069 priceAtYield
 MK-NW-F-070 accruedInterestCaveat
 MK-NW-F-072 rowOf
@@ -6647,7 +6644,7 @@
         </is>
       </c>
       <c r="I17" s="2" t="n">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
@@ -6754,6 +6751,7 @@
 MK-NW-F-054 reclassifyAccounts
 MK-NW-F-065 buildNetWorth
 MK-NW-F-066 sumWhere
+MK-NW-F-068 prettyDay
 MK-NW-F-071 isCertificateOfDeposit
 MK-NW-F-090 windowStartKey
 MK-NW-F-091 pricedGainOf
@@ -7229,7 +7227,6 @@
 MK-NW-F-061 bondSummary
 MK-NW-F-064 bondRateSensitivity
 MK-NW-F-067 plural
-MK-NW-F-068 prettyDay
 MK-NW-F-069 priceAtYield
 MK-NW-F-070 accruedInterestCaveat
 MK-NW-F-072 rowOf
@@ -7265,7 +7262,7 @@
         </is>
       </c>
       <c r="I18" s="2" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
@@ -7820,7 +7817,6 @@
 MK-NW-F-061 bondSummary
 MK-NW-F-064 bondRateSensitivity
 MK-NW-F-067 plural
-MK-NW-F-068 prettyDay
 MK-NW-F-069 priceAtYield
 MK-NW-F-070 accruedInterestCaveat
 MK-NW-F-072 rowOf
@@ -7856,7 +7852,7 @@
         </is>
       </c>
       <c r="I19" s="2" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
@@ -8369,7 +8365,6 @@
 MK-NW-F-065 buildNetWorth
 MK-NW-F-066 sumWhere
 MK-NW-F-067 plural
-MK-NW-F-068 prettyDay
 MK-NW-F-069 priceAtYield
 MK-NW-F-070 accruedInterestCaveat
 MK-NW-F-071 isCertificateOfDeposit
@@ -8720,8 +8715,8 @@
 MK-NW-F-008 incomeBearingClassOf
 MK-NW-F-009 maturityClass
 MK-NW-F-011 assetClassOf
-MK-NW-F-068 prettyDay
 MK-NW-F-120 classEvidenceOf
+MK-NW-F-124 maturityParts
 MK-ST-F-010 nameEvidence
 MK-ST-F-027 accountId
 MK-ST-F-047 activeCurrency
@@ -8926,7 +8921,6 @@
 MK-NW-F-061 bondSummary
 MK-NW-F-064 bondRateSensitivity
 MK-NW-F-067 plural
-MK-NW-F-068 prettyDay
 MK-NW-F-069 priceAtYield
 MK-NW-F-070 accruedInterestCaveat
 MK-NW-F-072 rowOf
@@ -8962,7 +8956,7 @@
         </is>
       </c>
       <c r="I22" s="2" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
@@ -9280,7 +9274,6 @@
 MK-NW-F-065 buildNetWorth
 MK-NW-F-066 sumWhere
 MK-NW-F-067 plural
-MK-NW-F-068 prettyDay
 MK-NW-F-069 priceAtYield
 MK-NW-F-070 accruedInterestCaveat
 MK-NW-F-071 isCertificateOfDeposit
@@ -9715,7 +9708,6 @@
 MK-NW-F-065 buildNetWorth
 MK-NW-F-066 sumWhere
 MK-NW-F-067 plural
-MK-NW-F-068 prettyDay
 MK-NW-F-069 priceAtYield
 MK-NW-F-070 accruedInterestCaveat
 MK-NW-F-072 rowOf
@@ -26124,7 +26116,7 @@
       </c>
       <c r="G412" s="2" t="inlineStr">
         <is>
-          <t>MK-PF-M-014 Wealth generated, MK-PF-M-006 WHAT EACH CATEGORY EARNED — RETURN, MK-PF-M-017 Return</t>
+          <t>MK-PF-M-014 Wealth generated, MK-PF-M-017 Return, MK-PF-M-006 WHAT EACH CATEGORY EARNED — RETURN</t>
         </is>
       </c>
       <c r="H412" s="2" t="inlineStr">
@@ -26296,7 +26288,7 @@
       </c>
       <c r="G416" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H416" s="2" t="inlineStr">
@@ -26339,7 +26331,7 @@
       </c>
       <c r="G417" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H417" s="2" t="inlineStr">
@@ -26382,7 +26374,7 @@
       </c>
       <c r="G418" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-059 total interest, MK-CF-M-004 each row of the month — what it is and w</t>
+          <t>MK-CF-M-004 each row of the month — what it is and w, MK-CF-M-059 total interest</t>
         </is>
       </c>
       <c r="H418" s="2" t="inlineStr">
@@ -26511,7 +26503,7 @@
       </c>
       <c r="G421" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-020 THIS MONTH — free to use, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-CF-M-020 THIS MONTH — free to use</t>
         </is>
       </c>
       <c r="H421" s="2" t="inlineStr">
@@ -28102,7 +28094,7 @@
       </c>
       <c r="G458" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H458" s="2" t="inlineStr">
@@ -28145,7 +28137,7 @@
       </c>
       <c r="G459" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H459" s="2" t="inlineStr">
@@ -28188,7 +28180,7 @@
       </c>
       <c r="G460" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H460" s="2" t="inlineStr">
@@ -28231,7 +28223,7 @@
       </c>
       <c r="G461" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
+          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H461" s="2" t="inlineStr">
@@ -28274,7 +28266,7 @@
       </c>
       <c r="G462" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
+          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H462" s="2" t="inlineStr">
@@ -28317,7 +28309,7 @@
       </c>
       <c r="G463" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
+          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H463" s="2" t="inlineStr">
@@ -28360,7 +28352,7 @@
       </c>
       <c r="G464" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-014 Employer 401(k) match, MK-MN-M-012 Gross / year, MK-MN-M-011 TAKE-HOME / YEAR</t>
+          <t>MK-MN-M-014 Employer 401(k) match, MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H464" s="2" t="inlineStr">
@@ -28532,7 +28524,7 @@
       </c>
       <c r="G468" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H468" s="2" t="inlineStr">
@@ -29349,7 +29341,7 @@
       </c>
       <c r="G487" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H487" s="2" t="inlineStr">
@@ -29392,7 +29384,7 @@
       </c>
       <c r="G488" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H488" s="2" t="inlineStr">
@@ -29435,7 +29427,7 @@
       </c>
       <c r="G489" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H489" s="2" t="inlineStr">
@@ -29478,7 +29470,7 @@
       </c>
       <c r="G490" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H490" s="2" t="inlineStr">
@@ -29521,7 +29513,7 @@
       </c>
       <c r="G491" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed</t>
         </is>
       </c>
       <c r="H491" s="2" t="inlineStr">
@@ -30854,7 +30846,7 @@
       </c>
       <c r="G522" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-024 You could cover a $X hit</t>
+          <t>MK-MN-M-024 You could cover a $X hit, MK-MN-M-026 your $X/month of essentials, MK-MN-M-025 You'd have $X left — about N months of e</t>
         </is>
       </c>
       <c r="H522" s="2" t="inlineStr">
@@ -30897,7 +30889,7 @@
       </c>
       <c r="G523" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-024 You could cover a $X hit</t>
+          <t>MK-MN-M-024 You could cover a $X hit, MK-MN-M-026 your $X/month of essentials, MK-MN-M-025 You'd have $X left — about N months of e</t>
         </is>
       </c>
       <c r="H523" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Itemize form: a typed 0% bond/CD rate is 0%, an empty box is unknown (DEC-2748b); guard reads every screen for the num(coupon) > 0 pattern
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
+++ b/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
@@ -26288,7 +26288,7 @@
       </c>
       <c r="G416" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H416" s="2" t="inlineStr">
@@ -26331,7 +26331,7 @@
       </c>
       <c r="G417" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H417" s="2" t="inlineStr">
@@ -26374,7 +26374,7 @@
       </c>
       <c r="G418" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-004 each row of the month — what it is and w, MK-CF-M-059 total interest</t>
+          <t>MK-CF-M-059 total interest, MK-CF-M-004 each row of the month — what it is and w</t>
         </is>
       </c>
       <c r="H418" s="2" t="inlineStr">
@@ -26460,7 +26460,7 @@
       </c>
       <c r="G420" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
+          <t>MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H420" s="2" t="inlineStr">
@@ -27535,7 +27535,7 @@
       </c>
       <c r="G445" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
+          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
         </is>
       </c>
       <c r="H445" s="2" t="inlineStr">
@@ -27621,7 +27621,7 @@
       </c>
       <c r="G447" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
+          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
         </is>
       </c>
       <c r="H447" s="2" t="inlineStr">
@@ -27664,7 +27664,7 @@
       </c>
       <c r="G448" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
+          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
         </is>
       </c>
       <c r="H448" s="2" t="inlineStr">
@@ -27879,7 +27879,7 @@
       </c>
       <c r="G453" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
+          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
         </is>
       </c>
       <c r="H453" s="2" t="inlineStr">
@@ -28094,7 +28094,7 @@
       </c>
       <c r="G458" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H458" s="2" t="inlineStr">
@@ -28137,7 +28137,7 @@
       </c>
       <c r="G459" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H459" s="2" t="inlineStr">
@@ -28180,7 +28180,7 @@
       </c>
       <c r="G460" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H460" s="2" t="inlineStr">
@@ -28223,7 +28223,7 @@
       </c>
       <c r="G461" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
+          <t>MK-MN-M-013 Take-home / month, MK-MN-M-012 Gross / year, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H461" s="2" t="inlineStr">
@@ -28266,7 +28266,7 @@
       </c>
       <c r="G462" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
+          <t>MK-MN-M-013 Take-home / month, MK-MN-M-012 Gross / year, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H462" s="2" t="inlineStr">
@@ -28352,7 +28352,7 @@
       </c>
       <c r="G464" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-014 Employer 401(k) match, MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month</t>
+          <t>MK-MN-M-013 Take-home / month, MK-MN-M-014 Employer 401(k) match, MK-MN-M-012 Gross / year</t>
         </is>
       </c>
       <c r="H464" s="2" t="inlineStr">
@@ -28524,7 +28524,7 @@
       </c>
       <c r="G468" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
         </is>
       </c>
       <c r="H468" s="2" t="inlineStr">
@@ -29384,7 +29384,7 @@
       </c>
       <c r="G488" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H488" s="2" t="inlineStr">
@@ -29427,7 +29427,7 @@
       </c>
       <c r="G489" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H489" s="2" t="inlineStr">
@@ -29470,7 +29470,7 @@
       </c>
       <c r="G490" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H490" s="2" t="inlineStr">
@@ -29513,7 +29513,7 @@
       </c>
       <c r="G491" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed, MK-PL-M-005 + Draw from savings</t>
         </is>
       </c>
       <c r="H491" s="2" t="inlineStr">
@@ -30846,7 +30846,7 @@
       </c>
       <c r="G522" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-024 You could cover a $X hit, MK-MN-M-026 your $X/month of essentials, MK-MN-M-025 You'd have $X left — about N months of e</t>
+          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit, MK-MN-M-025 You'd have $X left — about N months of e</t>
         </is>
       </c>
       <c r="H522" s="2" t="inlineStr">
@@ -30889,7 +30889,7 @@
       </c>
       <c r="G523" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-024 You could cover a $X hit, MK-MN-M-026 your $X/month of essentials, MK-MN-M-025 You'd have $X left — about N months of e</t>
+          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit, MK-MN-M-025 You'd have $X left — about N months of e</t>
         </is>
       </c>
       <c r="H523" s="2" t="inlineStr">

</xml_diff>

<commit_message>
DEC-5068 on the Performance tab: summary, walk and window button show the worked-back figures and sentence the account card shows; Home uses the same holdings route
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
+++ b/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
@@ -26211,7 +26211,7 @@
       </c>
       <c r="G414" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-CF-M-034 Your 401(k)s, MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H414" s="2" t="inlineStr">
@@ -26297,7 +26297,7 @@
       </c>
       <c r="G416" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-007 Left / Over · left to spend this month</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H416" s="2" t="inlineStr">
@@ -26340,7 +26340,7 @@
       </c>
       <c r="G417" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-007 Left / Over · left to spend this month</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H417" s="2" t="inlineStr">
@@ -26383,7 +26383,7 @@
       </c>
       <c r="G418" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-059 total interest, MK-CF-M-004 each row of the month — what it is and w</t>
+          <t>MK-CF-M-004 each row of the month — what it is and w, MK-CF-M-059 total interest</t>
         </is>
       </c>
       <c r="H418" s="2" t="inlineStr">
@@ -26393,7 +26393,7 @@
       </c>
       <c r="I418" s="2" t="n"/>
     </row>
-    <row r="419" ht="45" customHeight="1">
+    <row r="419" ht="60" customHeight="1">
       <c r="A419" s="2" t="inlineStr">
         <is>
           <t>money figure — more than one row could be it</t>
@@ -26426,7 +26426,7 @@
       </c>
       <c r="G419" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-CF-M-001 Expenses, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-CF-M-001 Expenses, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H419" s="2" t="inlineStr">
@@ -27997,7 +27997,7 @@
       </c>
       <c r="C456" s="2" t="inlineStr">
         <is>
-          <t>src/screens/HomeScreen.tsx:306 (+1 spoken/visible twin)</t>
+          <t>src/screens/HomeScreen.tsx:309 (+1 spoken/visible twin)</t>
         </is>
       </c>
       <c r="D456" s="2" t="inlineStr">
@@ -28040,7 +28040,7 @@
       </c>
       <c r="C457" s="2" t="inlineStr">
         <is>
-          <t>src/screens/HomeScreen.tsx:421 (+1 spoken/visible twin)</t>
+          <t>src/screens/HomeScreen.tsx:426 (+1 spoken/visible twin)</t>
         </is>
       </c>
       <c r="D457" s="2" t="inlineStr">
@@ -28083,7 +28083,7 @@
       </c>
       <c r="C458" s="2" t="inlineStr">
         <is>
-          <t>src/screens/HomeScreen.tsx:508</t>
+          <t>src/screens/HomeScreen.tsx:513</t>
         </is>
       </c>
       <c r="D458" s="2" t="inlineStr">
@@ -28126,7 +28126,7 @@
       </c>
       <c r="C459" s="2" t="inlineStr">
         <is>
-          <t>src/screens/HomeScreen.tsx:521 (+1 spoken/visible twin)</t>
+          <t>src/screens/HomeScreen.tsx:526 (+1 spoken/visible twin)</t>
         </is>
       </c>
       <c r="D459" s="2" t="inlineStr">
@@ -28169,7 +28169,7 @@
       </c>
       <c r="C460" s="2" t="inlineStr">
         <is>
-          <t>src/screens/HomeScreen.tsx:522</t>
+          <t>src/screens/HomeScreen.tsx:527</t>
         </is>
       </c>
       <c r="D460" s="2" t="inlineStr">
@@ -28189,7 +28189,7 @@
       </c>
       <c r="G460" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-007 Left / Over · left to spend this month</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H460" s="2" t="inlineStr">
@@ -28232,7 +28232,7 @@
       </c>
       <c r="G461" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
+          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H461" s="2" t="inlineStr">
@@ -28275,7 +28275,7 @@
       </c>
       <c r="G462" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
+          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H462" s="2" t="inlineStr">
@@ -28318,7 +28318,7 @@
       </c>
       <c r="G463" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
+          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H463" s="2" t="inlineStr">
@@ -28361,7 +28361,7 @@
       </c>
       <c r="G464" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
+          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-014 Employer 401(k) match, MK-MN-M-012 Gross / year</t>
         </is>
       </c>
       <c r="H464" s="2" t="inlineStr">
@@ -28533,7 +28533,7 @@
       </c>
       <c r="G468" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-007 Left / Over · left to spend this month</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H468" s="2" t="inlineStr">
@@ -29350,7 +29350,7 @@
       </c>
       <c r="G487" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H487" s="2" t="inlineStr">
@@ -29393,7 +29393,7 @@
       </c>
       <c r="G488" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-005 + Draw from savings</t>
         </is>
       </c>
       <c r="H488" s="2" t="inlineStr">
@@ -29436,7 +29436,7 @@
       </c>
       <c r="G489" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-005 + Draw from savings</t>
         </is>
       </c>
       <c r="H489" s="2" t="inlineStr">
@@ -29479,7 +29479,7 @@
       </c>
       <c r="G490" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H490" s="2" t="inlineStr">
@@ -29522,7 +29522,7 @@
       </c>
       <c r="G491" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed, MK-PL-M-005 + Draw from savings</t>
         </is>
       </c>
       <c r="H491" s="2" t="inlineStr">
@@ -30855,7 +30855,7 @@
       </c>
       <c r="G522" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit</t>
+          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit, MK-MN-M-025 You'd have $X left — about N months of e</t>
         </is>
       </c>
       <c r="H522" s="2" t="inlineStr">
@@ -30898,7 +30898,7 @@
       </c>
       <c r="G523" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit</t>
+          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit, MK-MN-M-025 You'd have $X left — about N months of e</t>
         </is>
       </c>
       <c r="H523" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Net worth, no accounts past day one: one 'Add your accounts ›' door block instead of one per empty group (DEC-0227, v08 state C)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
+++ b/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
@@ -26393,7 +26393,7 @@
       </c>
       <c r="G412" s="2" t="inlineStr">
         <is>
-          <t>MK-PF-M-014 Wealth generated, MK-PF-M-002 Wealth generated, MK-PF-M-017 Return</t>
+          <t>MK-PF-M-014 Wealth generated, MK-PF-M-002 Wealth generated, MK-PF-M-006 WHAT EACH CATEGORY EARNED — RETURN</t>
         </is>
       </c>
       <c r="H412" s="2" t="inlineStr">
@@ -26479,7 +26479,7 @@
       </c>
       <c r="G414" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-034 Your 401(k)s, MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-XS-M-006 Income · In (received) · In (take-home)</t>
         </is>
       </c>
       <c r="H414" s="2" t="inlineStr">
@@ -26565,7 +26565,7 @@
       </c>
       <c r="G416" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-XS-M-007 Left / Over · left to spend this month</t>
         </is>
       </c>
       <c r="H416" s="2" t="inlineStr">
@@ -26608,7 +26608,7 @@
       </c>
       <c r="G417" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-XS-M-007 Left / Over · left to spend this month</t>
         </is>
       </c>
       <c r="H417" s="2" t="inlineStr">
@@ -26737,7 +26737,7 @@
       </c>
       <c r="G420" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
+          <t>MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-020 THIS MONTH — free to use</t>
         </is>
       </c>
       <c r="H420" s="2" t="inlineStr">
@@ -26780,7 +26780,7 @@
       </c>
       <c r="G421" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-020 THIS MONTH — free to use, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H421" s="2" t="inlineStr">
@@ -27812,7 +27812,7 @@
       </c>
       <c r="G445" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
+          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
         </is>
       </c>
       <c r="H445" s="2" t="inlineStr">
@@ -27898,7 +27898,7 @@
       </c>
       <c r="G447" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
+          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
         </is>
       </c>
       <c r="H447" s="2" t="inlineStr">
@@ -27941,7 +27941,7 @@
       </c>
       <c r="G448" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
+          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
         </is>
       </c>
       <c r="H448" s="2" t="inlineStr">
@@ -28156,7 +28156,7 @@
       </c>
       <c r="G453" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
+          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
         </is>
       </c>
       <c r="H453" s="2" t="inlineStr">
@@ -28371,7 +28371,7 @@
       </c>
       <c r="G458" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H458" s="2" t="inlineStr">
@@ -28414,7 +28414,7 @@
       </c>
       <c r="G459" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H459" s="2" t="inlineStr">
@@ -28457,7 +28457,7 @@
       </c>
       <c r="G460" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-XS-M-007 Left / Over · left to spend this month</t>
         </is>
       </c>
       <c r="H460" s="2" t="inlineStr">
@@ -28500,7 +28500,7 @@
       </c>
       <c r="G461" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month</t>
+          <t>MK-MN-M-013 Take-home / month, MK-MN-M-012 Gross / year, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H461" s="2" t="inlineStr">
@@ -28543,7 +28543,7 @@
       </c>
       <c r="G462" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month</t>
+          <t>MK-MN-M-013 Take-home / month, MK-MN-M-012 Gross / year, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H462" s="2" t="inlineStr">
@@ -28586,7 +28586,7 @@
       </c>
       <c r="G463" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
+          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H463" s="2" t="inlineStr">
@@ -28629,7 +28629,7 @@
       </c>
       <c r="G464" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-014 Employer 401(k) match, MK-MN-M-012 Gross / year</t>
+          <t>MK-MN-M-013 Take-home / month, MK-MN-M-012 Gross / year, MK-MN-M-014 Employer 401(k) match</t>
         </is>
       </c>
       <c r="H464" s="2" t="inlineStr">
@@ -28801,7 +28801,7 @@
       </c>
       <c r="G468" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-XS-M-007 Left / Over · left to spend this month</t>
         </is>
       </c>
       <c r="H468" s="2" t="inlineStr">
@@ -30908,7 +30908,7 @@
       </c>
       <c r="G517" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H517" s="2" t="inlineStr">
@@ -30951,7 +30951,7 @@
       </c>
       <c r="G518" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H518" s="2" t="inlineStr">
@@ -30994,7 +30994,7 @@
       </c>
       <c r="G519" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H519" s="2" t="inlineStr">
@@ -31037,7 +31037,7 @@
       </c>
       <c r="G520" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N</t>
+          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month</t>
         </is>
       </c>
       <c r="H520" s="2" t="inlineStr">
@@ -31123,7 +31123,7 @@
       </c>
       <c r="G522" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-024 You could cover a $X hit</t>
+          <t>MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit</t>
         </is>
       </c>
       <c r="H522" s="2" t="inlineStr">
@@ -31166,7 +31166,7 @@
       </c>
       <c r="G523" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-024 You could cover a $X hit</t>
+          <t>MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit</t>
         </is>
       </c>
       <c r="H523" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Account page: info dot on the Bonds & CDs yearly rate (DEC-5847), 'the income is' wording (DEC-5848), Itemize door only on one-total investment accounts (DEC-5849) and amber (DEC-5982), HISTORIC 12-MONTH RETURN card wording (DEC-6005)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
+++ b/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
@@ -26480,7 +26480,7 @@
       </c>
       <c r="G414" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-020 THIS MONTH — free to use, MK-XS-M-006 Income · In (received) · In (take-home)</t>
+          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-CF-M-020 THIS MONTH — free to use</t>
         </is>
       </c>
       <c r="H414" s="2" t="inlineStr">
@@ -26662,7 +26662,7 @@
       </c>
       <c r="I418" s="2" t="n"/>
     </row>
-    <row r="419" ht="45" customHeight="1">
+    <row r="419" ht="60" customHeight="1">
       <c r="A419" s="2" t="inlineStr">
         <is>
           <t>money figure — more than one row could be it</t>
@@ -26695,7 +26695,7 @@
       </c>
       <c r="G419" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-CF-M-001 Expenses, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-CF-M-001 Expenses, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H419" s="2" t="inlineStr">
@@ -26738,7 +26738,7 @@
       </c>
       <c r="G420" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H420" s="2" t="inlineStr">
@@ -26781,7 +26781,7 @@
       </c>
       <c r="G421" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-020 THIS MONTH — free to use, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-CF-M-020 THIS MONTH — free to use</t>
         </is>
       </c>
       <c r="H421" s="2" t="inlineStr">
@@ -28501,7 +28501,7 @@
       </c>
       <c r="G461" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month, MK-MN-M-012 Gross / year</t>
+          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-012 Gross / year</t>
         </is>
       </c>
       <c r="H461" s="2" t="inlineStr">
@@ -28544,7 +28544,7 @@
       </c>
       <c r="G462" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month, MK-MN-M-012 Gross / year</t>
+          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-012 Gross / year</t>
         </is>
       </c>
       <c r="H462" s="2" t="inlineStr">
@@ -28630,7 +28630,7 @@
       </c>
       <c r="G464" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-014 Employer 401(k) match, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month</t>
+          <t>MK-MN-M-013 Take-home / month, MK-MN-M-014 Employer 401(k) match, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H464" s="2" t="inlineStr">
@@ -29619,7 +29619,7 @@
       </c>
       <c r="G487" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H487" s="2" t="inlineStr">
@@ -29662,7 +29662,7 @@
       </c>
       <c r="G488" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-005 + Draw from savings</t>
         </is>
       </c>
       <c r="H488" s="2" t="inlineStr">
@@ -29748,7 +29748,7 @@
       </c>
       <c r="G490" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H490" s="2" t="inlineStr">
@@ -29791,7 +29791,7 @@
       </c>
       <c r="G491" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed, MK-PL-M-005 + Draw from savings</t>
         </is>
       </c>
       <c r="H491" s="2" t="inlineStr">

</xml_diff>

<commit_message>
DEC-6323: the line under a bond adds its maturity date; the Since window is never greyed (matches v17 day one; fixes tapping back to Since)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
+++ b/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
@@ -26488,7 +26488,7 @@
       </c>
       <c r="C413" s="2" t="inlineStr">
         <is>
-          <t>MoneyKeel/functions/_figure-spec.ts:146</t>
+          <t>MoneyKeel/functions/_figure-spec.ts:115</t>
         </is>
       </c>
       <c r="D413" s="2" t="inlineStr">
@@ -26508,7 +26508,7 @@
       </c>
       <c r="G413" s="2" t="inlineStr">
         <is>
-          <t>MK-PF-M-014 Wealth generated, MK-PF-M-002 Wealth generated, MK-PF-M-017 Return</t>
+          <t>MK-PF-M-014 Wealth generated, MK-PF-M-002 Wealth generated, MK-PF-M-006 WHAT EACH CATEGORY EARNED — RETURN</t>
         </is>
       </c>
       <c r="H413" s="2" t="inlineStr">
@@ -26531,7 +26531,7 @@
       </c>
       <c r="C414" s="2" t="inlineStr">
         <is>
-          <t>MoneyKeel/functions/_figure-spec.ts:148</t>
+          <t>MoneyKeel/functions/_figure-spec.ts:117</t>
         </is>
       </c>
       <c r="D414" s="2" t="inlineStr">
@@ -26594,7 +26594,7 @@
       </c>
       <c r="G415" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-020 THIS MONTH — free to use, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
+          <t>MK-CF-M-034 Your 401(k)s, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-CF-M-020 THIS MONTH — free to use</t>
         </is>
       </c>
       <c r="H415" s="2" t="inlineStr">
@@ -26680,7 +26680,7 @@
       </c>
       <c r="G417" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H417" s="2" t="inlineStr">
@@ -26723,7 +26723,7 @@
       </c>
       <c r="G418" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H418" s="2" t="inlineStr">
@@ -26776,7 +26776,7 @@
       </c>
       <c r="I419" s="2" t="n"/>
     </row>
-    <row r="420" ht="45" customHeight="1">
+    <row r="420" ht="60" customHeight="1">
       <c r="A420" s="2" t="inlineStr">
         <is>
           <t>money figure — more than one row could be it</t>
@@ -26809,7 +26809,7 @@
       </c>
       <c r="G420" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-CF-M-001 Expenses, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-XS-M-005 Spent so far · Spent $X of $Y left to sp, MK-CF-M-001 Expenses, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H420" s="2" t="inlineStr">
@@ -26852,7 +26852,7 @@
       </c>
       <c r="G421" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H421" s="2" t="inlineStr">
@@ -27927,7 +27927,7 @@
       </c>
       <c r="G446" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
+          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
         </is>
       </c>
       <c r="H446" s="2" t="inlineStr">
@@ -28013,7 +28013,7 @@
       </c>
       <c r="G448" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
+          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
         </is>
       </c>
       <c r="H448" s="2" t="inlineStr">
@@ -28056,7 +28056,7 @@
       </c>
       <c r="G449" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
+          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
         </is>
       </c>
       <c r="H449" s="2" t="inlineStr">
@@ -28271,7 +28271,7 @@
       </c>
       <c r="G454" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-010 your non-monthly budget, MK-MN-M-009 each goal — $X of $Y · $Z to go</t>
+          <t>MK-MN-M-009 each goal — $X of $Y · $Z to go, MK-MN-M-010 your non-monthly budget</t>
         </is>
       </c>
       <c r="H454" s="2" t="inlineStr">
@@ -28486,7 +28486,7 @@
       </c>
       <c r="G459" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H459" s="2" t="inlineStr">
@@ -28529,7 +28529,7 @@
       </c>
       <c r="G460" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H460" s="2" t="inlineStr">
@@ -28572,7 +28572,7 @@
       </c>
       <c r="G461" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H461" s="2" t="inlineStr">
@@ -28615,7 +28615,7 @@
       </c>
       <c r="G462" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-012 Gross / year</t>
+          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H462" s="2" t="inlineStr">
@@ -28658,7 +28658,7 @@
       </c>
       <c r="G463" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-012 Gross / year</t>
+          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR</t>
         </is>
       </c>
       <c r="H463" s="2" t="inlineStr">
@@ -28744,7 +28744,7 @@
       </c>
       <c r="G465" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-013 Take-home / month, MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-014 Employer 401(k) match</t>
+          <t>MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month, MK-MN-M-014 Employer 401(k) match</t>
         </is>
       </c>
       <c r="H465" s="2" t="inlineStr">
@@ -28916,7 +28916,7 @@
       </c>
       <c r="G469" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H469" s="2" t="inlineStr">
@@ -29733,7 +29733,7 @@
       </c>
       <c r="G488" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed</t>
         </is>
       </c>
       <c r="H488" s="2" t="inlineStr">
@@ -29776,7 +29776,7 @@
       </c>
       <c r="G489" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed</t>
         </is>
       </c>
       <c r="H489" s="2" t="inlineStr">
@@ -29819,7 +29819,7 @@
       </c>
       <c r="G490" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-005 + Draw from savings</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-005 + Draw from savings</t>
         </is>
       </c>
       <c r="H490" s="2" t="inlineStr">
@@ -29862,7 +29862,7 @@
       </c>
       <c r="G491" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed</t>
         </is>
       </c>
       <c r="H491" s="2" t="inlineStr">
@@ -29905,7 +29905,7 @@
       </c>
       <c r="G492" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-005 + Draw from savings</t>
+          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed</t>
         </is>
       </c>
       <c r="H492" s="2" t="inlineStr">
@@ -31238,7 +31238,7 @@
       </c>
       <c r="G523" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-024 You could cover a $X hit, MK-MN-M-026 your $X/month of essentials</t>
+          <t>MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit</t>
         </is>
       </c>
       <c r="H523" s="2" t="inlineStr">
@@ -31281,7 +31281,7 @@
       </c>
       <c r="G524" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-024 You could cover a $X hit, MK-MN-M-026 your $X/month of essentials</t>
+          <t>MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit</t>
         </is>
       </c>
       <c r="H524" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Records: six Performance decisions settled for the compliance check (his "Fix the records only", 2026-10-23)
- DEC-0470, DEC-7314, DEC-7315, DEC-7318 now govern the v02 sheet drawings (Update value, holding editor, trade sheet, edit record); the v01s were archived 2026-10-22
- DEC-7306, DEC-7316 mark their quoted old wording with "replaced by", so the check reads it as gone rather than required; the check itself is unchanged

validate-module-complies performance: 0 breached, 0 broken record, 0 not found. build-all: every guard passed; 503 of 503 suites, 7,647 tests.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
+++ b/MoneyKeel/documents/standards/moneykeel_calc_spec_orchestrator-map_v01.xlsx
@@ -29692,7 +29692,7 @@
       </c>
       <c r="G455" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H455" s="2" t="inlineStr">
@@ -29735,7 +29735,7 @@
       </c>
       <c r="G456" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H456" s="2" t="inlineStr">
@@ -29864,7 +29864,7 @@
       </c>
       <c r="G459" s="2" t="inlineStr">
         <is>
-          <t>MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-CF-M-023 YOUR FUTURE PAYCHECK — Social Security ·, MK-CF-M-011 YOUR SOURCES — Social Security · pension, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H459" s="2" t="inlineStr">
@@ -29907,7 +29907,7 @@
       </c>
       <c r="G460" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon, MK-CF-M-020 THIS MONTH — free to use</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-CF-M-020 THIS MONTH — free to use, MK-CF-M-022 YOUR FUTURE PAYCHECK — At &lt;age&gt;: ~$X/mon</t>
         </is>
       </c>
       <c r="H460" s="2" t="inlineStr">
@@ -31412,7 +31412,7 @@
       </c>
       <c r="G495" s="2" t="inlineStr">
         <is>
-          <t>MK-HM-M-001 prices updated &lt;when&gt;, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-HM-M-001 prices updated &lt;when&gt;</t>
         </is>
       </c>
       <c r="H495" s="2" t="inlineStr">
@@ -31455,7 +31455,7 @@
       </c>
       <c r="G496" s="2" t="inlineStr">
         <is>
-          <t>MK-HM-M-001 prices updated &lt;when&gt;, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-HM-M-001 prices updated &lt;when&gt;</t>
         </is>
       </c>
       <c r="H496" s="2" t="inlineStr">
@@ -31627,7 +31627,7 @@
       </c>
       <c r="G500" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H500" s="2" t="inlineStr">
@@ -31670,7 +31670,7 @@
       </c>
       <c r="G501" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month, MK-MN-M-012 Gross / year</t>
+          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H501" s="2" t="inlineStr">
@@ -31713,7 +31713,7 @@
       </c>
       <c r="G502" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-013 Take-home / month, MK-MN-M-012 Gross / year</t>
+          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-012 Gross / year, MK-MN-M-013 Take-home / month</t>
         </is>
       </c>
       <c r="H502" s="2" t="inlineStr">
@@ -31799,7 +31799,7 @@
       </c>
       <c r="G504" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-014 Employer 401(k) match, MK-MN-M-013 Take-home / month</t>
+          <t>MK-MN-M-011 TAKE-HOME / YEAR, MK-MN-M-014 Employer 401(k) match, MK-MN-M-012 Gross / year</t>
         </is>
       </c>
       <c r="H504" s="2" t="inlineStr">
@@ -31928,7 +31928,7 @@
       </c>
       <c r="G507" s="2" t="inlineStr">
         <is>
-          <t>MK-HM-M-001 prices updated &lt;when&gt;, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-HM-M-001 prices updated &lt;when&gt;</t>
         </is>
       </c>
       <c r="H507" s="2" t="inlineStr">
@@ -31971,7 +31971,7 @@
       </c>
       <c r="G508" s="2" t="inlineStr">
         <is>
-          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-XS-M-007 Left / Over · left to spend this month, MK-HM-M-004 &lt;n&gt;% spent · day n of m</t>
+          <t>MK-XS-M-006 Income · In (received) · In (take-home), MK-HM-M-004 &lt;n&gt;% spent · day n of m, MK-XS-M-005 Spent so far · Spent $X of $Y left to sp</t>
         </is>
       </c>
       <c r="H508" s="2" t="inlineStr">
@@ -32788,7 +32788,7 @@
       </c>
       <c r="G527" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H527" s="2" t="inlineStr">
@@ -32831,7 +32831,7 @@
       </c>
       <c r="G528" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-005 + Draw from savings</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H528" s="2" t="inlineStr">
@@ -32874,7 +32874,7 @@
       </c>
       <c r="G529" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-006 Your paycheck $X/mo</t>
         </is>
       </c>
       <c r="H529" s="2" t="inlineStr">
@@ -32917,7 +32917,7 @@
       </c>
       <c r="G530" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
+          <t>MK-PL-M-005 + Draw from savings, MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H530" s="2" t="inlineStr">
@@ -32960,7 +32960,7 @@
       </c>
       <c r="G531" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante, MK-PL-M-005 + Draw from savings</t>
+          <t>MK-PL-M-006 Your paycheck $X/mo, MK-PL-M-004 = Guaranteed, MK-PL-M-003 YOUR RETIREMENT PAYCHECK — each guarante</t>
         </is>
       </c>
       <c r="H531" s="2" t="inlineStr">
@@ -34078,7 +34078,7 @@
       </c>
       <c r="G557" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H557" s="2" t="inlineStr">
@@ -34121,7 +34121,7 @@
       </c>
       <c r="G558" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H558" s="2" t="inlineStr">
@@ -34164,7 +34164,7 @@
       </c>
       <c r="G559" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N, MK-PL-M-021 Showing example numbers (a $X/mo stateme</t>
         </is>
       </c>
       <c r="H559" s="2" t="inlineStr">
@@ -34207,7 +34207,7 @@
       </c>
       <c r="G560" s="2" t="inlineStr">
         <is>
-          <t>MK-PL-M-020 about $X in total by age N, MK-PL-M-019 Claiming at N pays $X a month</t>
+          <t>MK-PL-M-019 Claiming at N pays $X a month, MK-PL-M-020 about $X in total by age N</t>
         </is>
       </c>
       <c r="H560" s="2" t="inlineStr">
@@ -34293,7 +34293,7 @@
       </c>
       <c r="G562" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit</t>
+          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit, MK-MN-M-025 You'd have $X left — about N months of e</t>
         </is>
       </c>
       <c r="H562" s="2" t="inlineStr">
@@ -34336,7 +34336,7 @@
       </c>
       <c r="G563" s="2" t="inlineStr">
         <is>
-          <t>MK-MN-M-025 You'd have $X left — about N months of e, MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit</t>
+          <t>MK-MN-M-026 your $X/month of essentials, MK-MN-M-024 You could cover a $X hit, MK-MN-M-025 You'd have $X left — about N months of e</t>
         </is>
       </c>
       <c r="H563" s="2" t="inlineStr">

</xml_diff>